<commit_message>
docs: design spec, API contract and test matrix for the redesign
- DDD-spec rewritten for the Lantern Night system (role rules, contrast table,
  page contract, checkout and routing behaviour)
- api-contract: ?lang, locale, saved journeys, MBTI, recharge tiers and bonus
- SDD/TDD: new requirements and test IDs; regenerated docs/generated + app.xlsx
- README: both themes and bilingual UI, 63 Playwright tests
</commit_message>
<xml_diff>
--- a/app.xlsx
+++ b/app.xlsx
@@ -154,7 +154,7 @@
         </is>
       </c>
       <c r="B4">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -217,7 +217,7 @@
         </is>
       </c>
       <c r="E6">
-        <v>23</v>
+        <v>28</v>
       </c>
     </row>
     <row r="7">
@@ -242,7 +242,7 @@
         </is>
       </c>
       <c r="E7">
-        <v>27</v>
+        <v>35</v>
       </c>
     </row>
     <row r="8">
@@ -780,7 +780,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>order_handler_test</t>
+          <t>me_handler_test</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -790,7 +790,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>internal/handler/order_handler_test.go</t>
+          <t>internal/handler/me_handler_test.go</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -817,7 +817,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>cors_test</t>
+          <t>order_handler_test</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -827,7 +827,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>internal/middleware/cors_test.go</t>
+          <t>internal/handler/order_handler_test.go</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -854,7 +854,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>jwt_test</t>
+          <t>payment_handler_test</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -864,7 +864,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>internal/middleware/jwt_test.go</t>
+          <t>internal/handler/payment_handler_test.go</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -891,7 +891,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>request_id_test</t>
+          <t>cors_test</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -901,7 +901,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>internal/middleware/request_id_test.go</t>
+          <t>internal/middleware/cors_test.go</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -928,7 +928,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>journey_repo_sqlite_test</t>
+          <t>jwt_test</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -938,7 +938,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>internal/repository/journey_repo_sqlite_test.go</t>
+          <t>internal/middleware/jwt_test.go</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -965,7 +965,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>order_repo_test</t>
+          <t>request_id_test</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -975,7 +975,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>internal/repository/order_repo_test.go</t>
+          <t>internal/middleware/request_id_test.go</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1002,7 +1002,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>user_repo_test</t>
+          <t>journey_repo_sqlite_test</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1012,7 +1012,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>internal/repository/user_repo_test.go</t>
+          <t>internal/repository/journey_repo_sqlite_test.go</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1039,7 +1039,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>journey_service_test</t>
+          <t>order_repo_test</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1049,7 +1049,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>internal/service/journey_service_test.go</t>
+          <t>internal/repository/order_repo_test.go</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1071,12 +1071,12 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Playwright E2E</t>
+          <t>Go unit/integration / Go 单元集成</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>auth.spec</t>
+          <t>user_repo_test</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1086,7 +1086,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>e2e/tests/auth.spec.js</t>
+          <t>internal/repository/user_repo_test.go</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1108,12 +1108,12 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Playwright E2E</t>
+          <t>Go unit/integration / Go 单元集成</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>detail.spec</t>
+          <t>journey_service_test</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1123,7 +1123,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>e2e/tests/detail.spec.js</t>
+          <t>internal/service/journey_service_test.go</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1145,12 +1145,12 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Playwright E2E</t>
+          <t>Go unit/integration / Go 单元集成</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>explore.spec</t>
+          <t>locale_test</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1160,7 +1160,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>e2e/tests/explore.spec.js</t>
+          <t>internal/service/locale_test.go</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1182,12 +1182,12 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Playwright E2E</t>
+          <t>Go unit/integration / Go 单元集成</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>home.spec</t>
+          <t>index_test</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1197,7 +1197,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>e2e/tests/home.spec.js</t>
+          <t>internal/webapp/index_test.go</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1224,7 +1224,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>orders.spec</t>
+          <t>a11y.spec</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1234,7 +1234,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>e2e/tests/orders.spec.js</t>
+          <t>e2e/tests/a11y.spec.js</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1256,12 +1256,12 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Playwright support / E2E 支撑文件</t>
+          <t>Playwright E2E</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>helpers</t>
+          <t>auth.spec</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1271,7 +1271,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>e2e/tests/helpers.js</t>
+          <t>e2e/tests/auth.spec.js</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1293,12 +1293,12 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Go stress</t>
+          <t>Playwright E2E</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>stress_test</t>
+          <t>detail.spec</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>tests/stress/stress_test.go</t>
+          <t>e2e/tests/detail.spec.js</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1330,12 +1330,12 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>k6 load / k6 负载</t>
+          <t>Playwright E2E</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>admin-analytics-export.k6</t>
+          <t>explore.spec</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -1345,7 +1345,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>tests/load/admin-analytics-export.k6.js</t>
+          <t>e2e/tests/explore.spec.js</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1367,12 +1367,12 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>k6 load / k6 负载</t>
+          <t>Playwright E2E</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>auth-register-login.k6</t>
+          <t>home.spec</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1382,7 +1382,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>tests/load/auth-register-login.k6.js</t>
+          <t>e2e/tests/home.spec.js</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1404,12 +1404,12 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>k6 load / k6 负载</t>
+          <t>Playwright E2E</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>image-static-cache.k6</t>
+          <t>i18n.spec</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1419,7 +1419,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>tests/load/image-static-cache.k6.js</t>
+          <t>e2e/tests/i18n.spec.js</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -1441,12 +1441,12 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>k6 load / k6 负载</t>
+          <t>Playwright E2E</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>order-payment-audit.k6</t>
+          <t>mobile.spec</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1456,7 +1456,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>tests/load/order-payment-audit.k6.js</t>
+          <t>e2e/tests/mobile.spec.js</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -1478,12 +1478,12 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>k6 load / k6 负载</t>
+          <t>Playwright E2E</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>pet-chat-analytics.k6</t>
+          <t>orders.spec</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -1493,7 +1493,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>tests/load/pet-chat-analytics.k6.js</t>
+          <t>e2e/tests/orders.spec.js</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -1515,12 +1515,12 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>k6 load / k6 负载</t>
+          <t>Playwright E2E</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>public-content-flow.k6</t>
+          <t>persona.spec</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1530,7 +1530,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>tests/load/public-content-flow.k6.js</t>
+          <t>e2e/tests/persona.spec.js</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -1542,296 +1542,296 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Route</t>
+          <t>Test</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>ROUTE-001</t>
+          <t>TEST-028</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Admin</t>
+          <t>Playwright support / E2E 支撑文件</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>GET /api/admin/export</t>
+          <t>helpers</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Route is registered</t>
+          <t>File exists and is part of repo</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>internal/handler/admin_handler.go</t>
+          <t>e2e/tests/helpers.js</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Specified</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Route</t>
+          <t>Test</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>ROUTE-002</t>
+          <t>TEST-029</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Admin</t>
+          <t>Go stress</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>GET /api/admin/stats</t>
+          <t>stress_test</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Route is registered</t>
+          <t>File exists and is part of repo</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>internal/handler/admin_handler.go</t>
+          <t>tests/stress/stress_test.go</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Specified</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Route</t>
+          <t>Test</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>ROUTE-003</t>
+          <t>TEST-030</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Admin</t>
+          <t>k6 load / k6 负载</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>GET /api/admin/users</t>
+          <t>admin-analytics-export.k6</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Route is registered</t>
+          <t>File exists and is part of repo</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>internal/handler/admin_handler.go</t>
+          <t>tests/load/admin-analytics-export.k6.js</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Specified</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Route</t>
+          <t>Test</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>ROUTE-004</t>
+          <t>TEST-031</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>k6 load / k6 负载</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>POST /api/ai/chat</t>
+          <t>auth-register-login.k6</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Route is registered</t>
+          <t>File exists and is part of repo</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>tests/load/auth-register-login.k6.js</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Specified</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Route</t>
+          <t>Test</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>ROUTE-005</t>
+          <t>TEST-032</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>k6 load / k6 负载</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>POST /api/analytics/events</t>
+          <t>image-static-cache.k6</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Route is registered</t>
+          <t>File exists and is part of repo</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>tests/load/image-static-cache.k6.js</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Specified</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Route</t>
+          <t>Test</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>ROUTE-006</t>
+          <t>TEST-033</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>k6 load / k6 负载</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>POST /api/audit/client-error</t>
+          <t>order-payment-audit.k6</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Route is registered</t>
+          <t>File exists and is part of repo</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>tests/load/order-payment-audit.k6.js</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Specified</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Route</t>
+          <t>Test</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>ROUTE-007</t>
+          <t>TEST-034</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>k6 load / k6 负载</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>POST /api/auth/avatar</t>
+          <t>pet-chat-analytics.k6</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Route is registered</t>
+          <t>File exists and is part of repo</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>tests/load/pet-chat-analytics.k6.js</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Specified</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Route</t>
+          <t>Test</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>ROUTE-008</t>
+          <t>TEST-035</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>k6 load / k6 负载</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>POST /api/auth/login</t>
+          <t>public-content-flow.k6</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Route is registered</t>
+          <t>File exists and is part of repo</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>tests/load/public-content-flow.k6.js</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Specified</t>
         </is>
       </c>
     </row>
@@ -1843,17 +1843,17 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>ROUTE-009</t>
+          <t>ROUTE-001</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Admin</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>GET /api/auth/me</t>
+          <t>GET /api/admin/export</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -1863,7 +1863,7 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>internal/handler/admin_handler.go</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -1880,17 +1880,17 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>ROUTE-010</t>
+          <t>ROUTE-002</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>Admin</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>POST /api/auth/register</t>
+          <t>GET /api/admin/stats</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -1900,7 +1900,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>internal/handler/admin_handler.go</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -1917,17 +1917,17 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>ROUTE-011</t>
+          <t>ROUTE-003</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>Admin</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>GET /api/captcha</t>
+          <t>GET /api/admin/users</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -1937,7 +1937,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>internal/handler/admin_handler.go</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -1954,7 +1954,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>ROUTE-012</t>
+          <t>ROUTE-004</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -1964,7 +1964,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>GET /api/health</t>
+          <t>POST /api/ai/chat</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -1991,7 +1991,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>ROUTE-013</t>
+          <t>ROUTE-005</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2001,7 +2001,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>GET /api/journeys</t>
+          <t>POST /api/analytics/events</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -2028,7 +2028,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>ROUTE-014</t>
+          <t>ROUTE-006</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2038,7 +2038,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>GET /api/journeys/:slug</t>
+          <t>POST /api/audit/client-error</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -2065,17 +2065,17 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>ROUTE-015</t>
+          <t>ROUTE-007</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>JWT</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>GET /api/journeys/:slug/book</t>
+          <t>POST /api/auth/avatar</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -2102,7 +2102,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>ROUTE-016</t>
+          <t>ROUTE-008</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2112,7 +2112,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>GET /api/mbti</t>
+          <t>POST /api/auth/login</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -2139,7 +2139,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>ROUTE-017</t>
+          <t>ROUTE-009</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2149,7 +2149,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>GET /api/orders</t>
+          <t>PUT /api/auth/mbti</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -2159,7 +2159,7 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>internal/handler/order_handler.go</t>
+          <t>internal/handler/me_handler.go</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -2176,7 +2176,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>ROUTE-018</t>
+          <t>ROUTE-010</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2186,7 +2186,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>POST /api/orders</t>
+          <t>GET /api/auth/me</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -2196,7 +2196,7 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>internal/handler/order_handler.go</t>
+          <t>cmd/server/main.go</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -2213,17 +2213,17 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>ROUTE-019</t>
+          <t>ROUTE-011</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>GET /api/orders/:id</t>
+          <t>POST /api/auth/register</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -2233,7 +2233,7 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>internal/handler/order_handler.go</t>
+          <t>cmd/server/main.go</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -2250,7 +2250,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>ROUTE-020</t>
+          <t>ROUTE-012</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2260,7 +2260,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>POST /api/orders/:id/pay</t>
+          <t>GET /api/auth/saved</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -2270,7 +2270,7 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>internal/handler/order_handler.go</t>
+          <t>internal/handler/me_handler.go</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -2287,7 +2287,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>ROUTE-021</t>
+          <t>ROUTE-013</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2297,7 +2297,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>POST /api/payments/recharge</t>
+          <t>DELETE /api/auth/saved/:slug</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -2307,7 +2307,7 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>internal/handler/payment_handler.go</t>
+          <t>internal/handler/me_handler.go</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -2324,7 +2324,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>ROUTE-022</t>
+          <t>ROUTE-014</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2334,7 +2334,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>GET /api/payments/transactions</t>
+          <t>PUT /api/auth/saved/:slug</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -2344,7 +2344,7 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>internal/handler/payment_handler.go</t>
+          <t>internal/handler/me_handler.go</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -2361,30 +2361,511 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
+          <t>ROUTE-015</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>GET /api/captcha</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Route is registered</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>cmd/server/main.go</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Route</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>ROUTE-016</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>GET /api/health</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Route is registered</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>cmd/server/main.go</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Route</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>ROUTE-017</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>GET /api/journeys</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Route is registered</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>cmd/server/main.go</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Route</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>ROUTE-018</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>GET /api/journeys/:slug</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Route is registered</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>cmd/server/main.go</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Route</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>ROUTE-019</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>GET /api/journeys/:slug/book</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Route is registered</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>cmd/server/main.go</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Route</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>ROUTE-020</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>GET /api/mbti</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Route is registered</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>cmd/server/main.go</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Route</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>ROUTE-021</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>JWT</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>GET /api/orders</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Route is registered</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>internal/handler/order_handler.go</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Route</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>ROUTE-022</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>JWT</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>POST /api/orders</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Route is registered</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>internal/handler/order_handler.go</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Route</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
           <t>ROUTE-023</t>
         </is>
       </c>
-      <c r="C56" t="inlineStr">
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>JWT</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>GET /api/orders/:id</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Route is registered</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>internal/handler/order_handler.go</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Route</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>ROUTE-024</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>JWT</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>POST /api/orders/:id/pay</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Route is registered</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>internal/handler/order_handler.go</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Route</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>ROUTE-025</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>JWT</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>POST /api/payments/recharge</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Route is registered</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>internal/handler/payment_handler.go</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Route</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>ROUTE-026</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
         <is>
           <t>Public</t>
         </is>
       </c>
-      <c r="D56" t="inlineStr">
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>GET /api/payments/tiers</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Route is registered</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>internal/handler/payment_handler.go</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Route</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>ROUTE-027</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>JWT</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>GET /api/payments/transactions</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Route is registered</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>internal/handler/payment_handler.go</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Route</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>ROUTE-028</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
         <is>
           <t>GET /api/tags</t>
         </is>
       </c>
-      <c r="E56" t="inlineStr">
+      <c r="E69" t="inlineStr">
         <is>
           <t>Route is registered</t>
         </is>
       </c>
-      <c r="F56" t="inlineStr">
+      <c r="F69" t="inlineStr">
         <is>
           <t>cmd/server/main.go</t>
         </is>
       </c>
-      <c r="G56" t="inlineStr">
+      <c r="G69" t="inlineStr">
         <is>
           <t>Implemented</t>
         </is>
@@ -2582,7 +3063,7 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>bolivia-salt-flat.jpg</t>
+          <t>generated/card-salt-mirror.jpg</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -2674,7 +3155,7 @@
       </c>
       <c r="O3" t="inlineStr" s="1">
         <is>
-          <t>iceland-lava-tunnel.jpg</t>
+          <t>generated/card-lava-tunnel.jpg</t>
         </is>
       </c>
       <c r="P3" t="inlineStr" s="1">
@@ -2766,7 +3247,7 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>japan-temple-onsen.jpg</t>
+          <t>generated/card-temple-onsen.jpg</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
@@ -2858,7 +3339,7 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>morocco-sahara-camp.jpg</t>
+          <t>generated/card-sahara-stars.jpg</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
@@ -2950,7 +3431,7 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>greenland-dog-sled.jpg</t>
+          <t>generated/card-greenland-sled.jpg</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
@@ -3042,7 +3523,7 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>norway-aurora.jpg</t>
+          <t>norway-aurora-2.jpg</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">

</xml_diff>

<commit_message>
feat(content): authored entrances as bilingual JSON, structured detail page
Each journey can now be written as one JSON file under internal/content/entrances
(embedded in the binary). Files are validated by tests (structure, vocabulary,
covers, and a lint that rejects type codes and "telling" copy) and synced into
SQLite at startup, overriding the seed rows they describe.

The API adds `entrance` and localized `content` to journeys; the detail page
renders the role, chapters, an interactive fork that marks the ticket, the
ending, and a "what is real, what is not" footnote with sources.

docs/content/SCHEMA.md documents the contract; IMAGE_SOURCES.md tracks cover
licences. Entrance No. 1 (Salar de Uyuni) is the first rewritten journey.
</commit_message>
<xml_diff>
--- a/app.xlsx
+++ b/app.xlsx
@@ -154,7 +154,7 @@
         </is>
       </c>
       <c r="B4">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -242,7 +242,7 @@
         </is>
       </c>
       <c r="E7">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="8">
@@ -669,7 +669,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>admin_handler_test</t>
+          <t>content_test</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -679,7 +679,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>internal/handler/admin_handler_test.go</t>
+          <t>internal/content/content_test.go</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -706,7 +706,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>auth_handler_test</t>
+          <t>admin_handler_test</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -716,7 +716,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>internal/handler/auth_handler_test.go</t>
+          <t>internal/handler/admin_handler_test.go</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -743,7 +743,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>journey_handler_test</t>
+          <t>auth_handler_test</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -753,7 +753,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>internal/handler/journey_handler_test.go</t>
+          <t>internal/handler/auth_handler_test.go</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -780,7 +780,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>me_handler_test</t>
+          <t>journey_handler_test</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -790,7 +790,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>internal/handler/me_handler_test.go</t>
+          <t>internal/handler/journey_handler_test.go</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -817,7 +817,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>order_handler_test</t>
+          <t>me_handler_test</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -827,7 +827,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>internal/handler/order_handler_test.go</t>
+          <t>internal/handler/me_handler_test.go</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -854,7 +854,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>payment_handler_test</t>
+          <t>order_handler_test</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -864,7 +864,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>internal/handler/payment_handler_test.go</t>
+          <t>internal/handler/order_handler_test.go</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -891,7 +891,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>cors_test</t>
+          <t>payment_handler_test</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -901,7 +901,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>internal/middleware/cors_test.go</t>
+          <t>internal/handler/payment_handler_test.go</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -928,7 +928,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>jwt_test</t>
+          <t>cors_test</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -938,7 +938,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>internal/middleware/jwt_test.go</t>
+          <t>internal/middleware/cors_test.go</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -965,7 +965,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>request_id_test</t>
+          <t>jwt_test</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -975,7 +975,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>internal/middleware/request_id_test.go</t>
+          <t>internal/middleware/jwt_test.go</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1002,7 +1002,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>journey_repo_sqlite_test</t>
+          <t>request_id_test</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1012,7 +1012,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>internal/repository/journey_repo_sqlite_test.go</t>
+          <t>internal/middleware/request_id_test.go</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1039,7 +1039,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>order_repo_test</t>
+          <t>journey_repo_sqlite_test</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1049,7 +1049,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>internal/repository/order_repo_test.go</t>
+          <t>internal/repository/journey_repo_sqlite_test.go</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1076,7 +1076,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>user_repo_test</t>
+          <t>order_repo_test</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1086,7 +1086,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>internal/repository/user_repo_test.go</t>
+          <t>internal/repository/order_repo_test.go</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1113,7 +1113,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>journey_service_test</t>
+          <t>user_repo_test</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1123,7 +1123,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>internal/service/journey_service_test.go</t>
+          <t>internal/repository/user_repo_test.go</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1150,7 +1150,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>locale_test</t>
+          <t>journey_service_test</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1160,7 +1160,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>internal/service/locale_test.go</t>
+          <t>internal/service/journey_service_test.go</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1187,7 +1187,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>index_test</t>
+          <t>locale_test</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1197,7 +1197,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>internal/webapp/index_test.go</t>
+          <t>internal/service/locale_test.go</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1219,12 +1219,12 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Playwright E2E</t>
+          <t>Go unit/integration / Go 单元集成</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>a11y.spec</t>
+          <t>index_test</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1234,7 +1234,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>e2e/tests/a11y.spec.js</t>
+          <t>internal/webapp/index_test.go</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1261,7 +1261,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>auth.spec</t>
+          <t>a11y.spec</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1271,7 +1271,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>e2e/tests/auth.spec.js</t>
+          <t>e2e/tests/a11y.spec.js</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1298,7 +1298,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>detail.spec</t>
+          <t>auth.spec</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>e2e/tests/detail.spec.js</t>
+          <t>e2e/tests/auth.spec.js</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1335,7 +1335,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>explore.spec</t>
+          <t>detail.spec</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -1345,7 +1345,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>e2e/tests/explore.spec.js</t>
+          <t>e2e/tests/detail.spec.js</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1372,7 +1372,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>home.spec</t>
+          <t>explore.spec</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1382,7 +1382,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>e2e/tests/home.spec.js</t>
+          <t>e2e/tests/explore.spec.js</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1409,7 +1409,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>i18n.spec</t>
+          <t>home.spec</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1419,7 +1419,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>e2e/tests/i18n.spec.js</t>
+          <t>e2e/tests/home.spec.js</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -1446,7 +1446,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>mobile.spec</t>
+          <t>i18n.spec</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1456,7 +1456,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>e2e/tests/mobile.spec.js</t>
+          <t>e2e/tests/i18n.spec.js</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -1483,7 +1483,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>orders.spec</t>
+          <t>mobile.spec</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -1493,7 +1493,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>e2e/tests/orders.spec.js</t>
+          <t>e2e/tests/mobile.spec.js</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -1520,7 +1520,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>persona.spec</t>
+          <t>orders.spec</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1530,7 +1530,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>e2e/tests/persona.spec.js</t>
+          <t>e2e/tests/orders.spec.js</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -1552,12 +1552,12 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Playwright support / E2E 支撑文件</t>
+          <t>Playwright E2E</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>helpers</t>
+          <t>persona.spec</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -1567,7 +1567,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>e2e/tests/helpers.js</t>
+          <t>e2e/tests/persona.spec.js</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -1589,12 +1589,12 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Go stress</t>
+          <t>Playwright support / E2E 支撑文件</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>stress_test</t>
+          <t>helpers</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -1604,7 +1604,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>tests/stress/stress_test.go</t>
+          <t>e2e/tests/helpers.js</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -1626,12 +1626,12 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>k6 load / k6 负载</t>
+          <t>Go stress</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>admin-analytics-export.k6</t>
+          <t>stress_test</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -1641,7 +1641,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>tests/load/admin-analytics-export.k6.js</t>
+          <t>tests/stress/stress_test.go</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -1668,7 +1668,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>auth-register-login.k6</t>
+          <t>admin-analytics-export.k6</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -1678,7 +1678,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>tests/load/auth-register-login.k6.js</t>
+          <t>tests/load/admin-analytics-export.k6.js</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -1705,7 +1705,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>image-static-cache.k6</t>
+          <t>auth-register-login.k6</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -1715,7 +1715,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>tests/load/image-static-cache.k6.js</t>
+          <t>tests/load/auth-register-login.k6.js</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -1742,7 +1742,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>order-payment-audit.k6</t>
+          <t>image-static-cache.k6</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -1752,7 +1752,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>tests/load/order-payment-audit.k6.js</t>
+          <t>tests/load/image-static-cache.k6.js</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -1779,7 +1779,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>pet-chat-analytics.k6</t>
+          <t>order-payment-audit.k6</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -1789,7 +1789,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>tests/load/pet-chat-analytics.k6.js</t>
+          <t>tests/load/order-payment-audit.k6.js</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -1816,7 +1816,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>public-content-flow.k6</t>
+          <t>pet-chat-analytics.k6</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -1826,7 +1826,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>tests/load/public-content-flow.k6.js</t>
+          <t>tests/load/pet-chat-analytics.k6.js</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -1838,37 +1838,37 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Route</t>
+          <t>Test</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>ROUTE-001</t>
+          <t>TEST-036</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Admin</t>
+          <t>k6 load / k6 负载</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>GET /api/admin/export</t>
+          <t>public-content-flow.k6</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Route is registered</t>
+          <t>File exists and is part of repo</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>internal/handler/admin_handler.go</t>
+          <t>tests/load/public-content-flow.k6.js</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Specified</t>
         </is>
       </c>
     </row>
@@ -1880,7 +1880,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>ROUTE-002</t>
+          <t>ROUTE-001</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1890,7 +1890,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>GET /api/admin/stats</t>
+          <t>GET /api/admin/export</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -1917,7 +1917,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>ROUTE-003</t>
+          <t>ROUTE-002</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -1927,7 +1927,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>GET /api/admin/users</t>
+          <t>GET /api/admin/stats</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -1954,17 +1954,17 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>ROUTE-004</t>
+          <t>ROUTE-003</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>Admin</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>POST /api/ai/chat</t>
+          <t>GET /api/admin/users</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -1974,7 +1974,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>internal/handler/admin_handler.go</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -1991,7 +1991,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>ROUTE-005</t>
+          <t>ROUTE-004</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2001,7 +2001,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>POST /api/analytics/events</t>
+          <t>POST /api/ai/chat</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -2028,7 +2028,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>ROUTE-006</t>
+          <t>ROUTE-005</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2038,7 +2038,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>POST /api/audit/client-error</t>
+          <t>POST /api/analytics/events</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -2065,17 +2065,17 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>ROUTE-007</t>
+          <t>ROUTE-006</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>POST /api/auth/avatar</t>
+          <t>POST /api/audit/client-error</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -2102,17 +2102,17 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>ROUTE-008</t>
+          <t>ROUTE-007</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>JWT</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>POST /api/auth/login</t>
+          <t>POST /api/auth/avatar</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -2139,17 +2139,17 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>ROUTE-009</t>
+          <t>ROUTE-008</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>PUT /api/auth/mbti</t>
+          <t>POST /api/auth/login</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -2159,7 +2159,7 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>internal/handler/me_handler.go</t>
+          <t>cmd/server/main.go</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -2176,7 +2176,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>ROUTE-010</t>
+          <t>ROUTE-009</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2186,7 +2186,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>GET /api/auth/me</t>
+          <t>PUT /api/auth/mbti</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -2196,7 +2196,7 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>internal/handler/me_handler.go</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -2213,17 +2213,17 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>ROUTE-011</t>
+          <t>ROUTE-010</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>JWT</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>POST /api/auth/register</t>
+          <t>GET /api/auth/me</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -2250,17 +2250,17 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>ROUTE-012</t>
+          <t>ROUTE-011</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>GET /api/auth/saved</t>
+          <t>POST /api/auth/register</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -2270,7 +2270,7 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>internal/handler/me_handler.go</t>
+          <t>cmd/server/main.go</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -2287,7 +2287,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>ROUTE-013</t>
+          <t>ROUTE-012</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2297,7 +2297,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>DELETE /api/auth/saved/:slug</t>
+          <t>GET /api/auth/saved</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -2324,7 +2324,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>ROUTE-014</t>
+          <t>ROUTE-013</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2334,7 +2334,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>PUT /api/auth/saved/:slug</t>
+          <t>DELETE /api/auth/saved/:slug</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -2361,17 +2361,17 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>ROUTE-015</t>
+          <t>ROUTE-014</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>JWT</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>GET /api/captcha</t>
+          <t>PUT /api/auth/saved/:slug</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -2381,7 +2381,7 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>internal/handler/me_handler.go</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -2398,7 +2398,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>ROUTE-016</t>
+          <t>ROUTE-015</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -2408,7 +2408,7 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>GET /api/health</t>
+          <t>GET /api/captcha</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -2435,7 +2435,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>ROUTE-017</t>
+          <t>ROUTE-016</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -2445,7 +2445,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>GET /api/journeys</t>
+          <t>GET /api/health</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -2472,7 +2472,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>ROUTE-018</t>
+          <t>ROUTE-017</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -2482,7 +2482,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>GET /api/journeys/:slug</t>
+          <t>GET /api/journeys</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -2509,7 +2509,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>ROUTE-019</t>
+          <t>ROUTE-018</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -2519,7 +2519,7 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>GET /api/journeys/:slug/book</t>
+          <t>GET /api/journeys/:slug</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -2546,7 +2546,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>ROUTE-020</t>
+          <t>ROUTE-019</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -2556,7 +2556,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>GET /api/mbti</t>
+          <t>GET /api/journeys/:slug/book</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -2583,17 +2583,17 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>ROUTE-021</t>
+          <t>ROUTE-020</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>GET /api/orders</t>
+          <t>GET /api/mbti</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -2603,7 +2603,7 @@
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>internal/handler/order_handler.go</t>
+          <t>cmd/server/main.go</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
@@ -2620,7 +2620,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>ROUTE-022</t>
+          <t>ROUTE-021</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -2630,7 +2630,7 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>POST /api/orders</t>
+          <t>GET /api/orders</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -2657,7 +2657,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>ROUTE-023</t>
+          <t>ROUTE-022</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -2667,7 +2667,7 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>GET /api/orders/:id</t>
+          <t>POST /api/orders</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -2694,7 +2694,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>ROUTE-024</t>
+          <t>ROUTE-023</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -2704,7 +2704,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>POST /api/orders/:id/pay</t>
+          <t>GET /api/orders/:id</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -2731,7 +2731,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>ROUTE-025</t>
+          <t>ROUTE-024</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -2741,7 +2741,7 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>POST /api/payments/recharge</t>
+          <t>POST /api/orders/:id/pay</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -2751,7 +2751,7 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>internal/handler/payment_handler.go</t>
+          <t>internal/handler/order_handler.go</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
@@ -2768,17 +2768,17 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>ROUTE-026</t>
+          <t>ROUTE-025</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>JWT</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>GET /api/payments/tiers</t>
+          <t>POST /api/payments/recharge</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -2805,17 +2805,17 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>ROUTE-027</t>
+          <t>ROUTE-026</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>GET /api/payments/transactions</t>
+          <t>GET /api/payments/tiers</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -2842,30 +2842,67 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
+          <t>ROUTE-027</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>JWT</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>GET /api/payments/transactions</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Route is registered</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>internal/handler/payment_handler.go</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Route</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
           <t>ROUTE-028</t>
         </is>
       </c>
-      <c r="C69" t="inlineStr">
+      <c r="C70" t="inlineStr">
         <is>
           <t>Public</t>
         </is>
       </c>
-      <c r="D69" t="inlineStr">
+      <c r="D70" t="inlineStr">
         <is>
           <t>GET /api/tags</t>
         </is>
       </c>
-      <c r="E69" t="inlineStr">
+      <c r="E70" t="inlineStr">
         <is>
           <t>Route is registered</t>
         </is>
       </c>
-      <c r="F69" t="inlineStr">
+      <c r="F70" t="inlineStr">
         <is>
           <t>cmd/server/main.go</t>
         </is>
       </c>
-      <c r="G69" t="inlineStr">
+      <c r="G70" t="inlineStr">
         <is>
           <t>Implemented</t>
         </is>

</xml_diff>

<commit_message>
Lantern Night redesign, bilingual content and checkout (#2)
- New "Lantern Night" design system with a working light theme; WCAG 2.1 AA (axe: 102 violation nodes on the old pages, 0 now).
- zh/en interface and content (`?lang=en`, English search).
- Saved journeys and travel personality stored on the account.
- In-page checkout with points discount; recharge tiers whose bonus is actually credited; daily login reward.
- Fixes: search hidden under the nav, filters stuck on skeletons, raw HTTP errors, no log-in on phones, 500 on unknown routes, stale assets after deploys (fingerprinted CSS/JS).
- README rewritten as a product page; internal process documents and a committed binary removed.
- Tests: +18 Go tests; Playwright rewritten (66 tests, desktop + Pixel 7, axe scans in both themes).
</commit_message>
<xml_diff>
--- a/app.xlsx
+++ b/app.xlsx
@@ -154,7 +154,7 @@
         </is>
       </c>
       <c r="B4">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -217,7 +217,7 @@
         </is>
       </c>
       <c r="E6">
-        <v>23</v>
+        <v>28</v>
       </c>
     </row>
     <row r="7">
@@ -242,7 +242,7 @@
         </is>
       </c>
       <c r="E7">
-        <v>27</v>
+        <v>35</v>
       </c>
     </row>
     <row r="8">
@@ -780,7 +780,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>order_handler_test</t>
+          <t>me_handler_test</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -790,7 +790,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>internal/handler/order_handler_test.go</t>
+          <t>internal/handler/me_handler_test.go</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -817,7 +817,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>cors_test</t>
+          <t>order_handler_test</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -827,7 +827,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>internal/middleware/cors_test.go</t>
+          <t>internal/handler/order_handler_test.go</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -854,7 +854,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>jwt_test</t>
+          <t>payment_handler_test</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -864,7 +864,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>internal/middleware/jwt_test.go</t>
+          <t>internal/handler/payment_handler_test.go</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -891,7 +891,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>request_id_test</t>
+          <t>cors_test</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -901,7 +901,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>internal/middleware/request_id_test.go</t>
+          <t>internal/middleware/cors_test.go</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -928,7 +928,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>journey_repo_sqlite_test</t>
+          <t>jwt_test</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -938,7 +938,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>internal/repository/journey_repo_sqlite_test.go</t>
+          <t>internal/middleware/jwt_test.go</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -965,7 +965,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>order_repo_test</t>
+          <t>request_id_test</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -975,7 +975,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>internal/repository/order_repo_test.go</t>
+          <t>internal/middleware/request_id_test.go</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1002,7 +1002,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>user_repo_test</t>
+          <t>journey_repo_sqlite_test</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1012,7 +1012,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>internal/repository/user_repo_test.go</t>
+          <t>internal/repository/journey_repo_sqlite_test.go</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1039,7 +1039,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>journey_service_test</t>
+          <t>order_repo_test</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1049,7 +1049,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>internal/service/journey_service_test.go</t>
+          <t>internal/repository/order_repo_test.go</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1071,12 +1071,12 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Playwright E2E</t>
+          <t>Go unit/integration / Go 单元集成</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>auth.spec</t>
+          <t>user_repo_test</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1086,7 +1086,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>e2e/tests/auth.spec.js</t>
+          <t>internal/repository/user_repo_test.go</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1108,12 +1108,12 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Playwright E2E</t>
+          <t>Go unit/integration / Go 单元集成</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>detail.spec</t>
+          <t>journey_service_test</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1123,7 +1123,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>e2e/tests/detail.spec.js</t>
+          <t>internal/service/journey_service_test.go</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1145,12 +1145,12 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Playwright E2E</t>
+          <t>Go unit/integration / Go 单元集成</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>explore.spec</t>
+          <t>locale_test</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1160,7 +1160,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>e2e/tests/explore.spec.js</t>
+          <t>internal/service/locale_test.go</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1182,12 +1182,12 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Playwright E2E</t>
+          <t>Go unit/integration / Go 单元集成</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>home.spec</t>
+          <t>index_test</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1197,7 +1197,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>e2e/tests/home.spec.js</t>
+          <t>internal/webapp/index_test.go</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1224,7 +1224,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>orders.spec</t>
+          <t>a11y.spec</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1234,7 +1234,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>e2e/tests/orders.spec.js</t>
+          <t>e2e/tests/a11y.spec.js</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1256,12 +1256,12 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Playwright support / E2E 支撑文件</t>
+          <t>Playwright E2E</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>helpers</t>
+          <t>auth.spec</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1271,7 +1271,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>e2e/tests/helpers.js</t>
+          <t>e2e/tests/auth.spec.js</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1293,12 +1293,12 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Go stress</t>
+          <t>Playwright E2E</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>stress_test</t>
+          <t>detail.spec</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>tests/stress/stress_test.go</t>
+          <t>e2e/tests/detail.spec.js</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1330,12 +1330,12 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>k6 load / k6 负载</t>
+          <t>Playwright E2E</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>admin-analytics-export.k6</t>
+          <t>explore.spec</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -1345,7 +1345,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>tests/load/admin-analytics-export.k6.js</t>
+          <t>e2e/tests/explore.spec.js</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1367,12 +1367,12 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>k6 load / k6 负载</t>
+          <t>Playwright E2E</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>auth-register-login.k6</t>
+          <t>home.spec</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1382,7 +1382,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>tests/load/auth-register-login.k6.js</t>
+          <t>e2e/tests/home.spec.js</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1404,12 +1404,12 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>k6 load / k6 负载</t>
+          <t>Playwright E2E</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>image-static-cache.k6</t>
+          <t>i18n.spec</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1419,7 +1419,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>tests/load/image-static-cache.k6.js</t>
+          <t>e2e/tests/i18n.spec.js</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -1441,12 +1441,12 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>k6 load / k6 负载</t>
+          <t>Playwright E2E</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>order-payment-audit.k6</t>
+          <t>mobile.spec</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1456,7 +1456,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>tests/load/order-payment-audit.k6.js</t>
+          <t>e2e/tests/mobile.spec.js</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -1478,12 +1478,12 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>k6 load / k6 负载</t>
+          <t>Playwright E2E</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>pet-chat-analytics.k6</t>
+          <t>orders.spec</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -1493,7 +1493,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>tests/load/pet-chat-analytics.k6.js</t>
+          <t>e2e/tests/orders.spec.js</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -1515,12 +1515,12 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>k6 load / k6 负载</t>
+          <t>Playwright E2E</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>public-content-flow.k6</t>
+          <t>persona.spec</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1530,7 +1530,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>tests/load/public-content-flow.k6.js</t>
+          <t>e2e/tests/persona.spec.js</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -1542,296 +1542,296 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Route</t>
+          <t>Test</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>ROUTE-001</t>
+          <t>TEST-028</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Admin</t>
+          <t>Playwright support / E2E 支撑文件</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>GET /api/admin/export</t>
+          <t>helpers</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Route is registered</t>
+          <t>File exists and is part of repo</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>internal/handler/admin_handler.go</t>
+          <t>e2e/tests/helpers.js</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Specified</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Route</t>
+          <t>Test</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>ROUTE-002</t>
+          <t>TEST-029</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Admin</t>
+          <t>Go stress</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>GET /api/admin/stats</t>
+          <t>stress_test</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Route is registered</t>
+          <t>File exists and is part of repo</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>internal/handler/admin_handler.go</t>
+          <t>tests/stress/stress_test.go</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Specified</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Route</t>
+          <t>Test</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>ROUTE-003</t>
+          <t>TEST-030</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Admin</t>
+          <t>k6 load / k6 负载</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>GET /api/admin/users</t>
+          <t>admin-analytics-export.k6</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Route is registered</t>
+          <t>File exists and is part of repo</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>internal/handler/admin_handler.go</t>
+          <t>tests/load/admin-analytics-export.k6.js</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Specified</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Route</t>
+          <t>Test</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>ROUTE-004</t>
+          <t>TEST-031</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>k6 load / k6 负载</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>POST /api/ai/chat</t>
+          <t>auth-register-login.k6</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Route is registered</t>
+          <t>File exists and is part of repo</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>tests/load/auth-register-login.k6.js</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Specified</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Route</t>
+          <t>Test</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>ROUTE-005</t>
+          <t>TEST-032</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>k6 load / k6 负载</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>POST /api/analytics/events</t>
+          <t>image-static-cache.k6</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Route is registered</t>
+          <t>File exists and is part of repo</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>tests/load/image-static-cache.k6.js</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Specified</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Route</t>
+          <t>Test</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>ROUTE-006</t>
+          <t>TEST-033</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>k6 load / k6 负载</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>POST /api/audit/client-error</t>
+          <t>order-payment-audit.k6</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Route is registered</t>
+          <t>File exists and is part of repo</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>tests/load/order-payment-audit.k6.js</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Specified</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Route</t>
+          <t>Test</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>ROUTE-007</t>
+          <t>TEST-034</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>k6 load / k6 负载</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>POST /api/auth/avatar</t>
+          <t>pet-chat-analytics.k6</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Route is registered</t>
+          <t>File exists and is part of repo</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>tests/load/pet-chat-analytics.k6.js</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Specified</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Route</t>
+          <t>Test</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>ROUTE-008</t>
+          <t>TEST-035</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>k6 load / k6 负载</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>POST /api/auth/login</t>
+          <t>public-content-flow.k6</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Route is registered</t>
+          <t>File exists and is part of repo</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>tests/load/public-content-flow.k6.js</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Specified</t>
         </is>
       </c>
     </row>
@@ -1843,17 +1843,17 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>ROUTE-009</t>
+          <t>ROUTE-001</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Admin</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>GET /api/auth/me</t>
+          <t>GET /api/admin/export</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -1863,7 +1863,7 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>internal/handler/admin_handler.go</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -1880,17 +1880,17 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>ROUTE-010</t>
+          <t>ROUTE-002</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>Admin</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>POST /api/auth/register</t>
+          <t>GET /api/admin/stats</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -1900,7 +1900,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>internal/handler/admin_handler.go</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -1917,17 +1917,17 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>ROUTE-011</t>
+          <t>ROUTE-003</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>Admin</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>GET /api/captcha</t>
+          <t>GET /api/admin/users</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -1937,7 +1937,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>internal/handler/admin_handler.go</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -1954,7 +1954,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>ROUTE-012</t>
+          <t>ROUTE-004</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -1964,7 +1964,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>GET /api/health</t>
+          <t>POST /api/ai/chat</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -1991,7 +1991,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>ROUTE-013</t>
+          <t>ROUTE-005</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2001,7 +2001,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>GET /api/journeys</t>
+          <t>POST /api/analytics/events</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -2028,7 +2028,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>ROUTE-014</t>
+          <t>ROUTE-006</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2038,7 +2038,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>GET /api/journeys/:slug</t>
+          <t>POST /api/audit/client-error</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -2065,17 +2065,17 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>ROUTE-015</t>
+          <t>ROUTE-007</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>JWT</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>GET /api/journeys/:slug/book</t>
+          <t>POST /api/auth/avatar</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -2102,7 +2102,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>ROUTE-016</t>
+          <t>ROUTE-008</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2112,7 +2112,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>GET /api/mbti</t>
+          <t>POST /api/auth/login</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -2139,7 +2139,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>ROUTE-017</t>
+          <t>ROUTE-009</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2149,7 +2149,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>GET /api/orders</t>
+          <t>PUT /api/auth/mbti</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -2159,7 +2159,7 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>internal/handler/order_handler.go</t>
+          <t>internal/handler/me_handler.go</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -2176,7 +2176,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>ROUTE-018</t>
+          <t>ROUTE-010</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2186,7 +2186,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>POST /api/orders</t>
+          <t>GET /api/auth/me</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -2196,7 +2196,7 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>internal/handler/order_handler.go</t>
+          <t>cmd/server/main.go</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -2213,17 +2213,17 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>ROUTE-019</t>
+          <t>ROUTE-011</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>GET /api/orders/:id</t>
+          <t>POST /api/auth/register</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -2233,7 +2233,7 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>internal/handler/order_handler.go</t>
+          <t>cmd/server/main.go</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -2250,7 +2250,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>ROUTE-020</t>
+          <t>ROUTE-012</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2260,7 +2260,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>POST /api/orders/:id/pay</t>
+          <t>GET /api/auth/saved</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -2270,7 +2270,7 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>internal/handler/order_handler.go</t>
+          <t>internal/handler/me_handler.go</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -2287,7 +2287,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>ROUTE-021</t>
+          <t>ROUTE-013</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2297,7 +2297,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>POST /api/payments/recharge</t>
+          <t>DELETE /api/auth/saved/:slug</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -2307,7 +2307,7 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>internal/handler/payment_handler.go</t>
+          <t>internal/handler/me_handler.go</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -2324,7 +2324,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>ROUTE-022</t>
+          <t>ROUTE-014</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2334,7 +2334,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>GET /api/payments/transactions</t>
+          <t>PUT /api/auth/saved/:slug</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -2344,7 +2344,7 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>internal/handler/payment_handler.go</t>
+          <t>internal/handler/me_handler.go</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -2361,30 +2361,511 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
+          <t>ROUTE-015</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>GET /api/captcha</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Route is registered</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>cmd/server/main.go</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Route</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>ROUTE-016</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>GET /api/health</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Route is registered</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>cmd/server/main.go</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Route</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>ROUTE-017</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>GET /api/journeys</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Route is registered</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>cmd/server/main.go</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Route</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>ROUTE-018</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>GET /api/journeys/:slug</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Route is registered</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>cmd/server/main.go</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Route</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>ROUTE-019</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>GET /api/journeys/:slug/book</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Route is registered</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>cmd/server/main.go</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Route</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>ROUTE-020</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>GET /api/mbti</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Route is registered</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>cmd/server/main.go</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Route</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>ROUTE-021</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>JWT</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>GET /api/orders</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Route is registered</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>internal/handler/order_handler.go</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Route</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>ROUTE-022</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>JWT</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>POST /api/orders</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Route is registered</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>internal/handler/order_handler.go</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Route</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
           <t>ROUTE-023</t>
         </is>
       </c>
-      <c r="C56" t="inlineStr">
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>JWT</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>GET /api/orders/:id</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Route is registered</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>internal/handler/order_handler.go</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Route</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>ROUTE-024</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>JWT</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>POST /api/orders/:id/pay</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Route is registered</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>internal/handler/order_handler.go</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Route</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>ROUTE-025</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>JWT</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>POST /api/payments/recharge</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Route is registered</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>internal/handler/payment_handler.go</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Route</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>ROUTE-026</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
         <is>
           <t>Public</t>
         </is>
       </c>
-      <c r="D56" t="inlineStr">
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>GET /api/payments/tiers</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Route is registered</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>internal/handler/payment_handler.go</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Route</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>ROUTE-027</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>JWT</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>GET /api/payments/transactions</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Route is registered</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>internal/handler/payment_handler.go</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Route</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>ROUTE-028</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
         <is>
           <t>GET /api/tags</t>
         </is>
       </c>
-      <c r="E56" t="inlineStr">
+      <c r="E69" t="inlineStr">
         <is>
           <t>Route is registered</t>
         </is>
       </c>
-      <c r="F56" t="inlineStr">
+      <c r="F69" t="inlineStr">
         <is>
           <t>cmd/server/main.go</t>
         </is>
       </c>
-      <c r="G56" t="inlineStr">
+      <c r="G69" t="inlineStr">
         <is>
           <t>Implemented</t>
         </is>
@@ -2582,7 +3063,7 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>bolivia-salt-flat.jpg</t>
+          <t>generated/card-salt-mirror.jpg</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -2674,7 +3155,7 @@
       </c>
       <c r="O3" t="inlineStr" s="1">
         <is>
-          <t>iceland-lava-tunnel.jpg</t>
+          <t>generated/card-lava-tunnel.jpg</t>
         </is>
       </c>
       <c r="P3" t="inlineStr" s="1">
@@ -2766,7 +3247,7 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>japan-temple-onsen.jpg</t>
+          <t>generated/card-temple-onsen.jpg</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
@@ -2858,7 +3339,7 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>morocco-sahara-camp.jpg</t>
+          <t>generated/card-sahara-stars.jpg</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
@@ -2950,7 +3431,7 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>greenland-dog-sled.jpg</t>
+          <t>generated/card-greenland-sled.jpg</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
@@ -3042,7 +3523,7 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>norway-aurora.jpg</t>
+          <t>norway-aurora-2.jpg</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
@@ -3825,7 +4306,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>workflow 已新增，远端运行待 push 后确认</t>
+          <t>Go、Playwright E2E、k6 smoke；main 全绿后自动部署到 AWS Lightsail</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Authored entrances: bilingual JSON content and structured detail page (#3)
- Journeys can be written as one bilingual JSON file each (internal/content/entrances), validated by tests and synced into SQLite at startup; contract in docs/content/SCHEMA.md.
- API adds `entrance` and localized `content`; the detail page renders role, chapters, a fork that marks the ticket, the ending, and a sourced "what is real, what is not" note.
- Entrance No. 1 (Salar de Uyuni) rewritten; cover licences tracked in docs/content/IMAGE_SOURCES.md.
</commit_message>
<xml_diff>
--- a/app.xlsx
+++ b/app.xlsx
@@ -154,7 +154,7 @@
         </is>
       </c>
       <c r="B4">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -242,7 +242,7 @@
         </is>
       </c>
       <c r="E7">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="8">
@@ -669,7 +669,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>admin_handler_test</t>
+          <t>content_test</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -679,7 +679,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>internal/handler/admin_handler_test.go</t>
+          <t>internal/content/content_test.go</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -706,7 +706,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>auth_handler_test</t>
+          <t>admin_handler_test</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -716,7 +716,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>internal/handler/auth_handler_test.go</t>
+          <t>internal/handler/admin_handler_test.go</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -743,7 +743,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>journey_handler_test</t>
+          <t>auth_handler_test</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -753,7 +753,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>internal/handler/journey_handler_test.go</t>
+          <t>internal/handler/auth_handler_test.go</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -780,7 +780,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>me_handler_test</t>
+          <t>journey_handler_test</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -790,7 +790,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>internal/handler/me_handler_test.go</t>
+          <t>internal/handler/journey_handler_test.go</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -817,7 +817,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>order_handler_test</t>
+          <t>me_handler_test</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -827,7 +827,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>internal/handler/order_handler_test.go</t>
+          <t>internal/handler/me_handler_test.go</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -854,7 +854,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>payment_handler_test</t>
+          <t>order_handler_test</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -864,7 +864,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>internal/handler/payment_handler_test.go</t>
+          <t>internal/handler/order_handler_test.go</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -891,7 +891,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>cors_test</t>
+          <t>payment_handler_test</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -901,7 +901,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>internal/middleware/cors_test.go</t>
+          <t>internal/handler/payment_handler_test.go</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -928,7 +928,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>jwt_test</t>
+          <t>cors_test</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -938,7 +938,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>internal/middleware/jwt_test.go</t>
+          <t>internal/middleware/cors_test.go</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -965,7 +965,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>request_id_test</t>
+          <t>jwt_test</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -975,7 +975,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>internal/middleware/request_id_test.go</t>
+          <t>internal/middleware/jwt_test.go</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1002,7 +1002,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>journey_repo_sqlite_test</t>
+          <t>request_id_test</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1012,7 +1012,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>internal/repository/journey_repo_sqlite_test.go</t>
+          <t>internal/middleware/request_id_test.go</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1039,7 +1039,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>order_repo_test</t>
+          <t>journey_repo_sqlite_test</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1049,7 +1049,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>internal/repository/order_repo_test.go</t>
+          <t>internal/repository/journey_repo_sqlite_test.go</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1076,7 +1076,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>user_repo_test</t>
+          <t>order_repo_test</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1086,7 +1086,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>internal/repository/user_repo_test.go</t>
+          <t>internal/repository/order_repo_test.go</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1113,7 +1113,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>journey_service_test</t>
+          <t>user_repo_test</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1123,7 +1123,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>internal/service/journey_service_test.go</t>
+          <t>internal/repository/user_repo_test.go</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1150,7 +1150,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>locale_test</t>
+          <t>journey_service_test</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1160,7 +1160,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>internal/service/locale_test.go</t>
+          <t>internal/service/journey_service_test.go</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1187,7 +1187,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>index_test</t>
+          <t>locale_test</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1197,7 +1197,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>internal/webapp/index_test.go</t>
+          <t>internal/service/locale_test.go</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1219,12 +1219,12 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Playwright E2E</t>
+          <t>Go unit/integration / Go 单元集成</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>a11y.spec</t>
+          <t>index_test</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1234,7 +1234,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>e2e/tests/a11y.spec.js</t>
+          <t>internal/webapp/index_test.go</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1261,7 +1261,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>auth.spec</t>
+          <t>a11y.spec</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1271,7 +1271,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>e2e/tests/auth.spec.js</t>
+          <t>e2e/tests/a11y.spec.js</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1298,7 +1298,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>detail.spec</t>
+          <t>auth.spec</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>e2e/tests/detail.spec.js</t>
+          <t>e2e/tests/auth.spec.js</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1335,7 +1335,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>explore.spec</t>
+          <t>detail.spec</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -1345,7 +1345,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>e2e/tests/explore.spec.js</t>
+          <t>e2e/tests/detail.spec.js</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1372,7 +1372,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>home.spec</t>
+          <t>explore.spec</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1382,7 +1382,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>e2e/tests/home.spec.js</t>
+          <t>e2e/tests/explore.spec.js</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1409,7 +1409,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>i18n.spec</t>
+          <t>home.spec</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1419,7 +1419,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>e2e/tests/i18n.spec.js</t>
+          <t>e2e/tests/home.spec.js</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -1446,7 +1446,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>mobile.spec</t>
+          <t>i18n.spec</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1456,7 +1456,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>e2e/tests/mobile.spec.js</t>
+          <t>e2e/tests/i18n.spec.js</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -1483,7 +1483,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>orders.spec</t>
+          <t>mobile.spec</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -1493,7 +1493,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>e2e/tests/orders.spec.js</t>
+          <t>e2e/tests/mobile.spec.js</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -1520,7 +1520,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>persona.spec</t>
+          <t>orders.spec</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1530,7 +1530,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>e2e/tests/persona.spec.js</t>
+          <t>e2e/tests/orders.spec.js</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -1552,12 +1552,12 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Playwright support / E2E 支撑文件</t>
+          <t>Playwright E2E</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>helpers</t>
+          <t>persona.spec</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -1567,7 +1567,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>e2e/tests/helpers.js</t>
+          <t>e2e/tests/persona.spec.js</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -1589,12 +1589,12 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Go stress</t>
+          <t>Playwright support / E2E 支撑文件</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>stress_test</t>
+          <t>helpers</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -1604,7 +1604,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>tests/stress/stress_test.go</t>
+          <t>e2e/tests/helpers.js</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -1626,12 +1626,12 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>k6 load / k6 负载</t>
+          <t>Go stress</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>admin-analytics-export.k6</t>
+          <t>stress_test</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -1641,7 +1641,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>tests/load/admin-analytics-export.k6.js</t>
+          <t>tests/stress/stress_test.go</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -1668,7 +1668,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>auth-register-login.k6</t>
+          <t>admin-analytics-export.k6</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -1678,7 +1678,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>tests/load/auth-register-login.k6.js</t>
+          <t>tests/load/admin-analytics-export.k6.js</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -1705,7 +1705,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>image-static-cache.k6</t>
+          <t>auth-register-login.k6</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -1715,7 +1715,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>tests/load/image-static-cache.k6.js</t>
+          <t>tests/load/auth-register-login.k6.js</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -1742,7 +1742,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>order-payment-audit.k6</t>
+          <t>image-static-cache.k6</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -1752,7 +1752,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>tests/load/order-payment-audit.k6.js</t>
+          <t>tests/load/image-static-cache.k6.js</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -1779,7 +1779,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>pet-chat-analytics.k6</t>
+          <t>order-payment-audit.k6</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -1789,7 +1789,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>tests/load/pet-chat-analytics.k6.js</t>
+          <t>tests/load/order-payment-audit.k6.js</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -1816,7 +1816,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>public-content-flow.k6</t>
+          <t>pet-chat-analytics.k6</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -1826,7 +1826,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>tests/load/public-content-flow.k6.js</t>
+          <t>tests/load/pet-chat-analytics.k6.js</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -1838,37 +1838,37 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Route</t>
+          <t>Test</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>ROUTE-001</t>
+          <t>TEST-036</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Admin</t>
+          <t>k6 load / k6 负载</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>GET /api/admin/export</t>
+          <t>public-content-flow.k6</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Route is registered</t>
+          <t>File exists and is part of repo</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>internal/handler/admin_handler.go</t>
+          <t>tests/load/public-content-flow.k6.js</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Specified</t>
         </is>
       </c>
     </row>
@@ -1880,7 +1880,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>ROUTE-002</t>
+          <t>ROUTE-001</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1890,7 +1890,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>GET /api/admin/stats</t>
+          <t>GET /api/admin/export</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -1917,7 +1917,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>ROUTE-003</t>
+          <t>ROUTE-002</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -1927,7 +1927,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>GET /api/admin/users</t>
+          <t>GET /api/admin/stats</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -1954,17 +1954,17 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>ROUTE-004</t>
+          <t>ROUTE-003</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>Admin</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>POST /api/ai/chat</t>
+          <t>GET /api/admin/users</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -1974,7 +1974,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>internal/handler/admin_handler.go</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -1991,7 +1991,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>ROUTE-005</t>
+          <t>ROUTE-004</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2001,7 +2001,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>POST /api/analytics/events</t>
+          <t>POST /api/ai/chat</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -2028,7 +2028,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>ROUTE-006</t>
+          <t>ROUTE-005</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2038,7 +2038,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>POST /api/audit/client-error</t>
+          <t>POST /api/analytics/events</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -2065,17 +2065,17 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>ROUTE-007</t>
+          <t>ROUTE-006</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>POST /api/auth/avatar</t>
+          <t>POST /api/audit/client-error</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -2102,17 +2102,17 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>ROUTE-008</t>
+          <t>ROUTE-007</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>JWT</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>POST /api/auth/login</t>
+          <t>POST /api/auth/avatar</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -2139,17 +2139,17 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>ROUTE-009</t>
+          <t>ROUTE-008</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>PUT /api/auth/mbti</t>
+          <t>POST /api/auth/login</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -2159,7 +2159,7 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>internal/handler/me_handler.go</t>
+          <t>cmd/server/main.go</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -2176,7 +2176,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>ROUTE-010</t>
+          <t>ROUTE-009</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2186,7 +2186,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>GET /api/auth/me</t>
+          <t>PUT /api/auth/mbti</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -2196,7 +2196,7 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>internal/handler/me_handler.go</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -2213,17 +2213,17 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>ROUTE-011</t>
+          <t>ROUTE-010</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>JWT</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>POST /api/auth/register</t>
+          <t>GET /api/auth/me</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -2250,17 +2250,17 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>ROUTE-012</t>
+          <t>ROUTE-011</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>GET /api/auth/saved</t>
+          <t>POST /api/auth/register</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -2270,7 +2270,7 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>internal/handler/me_handler.go</t>
+          <t>cmd/server/main.go</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -2287,7 +2287,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>ROUTE-013</t>
+          <t>ROUTE-012</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2297,7 +2297,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>DELETE /api/auth/saved/:slug</t>
+          <t>GET /api/auth/saved</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -2324,7 +2324,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>ROUTE-014</t>
+          <t>ROUTE-013</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2334,7 +2334,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>PUT /api/auth/saved/:slug</t>
+          <t>DELETE /api/auth/saved/:slug</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -2361,17 +2361,17 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>ROUTE-015</t>
+          <t>ROUTE-014</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>JWT</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>GET /api/captcha</t>
+          <t>PUT /api/auth/saved/:slug</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -2381,7 +2381,7 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>internal/handler/me_handler.go</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -2398,7 +2398,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>ROUTE-016</t>
+          <t>ROUTE-015</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -2408,7 +2408,7 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>GET /api/health</t>
+          <t>GET /api/captcha</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -2435,7 +2435,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>ROUTE-017</t>
+          <t>ROUTE-016</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -2445,7 +2445,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>GET /api/journeys</t>
+          <t>GET /api/health</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -2472,7 +2472,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>ROUTE-018</t>
+          <t>ROUTE-017</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -2482,7 +2482,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>GET /api/journeys/:slug</t>
+          <t>GET /api/journeys</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -2509,7 +2509,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>ROUTE-019</t>
+          <t>ROUTE-018</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -2519,7 +2519,7 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>GET /api/journeys/:slug/book</t>
+          <t>GET /api/journeys/:slug</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -2546,7 +2546,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>ROUTE-020</t>
+          <t>ROUTE-019</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -2556,7 +2556,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>GET /api/mbti</t>
+          <t>GET /api/journeys/:slug/book</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -2583,17 +2583,17 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>ROUTE-021</t>
+          <t>ROUTE-020</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>GET /api/orders</t>
+          <t>GET /api/mbti</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -2603,7 +2603,7 @@
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>internal/handler/order_handler.go</t>
+          <t>cmd/server/main.go</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
@@ -2620,7 +2620,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>ROUTE-022</t>
+          <t>ROUTE-021</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -2630,7 +2630,7 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>POST /api/orders</t>
+          <t>GET /api/orders</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -2657,7 +2657,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>ROUTE-023</t>
+          <t>ROUTE-022</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -2667,7 +2667,7 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>GET /api/orders/:id</t>
+          <t>POST /api/orders</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -2694,7 +2694,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>ROUTE-024</t>
+          <t>ROUTE-023</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -2704,7 +2704,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>POST /api/orders/:id/pay</t>
+          <t>GET /api/orders/:id</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -2731,7 +2731,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>ROUTE-025</t>
+          <t>ROUTE-024</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -2741,7 +2741,7 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>POST /api/payments/recharge</t>
+          <t>POST /api/orders/:id/pay</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -2751,7 +2751,7 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>internal/handler/payment_handler.go</t>
+          <t>internal/handler/order_handler.go</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
@@ -2768,17 +2768,17 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>ROUTE-026</t>
+          <t>ROUTE-025</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>JWT</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>GET /api/payments/tiers</t>
+          <t>POST /api/payments/recharge</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -2805,17 +2805,17 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>ROUTE-027</t>
+          <t>ROUTE-026</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>GET /api/payments/transactions</t>
+          <t>GET /api/payments/tiers</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -2842,30 +2842,67 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
+          <t>ROUTE-027</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>JWT</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>GET /api/payments/transactions</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Route is registered</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>internal/handler/payment_handler.go</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Route</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
           <t>ROUTE-028</t>
         </is>
       </c>
-      <c r="C69" t="inlineStr">
+      <c r="C70" t="inlineStr">
         <is>
           <t>Public</t>
         </is>
       </c>
-      <c r="D69" t="inlineStr">
+      <c r="D70" t="inlineStr">
         <is>
           <t>GET /api/tags</t>
         </is>
       </c>
-      <c r="E69" t="inlineStr">
+      <c r="E70" t="inlineStr">
         <is>
           <t>Route is registered</t>
         </is>
       </c>
-      <c r="F69" t="inlineStr">
+      <c r="F70" t="inlineStr">
         <is>
           <t>cmd/server/main.go</t>
         </is>
       </c>
-      <c r="G69" t="inlineStr">
+      <c r="G70" t="inlineStr">
         <is>
           <t>Implemented</t>
         </is>

</xml_diff>

<commit_message>
feat(web): find your type, walk with the guide, enter your space
The core flow now has three ways in and no dead ends:
- Home invitation: I know my type / walk with the guide / just browse;
  returning visitors get a way back to their space.
- #/find: sixteen type cards in four groups; not sure hands over to the guide.
- #/guide: six small scenes with progress; leave and resume where you were;
  ends in a reveal that leads into the space.
- #/space: entrances ordered for your type, what you took home from each fork,
  saved journeys, and for guests a prompt to keep it all in an account.
- Guest state (type, fork picks) merges into the account on sign-in; signed in,
  fork picks are stored on the account. The nav links to your space.
- Funnel events with an anonymous visitor id; admin dashboard funnel panel.
- E2E for every path in zh and en, mobile, and axe scans of the new pages.
</commit_message>
<xml_diff>
--- a/app.xlsx
+++ b/app.xlsx
@@ -154,7 +154,7 @@
         </is>
       </c>
       <c r="B4">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -242,7 +242,7 @@
         </is>
       </c>
       <c r="E7">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="8">
@@ -1076,7 +1076,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>order_repo_test</t>
+          <t>migrate_test</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1086,7 +1086,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>internal/repository/order_repo_test.go</t>
+          <t>internal/repository/migrate_test.go</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1113,7 +1113,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>user_repo_test</t>
+          <t>order_repo_test</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1123,7 +1123,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>internal/repository/user_repo_test.go</t>
+          <t>internal/repository/order_repo_test.go</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1150,7 +1150,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>journey_service_test</t>
+          <t>user_repo_test</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1160,7 +1160,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>internal/service/journey_service_test.go</t>
+          <t>internal/repository/user_repo_test.go</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1187,7 +1187,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>locale_test</t>
+          <t>journey_service_test</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1197,7 +1197,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>internal/service/locale_test.go</t>
+          <t>internal/service/journey_service_test.go</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1224,7 +1224,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>index_test</t>
+          <t>locale_test</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1234,7 +1234,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>internal/webapp/index_test.go</t>
+          <t>internal/service/locale_test.go</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1256,12 +1256,12 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Playwright E2E</t>
+          <t>Go unit/integration / Go 单元集成</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>a11y.spec</t>
+          <t>index_test</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1271,7 +1271,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>e2e/tests/a11y.spec.js</t>
+          <t>internal/webapp/index_test.go</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1298,7 +1298,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>auth.spec</t>
+          <t>a11y.spec</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>e2e/tests/auth.spec.js</t>
+          <t>e2e/tests/a11y.spec.js</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1335,7 +1335,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>detail.spec</t>
+          <t>auth.spec</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -1345,7 +1345,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>e2e/tests/detail.spec.js</t>
+          <t>e2e/tests/auth.spec.js</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1372,7 +1372,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>explore.spec</t>
+          <t>detail.spec</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1382,7 +1382,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>e2e/tests/explore.spec.js</t>
+          <t>e2e/tests/detail.spec.js</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1409,7 +1409,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>home.spec</t>
+          <t>explore.spec</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1419,7 +1419,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>e2e/tests/home.spec.js</t>
+          <t>e2e/tests/explore.spec.js</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -1446,7 +1446,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>i18n.spec</t>
+          <t>home.spec</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1456,7 +1456,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>e2e/tests/i18n.spec.js</t>
+          <t>e2e/tests/home.spec.js</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -1483,7 +1483,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>mobile.spec</t>
+          <t>i18n.spec</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -1493,7 +1493,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>e2e/tests/mobile.spec.js</t>
+          <t>e2e/tests/i18n.spec.js</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -1520,7 +1520,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>orders.spec</t>
+          <t>mobile.spec</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1530,7 +1530,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>e2e/tests/orders.spec.js</t>
+          <t>e2e/tests/mobile.spec.js</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -1557,7 +1557,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>persona.spec</t>
+          <t>orders.spec</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -1567,7 +1567,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>e2e/tests/persona.spec.js</t>
+          <t>e2e/tests/orders.spec.js</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -1589,12 +1589,12 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Playwright support / E2E 支撑文件</t>
+          <t>Playwright E2E</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>helpers</t>
+          <t>persona.spec</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -1604,7 +1604,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>e2e/tests/helpers.js</t>
+          <t>e2e/tests/persona.spec.js</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -1626,12 +1626,12 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Go stress</t>
+          <t>Playwright E2E</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>stress_test</t>
+          <t>space.spec</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -1641,7 +1641,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>tests/stress/stress_test.go</t>
+          <t>e2e/tests/space.spec.js</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -1663,12 +1663,12 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>k6 load / k6 负载</t>
+          <t>Playwright support / E2E 支撑文件</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>admin-analytics-export.k6</t>
+          <t>helpers</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -1678,7 +1678,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>tests/load/admin-analytics-export.k6.js</t>
+          <t>e2e/tests/helpers.js</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -1700,12 +1700,12 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>k6 load / k6 负载</t>
+          <t>Go stress</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>auth-register-login.k6</t>
+          <t>stress_test</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -1715,7 +1715,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>tests/load/auth-register-login.k6.js</t>
+          <t>tests/stress/stress_test.go</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -1742,7 +1742,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>image-static-cache.k6</t>
+          <t>admin-analytics-export.k6</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -1752,7 +1752,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>tests/load/image-static-cache.k6.js</t>
+          <t>tests/load/admin-analytics-export.k6.js</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -1779,7 +1779,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>order-payment-audit.k6</t>
+          <t>auth-register-login.k6</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -1789,7 +1789,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>tests/load/order-payment-audit.k6.js</t>
+          <t>tests/load/auth-register-login.k6.js</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -1816,7 +1816,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>pet-chat-analytics.k6</t>
+          <t>image-static-cache.k6</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -1826,7 +1826,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>tests/load/pet-chat-analytics.k6.js</t>
+          <t>tests/load/image-static-cache.k6.js</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -1853,7 +1853,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>public-content-flow.k6</t>
+          <t>order-payment-audit.k6</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -1863,7 +1863,7 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>tests/load/public-content-flow.k6.js</t>
+          <t>tests/load/order-payment-audit.k6.js</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -1875,74 +1875,74 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Route</t>
+          <t>Test</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>ROUTE-001</t>
+          <t>TEST-037</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Admin</t>
+          <t>k6 load / k6 负载</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>GET /api/admin/export</t>
+          <t>pet-chat-analytics.k6</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Route is registered</t>
+          <t>File exists and is part of repo</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>internal/handler/admin_handler.go</t>
+          <t>tests/load/pet-chat-analytics.k6.js</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Specified</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Route</t>
+          <t>Test</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>ROUTE-002</t>
+          <t>TEST-038</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Admin</t>
+          <t>k6 load / k6 负载</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>GET /api/admin/stats</t>
+          <t>public-content-flow.k6</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Route is registered</t>
+          <t>File exists and is part of repo</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>internal/handler/admin_handler.go</t>
+          <t>tests/load/public-content-flow.k6.js</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Specified</t>
         </is>
       </c>
     </row>
@@ -1954,7 +1954,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>ROUTE-003</t>
+          <t>ROUTE-001</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -1964,7 +1964,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>GET /api/admin/users</t>
+          <t>GET /api/admin/export</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -1991,17 +1991,17 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>ROUTE-004</t>
+          <t>ROUTE-002</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>Admin</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>POST /api/ai/chat</t>
+          <t>GET /api/admin/stats</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -2011,7 +2011,7 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>internal/handler/admin_handler.go</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -2028,17 +2028,17 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>ROUTE-005</t>
+          <t>ROUTE-003</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>Admin</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>POST /api/analytics/events</t>
+          <t>GET /api/admin/users</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -2048,7 +2048,7 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>internal/handler/admin_handler.go</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -2065,7 +2065,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>ROUTE-006</t>
+          <t>ROUTE-004</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2075,7 +2075,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>POST /api/audit/client-error</t>
+          <t>POST /api/ai/chat</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -2102,17 +2102,17 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>ROUTE-007</t>
+          <t>ROUTE-005</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>POST /api/auth/avatar</t>
+          <t>POST /api/analytics/events</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -2139,7 +2139,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>ROUTE-008</t>
+          <t>ROUTE-006</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2149,7 +2149,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>POST /api/auth/login</t>
+          <t>POST /api/audit/client-error</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -2176,7 +2176,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>ROUTE-009</t>
+          <t>ROUTE-007</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2186,7 +2186,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>PUT /api/auth/mbti</t>
+          <t>POST /api/auth/avatar</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -2196,7 +2196,7 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>internal/handler/me_handler.go</t>
+          <t>cmd/server/main.go</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -2213,17 +2213,17 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>ROUTE-010</t>
+          <t>ROUTE-008</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>GET /api/auth/me</t>
+          <t>POST /api/auth/login</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -2250,17 +2250,17 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>ROUTE-011</t>
+          <t>ROUTE-009</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>JWT</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>POST /api/auth/register</t>
+          <t>PUT /api/auth/mbti</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -2270,7 +2270,7 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>internal/handler/me_handler.go</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -2287,7 +2287,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>ROUTE-012</t>
+          <t>ROUTE-010</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2297,7 +2297,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>GET /api/auth/saved</t>
+          <t>GET /api/auth/me</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -2307,7 +2307,7 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>internal/handler/me_handler.go</t>
+          <t>cmd/server/main.go</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -2324,17 +2324,17 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>ROUTE-013</t>
+          <t>ROUTE-011</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>DELETE /api/auth/saved/:slug</t>
+          <t>POST /api/auth/register</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -2344,7 +2344,7 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>internal/handler/me_handler.go</t>
+          <t>cmd/server/main.go</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -2361,7 +2361,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>ROUTE-014</t>
+          <t>ROUTE-012</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2371,7 +2371,7 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>PUT /api/auth/saved/:slug</t>
+          <t>GET /api/auth/saved</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -2398,17 +2398,17 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>ROUTE-015</t>
+          <t>ROUTE-013</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>JWT</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>GET /api/captcha</t>
+          <t>DELETE /api/auth/saved/:slug</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -2418,7 +2418,7 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>internal/handler/me_handler.go</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -2435,17 +2435,17 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>ROUTE-016</t>
+          <t>ROUTE-014</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>JWT</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>GET /api/health</t>
+          <t>PUT /api/auth/saved/:slug</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -2455,7 +2455,7 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>internal/handler/me_handler.go</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
@@ -2472,7 +2472,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>ROUTE-017</t>
+          <t>ROUTE-015</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -2482,7 +2482,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>GET /api/journeys</t>
+          <t>GET /api/captcha</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -2509,7 +2509,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>ROUTE-018</t>
+          <t>ROUTE-016</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -2519,7 +2519,7 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>GET /api/journeys/:slug</t>
+          <t>GET /api/health</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -2546,7 +2546,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>ROUTE-019</t>
+          <t>ROUTE-017</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -2556,7 +2556,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>GET /api/journeys/:slug/book</t>
+          <t>GET /api/journeys</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -2583,7 +2583,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>ROUTE-020</t>
+          <t>ROUTE-018</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -2593,7 +2593,7 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>GET /api/mbti</t>
+          <t>GET /api/journeys/:slug</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -2620,17 +2620,17 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>ROUTE-021</t>
+          <t>ROUTE-019</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>GET /api/orders</t>
+          <t>GET /api/journeys/:slug/book</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -2640,7 +2640,7 @@
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>internal/handler/order_handler.go</t>
+          <t>cmd/server/main.go</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
@@ -2657,17 +2657,17 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>ROUTE-022</t>
+          <t>ROUTE-020</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>POST /api/orders</t>
+          <t>GET /api/mbti</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -2677,7 +2677,7 @@
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>internal/handler/order_handler.go</t>
+          <t>cmd/server/main.go</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -2694,7 +2694,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>ROUTE-023</t>
+          <t>ROUTE-021</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -2704,7 +2704,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>GET /api/orders/:id</t>
+          <t>GET /api/orders</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -2731,7 +2731,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>ROUTE-024</t>
+          <t>ROUTE-022</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -2741,7 +2741,7 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>POST /api/orders/:id/pay</t>
+          <t>POST /api/orders</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -2768,7 +2768,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>ROUTE-025</t>
+          <t>ROUTE-023</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -2778,7 +2778,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>POST /api/payments/recharge</t>
+          <t>GET /api/orders/:id</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -2788,7 +2788,7 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>internal/handler/payment_handler.go</t>
+          <t>internal/handler/order_handler.go</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -2805,17 +2805,17 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>ROUTE-026</t>
+          <t>ROUTE-024</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>JWT</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>GET /api/payments/tiers</t>
+          <t>POST /api/orders/:id/pay</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -2825,7 +2825,7 @@
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>internal/handler/payment_handler.go</t>
+          <t>internal/handler/order_handler.go</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
@@ -2842,7 +2842,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>ROUTE-027</t>
+          <t>ROUTE-025</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -2852,7 +2852,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>GET /api/payments/transactions</t>
+          <t>POST /api/payments/recharge</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -2879,30 +2879,104 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
+          <t>ROUTE-026</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>GET /api/payments/tiers</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Route is registered</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>internal/handler/payment_handler.go</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Route</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>ROUTE-027</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>JWT</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>GET /api/payments/transactions</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Route is registered</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>internal/handler/payment_handler.go</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Route</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
           <t>ROUTE-028</t>
         </is>
       </c>
-      <c r="C70" t="inlineStr">
+      <c r="C72" t="inlineStr">
         <is>
           <t>Public</t>
         </is>
       </c>
-      <c r="D70" t="inlineStr">
+      <c r="D72" t="inlineStr">
         <is>
           <t>GET /api/tags</t>
         </is>
       </c>
-      <c r="E70" t="inlineStr">
+      <c r="E72" t="inlineStr">
         <is>
           <t>Route is registered</t>
         </is>
       </c>
-      <c r="F70" t="inlineStr">
+      <c r="F72" t="inlineStr">
         <is>
           <t>cmd/server/main.go</t>
         </is>
       </c>
-      <c r="G70" t="inlineStr">
+      <c r="G72" t="inlineStr">
         <is>
           <t>Implemented</t>
         </is>

</xml_diff>

<commit_message>
Compose game: draw your own entrance
A tray of torn paper slips in six groups (place, hour, season, how long
you stay, small ritual, what you take home). Tap, drag or use the
keyboard to put slips into the lantern-frame ticket; its sentence is
built from per-language templates, blanks stay dashed, and a kept ticket
gets a stamp and a read-only share link.

- internal/compose: embedded bilingual slips, validated at startup and
  in tests (vocabulary keys, entrance slugs, the content lint, now
  exported as content.Lint)
- compositions table and API: public slips and share view, signed-in
  list/keep/delete; keeping is idempotent on the client id
- #/compose and #/compose/:code; guests keep tickets on the device and
  they are replayed into the account on sign-in; entry card on Explore
- IT-API-COMPOSE-001..005, UT-COMPOSE-001..004, E2E-COMPOSE-001..008,
  axe scans of the game and share view in both themes
</commit_message>
<xml_diff>
--- a/app.xlsx
+++ b/app.xlsx
@@ -154,7 +154,7 @@
         </is>
       </c>
       <c r="B4">
-        <v>69</v>
+        <v>77</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -217,7 +217,7 @@
         </is>
       </c>
       <c r="E6">
-        <v>28</v>
+        <v>33</v>
       </c>
     </row>
     <row r="7">
@@ -242,7 +242,7 @@
         </is>
       </c>
       <c r="E7">
-        <v>36</v>
+        <v>39</v>
       </c>
     </row>
     <row r="8">
@@ -669,7 +669,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>content_test</t>
+          <t>compose_test</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -679,7 +679,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>internal/content/content_test.go</t>
+          <t>internal/compose/compose_test.go</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -706,7 +706,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>admin_handler_test</t>
+          <t>content_test</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -716,7 +716,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>internal/handler/admin_handler_test.go</t>
+          <t>internal/content/content_test.go</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -743,7 +743,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>auth_handler_test</t>
+          <t>admin_handler_test</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -753,7 +753,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>internal/handler/auth_handler_test.go</t>
+          <t>internal/handler/admin_handler_test.go</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -780,7 +780,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>journey_handler_test</t>
+          <t>auth_handler_test</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -790,7 +790,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>internal/handler/journey_handler_test.go</t>
+          <t>internal/handler/auth_handler_test.go</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -817,7 +817,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>me_handler_test</t>
+          <t>compose_handler_test</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -827,7 +827,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>internal/handler/me_handler_test.go</t>
+          <t>internal/handler/compose_handler_test.go</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -854,7 +854,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>order_handler_test</t>
+          <t>journey_handler_test</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -864,7 +864,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>internal/handler/order_handler_test.go</t>
+          <t>internal/handler/journey_handler_test.go</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -891,7 +891,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>payment_handler_test</t>
+          <t>me_handler_test</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -901,7 +901,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>internal/handler/payment_handler_test.go</t>
+          <t>internal/handler/me_handler_test.go</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -928,7 +928,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>cors_test</t>
+          <t>order_handler_test</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -938,7 +938,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>internal/middleware/cors_test.go</t>
+          <t>internal/handler/order_handler_test.go</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -965,7 +965,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>jwt_test</t>
+          <t>payment_handler_test</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -975,7 +975,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>internal/middleware/jwt_test.go</t>
+          <t>internal/handler/payment_handler_test.go</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1002,7 +1002,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>request_id_test</t>
+          <t>cors_test</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1012,7 +1012,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>internal/middleware/request_id_test.go</t>
+          <t>internal/middleware/cors_test.go</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1039,7 +1039,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>journey_repo_sqlite_test</t>
+          <t>jwt_test</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1049,7 +1049,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>internal/repository/journey_repo_sqlite_test.go</t>
+          <t>internal/middleware/jwt_test.go</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1076,7 +1076,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>order_repo_test</t>
+          <t>request_id_test</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1086,7 +1086,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>internal/repository/order_repo_test.go</t>
+          <t>internal/middleware/request_id_test.go</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1113,7 +1113,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>user_repo_test</t>
+          <t>journey_repo_sqlite_test</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1123,7 +1123,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>internal/repository/user_repo_test.go</t>
+          <t>internal/repository/journey_repo_sqlite_test.go</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1150,7 +1150,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>journey_service_test</t>
+          <t>order_repo_test</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1160,7 +1160,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>internal/service/journey_service_test.go</t>
+          <t>internal/repository/order_repo_test.go</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1187,7 +1187,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>locale_test</t>
+          <t>user_repo_test</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1197,7 +1197,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>internal/service/locale_test.go</t>
+          <t>internal/repository/user_repo_test.go</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1224,7 +1224,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>index_test</t>
+          <t>journey_service_test</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1234,7 +1234,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>internal/webapp/index_test.go</t>
+          <t>internal/service/journey_service_test.go</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1256,12 +1256,12 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Playwright E2E</t>
+          <t>Go unit/integration / Go 单元集成</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>a11y.spec</t>
+          <t>locale_test</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1271,7 +1271,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>e2e/tests/a11y.spec.js</t>
+          <t>internal/service/locale_test.go</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1293,12 +1293,12 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Playwright E2E</t>
+          <t>Go unit/integration / Go 单元集成</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>auth.spec</t>
+          <t>index_test</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>e2e/tests/auth.spec.js</t>
+          <t>internal/webapp/index_test.go</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1335,7 +1335,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>detail.spec</t>
+          <t>a11y.spec</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -1345,7 +1345,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>e2e/tests/detail.spec.js</t>
+          <t>e2e/tests/a11y.spec.js</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1372,7 +1372,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>explore.spec</t>
+          <t>auth.spec</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1382,7 +1382,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>e2e/tests/explore.spec.js</t>
+          <t>e2e/tests/auth.spec.js</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1409,7 +1409,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>home.spec</t>
+          <t>compose.spec</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1419,7 +1419,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>e2e/tests/home.spec.js</t>
+          <t>e2e/tests/compose.spec.js</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -1446,7 +1446,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>i18n.spec</t>
+          <t>detail.spec</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1456,7 +1456,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>e2e/tests/i18n.spec.js</t>
+          <t>e2e/tests/detail.spec.js</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -1483,7 +1483,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>mobile.spec</t>
+          <t>explore.spec</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -1493,7 +1493,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>e2e/tests/mobile.spec.js</t>
+          <t>e2e/tests/explore.spec.js</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -1520,7 +1520,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>orders.spec</t>
+          <t>home.spec</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1530,7 +1530,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>e2e/tests/orders.spec.js</t>
+          <t>e2e/tests/home.spec.js</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -1557,7 +1557,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>persona.spec</t>
+          <t>i18n.spec</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -1567,7 +1567,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>e2e/tests/persona.spec.js</t>
+          <t>e2e/tests/i18n.spec.js</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -1589,12 +1589,12 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Playwright support / E2E 支撑文件</t>
+          <t>Playwright E2E</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>helpers</t>
+          <t>mobile.spec</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -1604,7 +1604,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>e2e/tests/helpers.js</t>
+          <t>e2e/tests/mobile.spec.js</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -1626,12 +1626,12 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Go stress</t>
+          <t>Playwright E2E</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>stress_test</t>
+          <t>orders.spec</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -1641,7 +1641,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>tests/stress/stress_test.go</t>
+          <t>e2e/tests/orders.spec.js</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -1663,12 +1663,12 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>k6 load / k6 负载</t>
+          <t>Playwright E2E</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>admin-analytics-export.k6</t>
+          <t>persona.spec</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -1678,7 +1678,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>tests/load/admin-analytics-export.k6.js</t>
+          <t>e2e/tests/persona.spec.js</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -1700,12 +1700,12 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>k6 load / k6 负载</t>
+          <t>Playwright support / E2E 支撑文件</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>auth-register-login.k6</t>
+          <t>helpers</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -1715,7 +1715,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>tests/load/auth-register-login.k6.js</t>
+          <t>e2e/tests/helpers.js</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -1737,12 +1737,12 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>k6 load / k6 负载</t>
+          <t>Go stress</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>image-static-cache.k6</t>
+          <t>stress_test</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -1752,7 +1752,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>tests/load/image-static-cache.k6.js</t>
+          <t>tests/stress/stress_test.go</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -1779,7 +1779,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>order-payment-audit.k6</t>
+          <t>admin-analytics-export.k6</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -1789,7 +1789,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>tests/load/order-payment-audit.k6.js</t>
+          <t>tests/load/admin-analytics-export.k6.js</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -1816,7 +1816,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>pet-chat-analytics.k6</t>
+          <t>auth-register-login.k6</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -1826,7 +1826,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>tests/load/pet-chat-analytics.k6.js</t>
+          <t>tests/load/auth-register-login.k6.js</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -1853,7 +1853,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>public-content-flow.k6</t>
+          <t>image-static-cache.k6</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -1863,7 +1863,7 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>tests/load/public-content-flow.k6.js</t>
+          <t>tests/load/image-static-cache.k6.js</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -1875,111 +1875,111 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Route</t>
+          <t>Test</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>ROUTE-001</t>
+          <t>TEST-037</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Admin</t>
+          <t>k6 load / k6 负载</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>GET /api/admin/export</t>
+          <t>order-payment-audit.k6</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Route is registered</t>
+          <t>File exists and is part of repo</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>internal/handler/admin_handler.go</t>
+          <t>tests/load/order-payment-audit.k6.js</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Specified</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Route</t>
+          <t>Test</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>ROUTE-002</t>
+          <t>TEST-038</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Admin</t>
+          <t>k6 load / k6 负载</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>GET /api/admin/stats</t>
+          <t>pet-chat-analytics.k6</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Route is registered</t>
+          <t>File exists and is part of repo</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>internal/handler/admin_handler.go</t>
+          <t>tests/load/pet-chat-analytics.k6.js</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Specified</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Route</t>
+          <t>Test</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>ROUTE-003</t>
+          <t>TEST-039</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Admin</t>
+          <t>k6 load / k6 负载</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>GET /api/admin/users</t>
+          <t>public-content-flow.k6</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Route is registered</t>
+          <t>File exists and is part of repo</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>internal/handler/admin_handler.go</t>
+          <t>tests/load/public-content-flow.k6.js</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Specified</t>
         </is>
       </c>
     </row>
@@ -1991,17 +1991,17 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>ROUTE-004</t>
+          <t>ROUTE-001</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>Admin</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>POST /api/ai/chat</t>
+          <t>GET /api/admin/export</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -2011,7 +2011,7 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>internal/handler/admin_handler.go</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -2028,17 +2028,17 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>ROUTE-005</t>
+          <t>ROUTE-002</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>Admin</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>POST /api/analytics/events</t>
+          <t>GET /api/admin/stats</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -2048,7 +2048,7 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>internal/handler/admin_handler.go</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -2065,17 +2065,17 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>ROUTE-006</t>
+          <t>ROUTE-003</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>Admin</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>POST /api/audit/client-error</t>
+          <t>GET /api/admin/users</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -2085,7 +2085,7 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>internal/handler/admin_handler.go</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -2102,17 +2102,17 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>ROUTE-007</t>
+          <t>ROUTE-004</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>POST /api/auth/avatar</t>
+          <t>POST /api/ai/chat</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -2139,7 +2139,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>ROUTE-008</t>
+          <t>ROUTE-005</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2149,7 +2149,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>POST /api/auth/login</t>
+          <t>POST /api/analytics/events</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -2176,17 +2176,17 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>ROUTE-009</t>
+          <t>ROUTE-006</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>PUT /api/auth/mbti</t>
+          <t>POST /api/audit/client-error</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -2196,7 +2196,7 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>internal/handler/me_handler.go</t>
+          <t>cmd/server/main.go</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -2213,7 +2213,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>ROUTE-010</t>
+          <t>ROUTE-007</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2223,7 +2223,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>GET /api/auth/me</t>
+          <t>POST /api/auth/avatar</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -2250,17 +2250,17 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>ROUTE-011</t>
+          <t>ROUTE-008</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>JWT</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>POST /api/auth/register</t>
+          <t>GET /api/auth/compositions</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -2270,7 +2270,7 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>internal/handler/compose_handler.go</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -2287,7 +2287,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>ROUTE-012</t>
+          <t>ROUTE-009</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2297,7 +2297,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>GET /api/auth/saved</t>
+          <t>POST /api/auth/compositions</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -2307,7 +2307,7 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>internal/handler/me_handler.go</t>
+          <t>internal/handler/compose_handler.go</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -2324,7 +2324,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>ROUTE-013</t>
+          <t>ROUTE-010</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2334,7 +2334,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>DELETE /api/auth/saved/:slug</t>
+          <t>DELETE /api/auth/compositions/:id</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -2344,7 +2344,7 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>internal/handler/me_handler.go</t>
+          <t>internal/handler/compose_handler.go</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -2361,17 +2361,17 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>ROUTE-014</t>
+          <t>ROUTE-011</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>PUT /api/auth/saved/:slug</t>
+          <t>POST /api/auth/login</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -2381,7 +2381,7 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>internal/handler/me_handler.go</t>
+          <t>cmd/server/main.go</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -2398,17 +2398,17 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>ROUTE-015</t>
+          <t>ROUTE-012</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>JWT</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>GET /api/captcha</t>
+          <t>PUT /api/auth/mbti</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -2418,7 +2418,7 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>internal/handler/me_handler.go</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -2435,17 +2435,17 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>ROUTE-016</t>
+          <t>ROUTE-013</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>JWT</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>GET /api/health</t>
+          <t>GET /api/auth/me</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -2472,7 +2472,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>ROUTE-017</t>
+          <t>ROUTE-014</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -2482,7 +2482,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>GET /api/journeys</t>
+          <t>POST /api/auth/register</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -2509,17 +2509,17 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>ROUTE-018</t>
+          <t>ROUTE-015</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>JWT</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>GET /api/journeys/:slug</t>
+          <t>GET /api/auth/saved</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -2529,7 +2529,7 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>internal/handler/me_handler.go</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -2546,17 +2546,17 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>ROUTE-019</t>
+          <t>ROUTE-016</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>JWT</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>GET /api/journeys/:slug/book</t>
+          <t>DELETE /api/auth/saved/:slug</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -2566,7 +2566,7 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>internal/handler/me_handler.go</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -2583,17 +2583,17 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>ROUTE-020</t>
+          <t>ROUTE-017</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>JWT</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>GET /api/mbti</t>
+          <t>PUT /api/auth/saved/:slug</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -2603,7 +2603,7 @@
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>internal/handler/me_handler.go</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
@@ -2620,17 +2620,17 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>ROUTE-021</t>
+          <t>ROUTE-018</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>GET /api/orders</t>
+          <t>GET /api/captcha</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -2640,7 +2640,7 @@
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>internal/handler/order_handler.go</t>
+          <t>cmd/server/main.go</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
@@ -2657,17 +2657,17 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>ROUTE-022</t>
+          <t>ROUTE-019</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>POST /api/orders</t>
+          <t>GET /api/compose/fragments</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -2677,7 +2677,7 @@
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>internal/handler/order_handler.go</t>
+          <t>internal/handler/compose_handler.go</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -2694,17 +2694,17 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>ROUTE-023</t>
+          <t>ROUTE-020</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>GET /api/orders/:id</t>
+          <t>GET /api/compositions/:code</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -2714,7 +2714,7 @@
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>internal/handler/order_handler.go</t>
+          <t>internal/handler/compose_handler.go</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
@@ -2731,17 +2731,17 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>ROUTE-024</t>
+          <t>ROUTE-021</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>POST /api/orders/:id/pay</t>
+          <t>GET /api/health</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -2751,7 +2751,7 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>internal/handler/order_handler.go</t>
+          <t>cmd/server/main.go</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
@@ -2768,17 +2768,17 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>ROUTE-025</t>
+          <t>ROUTE-022</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>POST /api/payments/recharge</t>
+          <t>GET /api/journeys</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -2788,7 +2788,7 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>internal/handler/payment_handler.go</t>
+          <t>cmd/server/main.go</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -2805,7 +2805,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>ROUTE-026</t>
+          <t>ROUTE-023</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -2815,7 +2815,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>GET /api/payments/tiers</t>
+          <t>GET /api/journeys/:slug</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -2825,7 +2825,7 @@
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>internal/handler/payment_handler.go</t>
+          <t>cmd/server/main.go</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
@@ -2842,17 +2842,17 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>ROUTE-027</t>
+          <t>ROUTE-024</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>GET /api/payments/transactions</t>
+          <t>GET /api/journeys/:slug/book</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -2862,7 +2862,7 @@
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>internal/handler/payment_handler.go</t>
+          <t>cmd/server/main.go</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
@@ -2879,30 +2879,326 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
+          <t>ROUTE-025</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>GET /api/mbti</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Route is registered</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>cmd/server/main.go</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Route</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>ROUTE-026</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>JWT</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>GET /api/orders</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Route is registered</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>internal/handler/order_handler.go</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Route</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>ROUTE-027</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>JWT</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>POST /api/orders</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Route is registered</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>internal/handler/order_handler.go</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Route</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
           <t>ROUTE-028</t>
         </is>
       </c>
-      <c r="C70" t="inlineStr">
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>JWT</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>GET /api/orders/:id</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Route is registered</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>internal/handler/order_handler.go</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Route</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>ROUTE-029</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>JWT</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>POST /api/orders/:id/pay</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Route is registered</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>internal/handler/order_handler.go</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Route</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>ROUTE-030</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>JWT</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>POST /api/payments/recharge</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>Route is registered</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>internal/handler/payment_handler.go</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Route</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>ROUTE-031</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
         <is>
           <t>Public</t>
         </is>
       </c>
-      <c r="D70" t="inlineStr">
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>GET /api/payments/tiers</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>Route is registered</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>internal/handler/payment_handler.go</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Route</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>ROUTE-032</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>JWT</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>GET /api/payments/transactions</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>Route is registered</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>internal/handler/payment_handler.go</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Route</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>ROUTE-033</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
         <is>
           <t>GET /api/tags</t>
         </is>
       </c>
-      <c r="E70" t="inlineStr">
+      <c r="E78" t="inlineStr">
         <is>
           <t>Route is registered</t>
         </is>
       </c>
-      <c r="F70" t="inlineStr">
+      <c r="F78" t="inlineStr">
         <is>
           <t>cmd/server/main.go</t>
         </is>
       </c>
-      <c r="G70" t="inlineStr">
+      <c r="G78" t="inlineStr">
         <is>
           <t>Implemented</t>
         </is>

</xml_diff>

<commit_message>
feat(ai): DeepSeek guide with a rule-based fallback
With DEEPSEEK_API_KEY set, the guide answers free-text questions through
DeepSeek's chat API, grounded in the journey catalogue in the reader's
language. Only catalogue journeys can be recommended (validated by slug, at most
three); the traveller's type steers the choice but is never named back.

Every failure falls back to the rule-based guide: no key, an 8s timeout, an
upstream error, an unusable reply, or all four concurrent slots busy. Replies
are capped at 320 tokens and messages at 1000 characters. The key and message or
reply bodies are never logged, only status codes. Responses carry
source=deepseek|mock; the widget shows typing dots and uses its own zh/en
rules when the model doesn't answer.
</commit_message>
<xml_diff>
--- a/app.xlsx
+++ b/app.xlsx
@@ -154,7 +154,7 @@
         </is>
       </c>
       <c r="B4">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -242,7 +242,7 @@
         </is>
       </c>
       <c r="E7">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="8">
@@ -558,7 +558,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>mock_ai_test</t>
+          <t>deepseek_test</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -568,7 +568,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>internal/ai/mock_ai_test.go</t>
+          <t>internal/ai/deepseek_test.go</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -595,7 +595,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>recommend_engine_test</t>
+          <t>mock_ai_test</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -605,7 +605,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>internal/ai/recommend_engine_test.go</t>
+          <t>internal/ai/mock_ai_test.go</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -632,7 +632,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>buffer_test</t>
+          <t>recommend_engine_test</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -642,7 +642,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>internal/analytics/buffer_test.go</t>
+          <t>internal/ai/recommend_engine_test.go</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -669,7 +669,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>content_test</t>
+          <t>buffer_test</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -679,7 +679,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>internal/content/content_test.go</t>
+          <t>internal/analytics/buffer_test.go</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -706,7 +706,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>admin_handler_test</t>
+          <t>content_test</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -716,7 +716,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>internal/handler/admin_handler_test.go</t>
+          <t>internal/content/content_test.go</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -743,7 +743,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>auth_handler_test</t>
+          <t>admin_handler_test</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -753,7 +753,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>internal/handler/auth_handler_test.go</t>
+          <t>internal/handler/admin_handler_test.go</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -780,7 +780,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>journey_handler_test</t>
+          <t>auth_handler_test</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -790,7 +790,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>internal/handler/journey_handler_test.go</t>
+          <t>internal/handler/auth_handler_test.go</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -817,7 +817,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>me_handler_test</t>
+          <t>journey_handler_test</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -827,7 +827,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>internal/handler/me_handler_test.go</t>
+          <t>internal/handler/journey_handler_test.go</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -854,7 +854,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>order_handler_test</t>
+          <t>me_handler_test</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -864,7 +864,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>internal/handler/order_handler_test.go</t>
+          <t>internal/handler/me_handler_test.go</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -891,7 +891,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>payment_handler_test</t>
+          <t>order_handler_test</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -901,7 +901,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>internal/handler/payment_handler_test.go</t>
+          <t>internal/handler/order_handler_test.go</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -928,7 +928,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>cors_test</t>
+          <t>payment_handler_test</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -938,7 +938,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>internal/middleware/cors_test.go</t>
+          <t>internal/handler/payment_handler_test.go</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -965,7 +965,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>jwt_test</t>
+          <t>cors_test</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -975,7 +975,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>internal/middleware/jwt_test.go</t>
+          <t>internal/middleware/cors_test.go</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1002,7 +1002,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>request_id_test</t>
+          <t>jwt_test</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1012,7 +1012,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>internal/middleware/request_id_test.go</t>
+          <t>internal/middleware/jwt_test.go</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1039,7 +1039,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>journey_repo_sqlite_test</t>
+          <t>request_id_test</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1049,7 +1049,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>internal/repository/journey_repo_sqlite_test.go</t>
+          <t>internal/middleware/request_id_test.go</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1076,7 +1076,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>migrate_test</t>
+          <t>journey_repo_sqlite_test</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1086,7 +1086,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>internal/repository/migrate_test.go</t>
+          <t>internal/repository/journey_repo_sqlite_test.go</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1113,7 +1113,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>order_repo_test</t>
+          <t>migrate_test</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1123,7 +1123,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>internal/repository/order_repo_test.go</t>
+          <t>internal/repository/migrate_test.go</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1150,7 +1150,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>user_repo_test</t>
+          <t>order_repo_test</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1160,7 +1160,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>internal/repository/user_repo_test.go</t>
+          <t>internal/repository/order_repo_test.go</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1187,7 +1187,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>journey_service_test</t>
+          <t>user_repo_test</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1197,7 +1197,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>internal/service/journey_service_test.go</t>
+          <t>internal/repository/user_repo_test.go</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1224,7 +1224,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>locale_test</t>
+          <t>journey_service_test</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1234,7 +1234,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>internal/service/locale_test.go</t>
+          <t>internal/service/journey_service_test.go</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1261,7 +1261,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>index_test</t>
+          <t>locale_test</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1271,7 +1271,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>internal/webapp/index_test.go</t>
+          <t>internal/service/locale_test.go</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1293,12 +1293,12 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Playwright E2E</t>
+          <t>Go unit/integration / Go 单元集成</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>a11y.spec</t>
+          <t>index_test</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>e2e/tests/a11y.spec.js</t>
+          <t>internal/webapp/index_test.go</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1335,7 +1335,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>auth.spec</t>
+          <t>a11y.spec</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -1345,7 +1345,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>e2e/tests/auth.spec.js</t>
+          <t>e2e/tests/a11y.spec.js</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1372,7 +1372,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>detail.spec</t>
+          <t>auth.spec</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1382,7 +1382,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>e2e/tests/detail.spec.js</t>
+          <t>e2e/tests/auth.spec.js</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1409,7 +1409,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>explore.spec</t>
+          <t>detail.spec</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1419,7 +1419,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>e2e/tests/explore.spec.js</t>
+          <t>e2e/tests/detail.spec.js</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -1446,7 +1446,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>home.spec</t>
+          <t>explore.spec</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1456,7 +1456,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>e2e/tests/home.spec.js</t>
+          <t>e2e/tests/explore.spec.js</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -1483,7 +1483,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>i18n.spec</t>
+          <t>home.spec</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -1493,7 +1493,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>e2e/tests/i18n.spec.js</t>
+          <t>e2e/tests/home.spec.js</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -1520,7 +1520,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>mobile.spec</t>
+          <t>i18n.spec</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1530,7 +1530,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>e2e/tests/mobile.spec.js</t>
+          <t>e2e/tests/i18n.spec.js</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -1557,7 +1557,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>orders.spec</t>
+          <t>mobile.spec</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -1567,7 +1567,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>e2e/tests/orders.spec.js</t>
+          <t>e2e/tests/mobile.spec.js</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -1594,7 +1594,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>persona.spec</t>
+          <t>orders.spec</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -1604,7 +1604,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>e2e/tests/persona.spec.js</t>
+          <t>e2e/tests/orders.spec.js</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -1631,7 +1631,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>space.spec</t>
+          <t>persona.spec</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -1641,7 +1641,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>e2e/tests/space.spec.js</t>
+          <t>e2e/tests/persona.spec.js</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -1663,12 +1663,12 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Playwright support / E2E 支撑文件</t>
+          <t>Playwright E2E</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>helpers</t>
+          <t>space.spec</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -1678,7 +1678,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>e2e/tests/helpers.js</t>
+          <t>e2e/tests/space.spec.js</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -1700,12 +1700,12 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Go stress</t>
+          <t>Playwright support / E2E 支撑文件</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>stress_test</t>
+          <t>helpers</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -1715,7 +1715,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>tests/stress/stress_test.go</t>
+          <t>e2e/tests/helpers.js</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -1737,12 +1737,12 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>k6 load / k6 负载</t>
+          <t>Go stress</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>admin-analytics-export.k6</t>
+          <t>stress_test</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -1752,7 +1752,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>tests/load/admin-analytics-export.k6.js</t>
+          <t>tests/stress/stress_test.go</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -1779,7 +1779,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>auth-register-login.k6</t>
+          <t>admin-analytics-export.k6</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -1789,7 +1789,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>tests/load/auth-register-login.k6.js</t>
+          <t>tests/load/admin-analytics-export.k6.js</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -1816,7 +1816,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>image-static-cache.k6</t>
+          <t>auth-register-login.k6</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -1826,7 +1826,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>tests/load/image-static-cache.k6.js</t>
+          <t>tests/load/auth-register-login.k6.js</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -1853,7 +1853,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>order-payment-audit.k6</t>
+          <t>image-static-cache.k6</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -1863,7 +1863,7 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>tests/load/order-payment-audit.k6.js</t>
+          <t>tests/load/image-static-cache.k6.js</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -1890,7 +1890,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>pet-chat-analytics.k6</t>
+          <t>order-payment-audit.k6</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -1900,7 +1900,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>tests/load/pet-chat-analytics.k6.js</t>
+          <t>tests/load/order-payment-audit.k6.js</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -1927,7 +1927,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>public-content-flow.k6</t>
+          <t>pet-chat-analytics.k6</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -1937,7 +1937,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>tests/load/public-content-flow.k6.js</t>
+          <t>tests/load/pet-chat-analytics.k6.js</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -1949,37 +1949,37 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Route</t>
+          <t>Test</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>ROUTE-001</t>
+          <t>TEST-039</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Admin</t>
+          <t>k6 load / k6 负载</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>GET /api/admin/export</t>
+          <t>public-content-flow.k6</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Route is registered</t>
+          <t>File exists and is part of repo</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>internal/handler/admin_handler.go</t>
+          <t>tests/load/public-content-flow.k6.js</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Specified</t>
         </is>
       </c>
     </row>
@@ -1991,7 +1991,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>ROUTE-002</t>
+          <t>ROUTE-001</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2001,7 +2001,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>GET /api/admin/stats</t>
+          <t>GET /api/admin/export</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -2028,7 +2028,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>ROUTE-003</t>
+          <t>ROUTE-002</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2038,7 +2038,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>GET /api/admin/users</t>
+          <t>GET /api/admin/stats</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -2065,17 +2065,17 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>ROUTE-004</t>
+          <t>ROUTE-003</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>Admin</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>POST /api/ai/chat</t>
+          <t>GET /api/admin/users</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -2085,7 +2085,7 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>internal/handler/admin_handler.go</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -2102,7 +2102,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>ROUTE-005</t>
+          <t>ROUTE-004</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2112,7 +2112,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>POST /api/analytics/events</t>
+          <t>POST /api/ai/chat</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -2139,7 +2139,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>ROUTE-006</t>
+          <t>ROUTE-005</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2149,7 +2149,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>POST /api/audit/client-error</t>
+          <t>POST /api/analytics/events</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -2176,17 +2176,17 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>ROUTE-007</t>
+          <t>ROUTE-006</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>POST /api/auth/avatar</t>
+          <t>POST /api/audit/client-error</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -2213,17 +2213,17 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>ROUTE-008</t>
+          <t>ROUTE-007</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>JWT</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>POST /api/auth/login</t>
+          <t>POST /api/auth/avatar</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -2250,17 +2250,17 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>ROUTE-009</t>
+          <t>ROUTE-008</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>PUT /api/auth/mbti</t>
+          <t>POST /api/auth/login</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -2270,7 +2270,7 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>internal/handler/me_handler.go</t>
+          <t>cmd/server/main.go</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -2287,7 +2287,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>ROUTE-010</t>
+          <t>ROUTE-009</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2297,7 +2297,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>GET /api/auth/me</t>
+          <t>PUT /api/auth/mbti</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -2307,7 +2307,7 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>internal/handler/me_handler.go</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -2324,17 +2324,17 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>ROUTE-011</t>
+          <t>ROUTE-010</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>JWT</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>POST /api/auth/register</t>
+          <t>GET /api/auth/me</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -2361,17 +2361,17 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>ROUTE-012</t>
+          <t>ROUTE-011</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>GET /api/auth/saved</t>
+          <t>POST /api/auth/register</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -2381,7 +2381,7 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>internal/handler/me_handler.go</t>
+          <t>cmd/server/main.go</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -2398,7 +2398,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>ROUTE-013</t>
+          <t>ROUTE-012</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -2408,7 +2408,7 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>DELETE /api/auth/saved/:slug</t>
+          <t>GET /api/auth/saved</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -2435,7 +2435,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>ROUTE-014</t>
+          <t>ROUTE-013</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -2445,7 +2445,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>PUT /api/auth/saved/:slug</t>
+          <t>DELETE /api/auth/saved/:slug</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -2472,17 +2472,17 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>ROUTE-015</t>
+          <t>ROUTE-014</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>JWT</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>GET /api/captcha</t>
+          <t>PUT /api/auth/saved/:slug</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -2492,7 +2492,7 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>internal/handler/me_handler.go</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
@@ -2509,7 +2509,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>ROUTE-016</t>
+          <t>ROUTE-015</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -2519,7 +2519,7 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>GET /api/health</t>
+          <t>GET /api/captcha</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -2546,7 +2546,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>ROUTE-017</t>
+          <t>ROUTE-016</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -2556,7 +2556,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>GET /api/journeys</t>
+          <t>GET /api/health</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -2583,7 +2583,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>ROUTE-018</t>
+          <t>ROUTE-017</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -2593,7 +2593,7 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>GET /api/journeys/:slug</t>
+          <t>GET /api/journeys</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -2620,7 +2620,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>ROUTE-019</t>
+          <t>ROUTE-018</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -2630,7 +2630,7 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>GET /api/journeys/:slug/book</t>
+          <t>GET /api/journeys/:slug</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -2657,7 +2657,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>ROUTE-020</t>
+          <t>ROUTE-019</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -2667,7 +2667,7 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>GET /api/mbti</t>
+          <t>GET /api/journeys/:slug/book</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -2694,17 +2694,17 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>ROUTE-021</t>
+          <t>ROUTE-020</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>GET /api/orders</t>
+          <t>GET /api/mbti</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -2714,7 +2714,7 @@
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>internal/handler/order_handler.go</t>
+          <t>cmd/server/main.go</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
@@ -2731,7 +2731,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>ROUTE-022</t>
+          <t>ROUTE-021</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -2741,7 +2741,7 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>POST /api/orders</t>
+          <t>GET /api/orders</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -2768,7 +2768,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>ROUTE-023</t>
+          <t>ROUTE-022</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -2778,7 +2778,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>GET /api/orders/:id</t>
+          <t>POST /api/orders</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -2805,7 +2805,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>ROUTE-024</t>
+          <t>ROUTE-023</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -2815,7 +2815,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>POST /api/orders/:id/pay</t>
+          <t>GET /api/orders/:id</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -2842,7 +2842,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>ROUTE-025</t>
+          <t>ROUTE-024</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -2852,7 +2852,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>POST /api/payments/recharge</t>
+          <t>POST /api/orders/:id/pay</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -2862,7 +2862,7 @@
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>internal/handler/payment_handler.go</t>
+          <t>internal/handler/order_handler.go</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
@@ -2879,17 +2879,17 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>ROUTE-026</t>
+          <t>ROUTE-025</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>JWT</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>GET /api/payments/tiers</t>
+          <t>POST /api/payments/recharge</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -2916,17 +2916,17 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>ROUTE-027</t>
+          <t>ROUTE-026</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>GET /api/payments/transactions</t>
+          <t>GET /api/payments/tiers</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -2953,30 +2953,67 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
+          <t>ROUTE-027</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>JWT</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>GET /api/payments/transactions</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Route is registered</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>internal/handler/payment_handler.go</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Route</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
           <t>ROUTE-028</t>
         </is>
       </c>
-      <c r="C72" t="inlineStr">
+      <c r="C73" t="inlineStr">
         <is>
           <t>Public</t>
         </is>
       </c>
-      <c r="D72" t="inlineStr">
+      <c r="D73" t="inlineStr">
         <is>
           <t>GET /api/tags</t>
         </is>
       </c>
-      <c r="E72" t="inlineStr">
+      <c r="E73" t="inlineStr">
         <is>
           <t>Route is registered</t>
         </is>
       </c>
-      <c r="F72" t="inlineStr">
+      <c r="F73" t="inlineStr">
         <is>
           <t>cmd/server/main.go</t>
         </is>
       </c>
-      <c r="G72" t="inlineStr">
+      <c r="G73" t="inlineStr">
         <is>
           <t>Implemented</t>
         </is>

</xml_diff>

<commit_message>
test: scenes, share links and reduced motion; axe on three journey scenes
</commit_message>
<xml_diff>
--- a/app.xlsx
+++ b/app.xlsx
@@ -154,7 +154,7 @@
         </is>
       </c>
       <c r="B4">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -242,7 +242,7 @@
         </is>
       </c>
       <c r="E7">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="8">
@@ -1330,12 +1330,12 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Playwright E2E</t>
+          <t>Go unit/integration / Go 单元集成</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>a11y.spec</t>
+          <t>share_test</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -1345,7 +1345,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>e2e/tests/a11y.spec.js</t>
+          <t>internal/webapp/share_test.go</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1372,7 +1372,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>auth.spec</t>
+          <t>a11y.spec</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1382,7 +1382,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>e2e/tests/auth.spec.js</t>
+          <t>e2e/tests/a11y.spec.js</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1409,7 +1409,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>detail.spec</t>
+          <t>auth.spec</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1419,7 +1419,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>e2e/tests/detail.spec.js</t>
+          <t>e2e/tests/auth.spec.js</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -1446,7 +1446,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>explore.spec</t>
+          <t>detail.spec</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1456,7 +1456,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>e2e/tests/explore.spec.js</t>
+          <t>e2e/tests/detail.spec.js</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -1483,7 +1483,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>home.spec</t>
+          <t>explore.spec</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -1493,7 +1493,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>e2e/tests/home.spec.js</t>
+          <t>e2e/tests/explore.spec.js</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -1520,7 +1520,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>i18n.spec</t>
+          <t>home.spec</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1530,7 +1530,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>e2e/tests/i18n.spec.js</t>
+          <t>e2e/tests/home.spec.js</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -1557,7 +1557,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>mobile.spec</t>
+          <t>i18n.spec</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -1567,7 +1567,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>e2e/tests/mobile.spec.js</t>
+          <t>e2e/tests/i18n.spec.js</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -1594,7 +1594,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>orders.spec</t>
+          <t>mobile.spec</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -1604,7 +1604,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>e2e/tests/orders.spec.js</t>
+          <t>e2e/tests/mobile.spec.js</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -1631,7 +1631,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>persona.spec</t>
+          <t>orders.spec</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -1641,7 +1641,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>e2e/tests/persona.spec.js</t>
+          <t>e2e/tests/orders.spec.js</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -1668,7 +1668,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>space.spec</t>
+          <t>persona.spec</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -1678,7 +1678,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>e2e/tests/space.spec.js</t>
+          <t>e2e/tests/persona.spec.js</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -1700,12 +1700,12 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Playwright support / E2E 支撑文件</t>
+          <t>Playwright E2E</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>helpers</t>
+          <t>space.spec</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -1715,7 +1715,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>e2e/tests/helpers.js</t>
+          <t>e2e/tests/space.spec.js</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -1737,12 +1737,12 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Go stress</t>
+          <t>Playwright support / E2E 支撑文件</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>stress_test</t>
+          <t>helpers</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -1752,7 +1752,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>tests/stress/stress_test.go</t>
+          <t>e2e/tests/helpers.js</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -1774,12 +1774,12 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>k6 load / k6 负载</t>
+          <t>Go stress</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>admin-analytics-export.k6</t>
+          <t>stress_test</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -1789,7 +1789,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>tests/load/admin-analytics-export.k6.js</t>
+          <t>tests/stress/stress_test.go</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -1816,7 +1816,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>auth-register-login.k6</t>
+          <t>admin-analytics-export.k6</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -1826,7 +1826,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>tests/load/auth-register-login.k6.js</t>
+          <t>tests/load/admin-analytics-export.k6.js</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -1853,7 +1853,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>image-static-cache.k6</t>
+          <t>auth-register-login.k6</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -1863,7 +1863,7 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>tests/load/image-static-cache.k6.js</t>
+          <t>tests/load/auth-register-login.k6.js</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -1890,7 +1890,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>order-payment-audit.k6</t>
+          <t>image-static-cache.k6</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -1900,7 +1900,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>tests/load/order-payment-audit.k6.js</t>
+          <t>tests/load/image-static-cache.k6.js</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -1927,7 +1927,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>pet-chat-analytics.k6</t>
+          <t>order-payment-audit.k6</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -1937,7 +1937,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>tests/load/pet-chat-analytics.k6.js</t>
+          <t>tests/load/order-payment-audit.k6.js</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -1964,7 +1964,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>public-content-flow.k6</t>
+          <t>pet-chat-analytics.k6</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -1974,7 +1974,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>tests/load/public-content-flow.k6.js</t>
+          <t>tests/load/pet-chat-analytics.k6.js</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -1986,37 +1986,37 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Route</t>
+          <t>Test</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>ROUTE-001</t>
+          <t>TEST-040</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Admin</t>
+          <t>k6 load / k6 负载</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>GET /api/admin/export</t>
+          <t>public-content-flow.k6</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Route is registered</t>
+          <t>File exists and is part of repo</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>internal/handler/admin_handler.go</t>
+          <t>tests/load/public-content-flow.k6.js</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Specified</t>
         </is>
       </c>
     </row>
@@ -2028,7 +2028,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>ROUTE-002</t>
+          <t>ROUTE-001</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2038,7 +2038,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>GET /api/admin/stats</t>
+          <t>GET /api/admin/export</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -2065,7 +2065,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>ROUTE-003</t>
+          <t>ROUTE-002</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2075,7 +2075,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>GET /api/admin/users</t>
+          <t>GET /api/admin/stats</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -2102,17 +2102,17 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>ROUTE-004</t>
+          <t>ROUTE-003</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>Admin</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>POST /api/ai/chat</t>
+          <t>GET /api/admin/users</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -2122,7 +2122,7 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>internal/handler/admin_handler.go</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -2139,7 +2139,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>ROUTE-005</t>
+          <t>ROUTE-004</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2149,7 +2149,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>POST /api/analytics/events</t>
+          <t>POST /api/ai/chat</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -2176,7 +2176,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>ROUTE-006</t>
+          <t>ROUTE-005</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2186,7 +2186,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>POST /api/audit/client-error</t>
+          <t>POST /api/analytics/events</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -2213,17 +2213,17 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>ROUTE-007</t>
+          <t>ROUTE-006</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>POST /api/auth/avatar</t>
+          <t>POST /api/audit/client-error</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -2250,17 +2250,17 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>ROUTE-008</t>
+          <t>ROUTE-007</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>JWT</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>POST /api/auth/login</t>
+          <t>POST /api/auth/avatar</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -2287,17 +2287,17 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>ROUTE-009</t>
+          <t>ROUTE-008</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>PUT /api/auth/mbti</t>
+          <t>POST /api/auth/login</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -2307,7 +2307,7 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>internal/handler/me_handler.go</t>
+          <t>cmd/server/main.go</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -2324,7 +2324,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>ROUTE-010</t>
+          <t>ROUTE-009</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2334,7 +2334,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>GET /api/auth/me</t>
+          <t>PUT /api/auth/mbti</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -2344,7 +2344,7 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>internal/handler/me_handler.go</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -2361,17 +2361,17 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>ROUTE-011</t>
+          <t>ROUTE-010</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>JWT</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>POST /api/auth/register</t>
+          <t>GET /api/auth/me</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -2398,17 +2398,17 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>ROUTE-012</t>
+          <t>ROUTE-011</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>GET /api/auth/saved</t>
+          <t>POST /api/auth/register</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -2418,7 +2418,7 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>internal/handler/me_handler.go</t>
+          <t>cmd/server/main.go</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -2435,7 +2435,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>ROUTE-013</t>
+          <t>ROUTE-012</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -2445,7 +2445,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>DELETE /api/auth/saved/:slug</t>
+          <t>GET /api/auth/saved</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -2472,7 +2472,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>ROUTE-014</t>
+          <t>ROUTE-013</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -2482,7 +2482,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>PUT /api/auth/saved/:slug</t>
+          <t>DELETE /api/auth/saved/:slug</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -2509,17 +2509,17 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>ROUTE-015</t>
+          <t>ROUTE-014</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>JWT</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>GET /api/captcha</t>
+          <t>PUT /api/auth/saved/:slug</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -2529,7 +2529,7 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>internal/handler/me_handler.go</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -2546,7 +2546,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>ROUTE-016</t>
+          <t>ROUTE-015</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -2556,7 +2556,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>GET /api/health</t>
+          <t>GET /api/captcha</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -2583,7 +2583,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>ROUTE-017</t>
+          <t>ROUTE-016</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -2593,7 +2593,7 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>GET /api/journeys</t>
+          <t>GET /api/health</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -2620,7 +2620,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>ROUTE-018</t>
+          <t>ROUTE-017</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -2630,7 +2630,7 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>GET /api/journeys/:slug</t>
+          <t>GET /api/journeys</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -2657,7 +2657,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>ROUTE-019</t>
+          <t>ROUTE-018</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -2667,7 +2667,7 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>GET /api/journeys/:slug/book</t>
+          <t>GET /api/journeys/:slug</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -2694,7 +2694,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>ROUTE-020</t>
+          <t>ROUTE-019</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -2704,7 +2704,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>GET /api/mbti</t>
+          <t>GET /api/journeys/:slug/book</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -2731,17 +2731,17 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>ROUTE-021</t>
+          <t>ROUTE-020</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>GET /api/orders</t>
+          <t>GET /api/mbti</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -2751,7 +2751,7 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>internal/handler/order_handler.go</t>
+          <t>cmd/server/main.go</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
@@ -2768,7 +2768,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>ROUTE-022</t>
+          <t>ROUTE-021</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -2778,7 +2778,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>POST /api/orders</t>
+          <t>GET /api/orders</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -2805,7 +2805,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>ROUTE-023</t>
+          <t>ROUTE-022</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -2815,7 +2815,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>GET /api/orders/:id</t>
+          <t>POST /api/orders</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -2842,7 +2842,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>ROUTE-024</t>
+          <t>ROUTE-023</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -2852,7 +2852,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>POST /api/orders/:id/pay</t>
+          <t>GET /api/orders/:id</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -2879,7 +2879,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>ROUTE-025</t>
+          <t>ROUTE-024</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -2889,7 +2889,7 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>POST /api/payments/recharge</t>
+          <t>POST /api/orders/:id/pay</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -2899,7 +2899,7 @@
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>internal/handler/payment_handler.go</t>
+          <t>internal/handler/order_handler.go</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
@@ -2916,17 +2916,17 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>ROUTE-026</t>
+          <t>ROUTE-025</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>JWT</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>GET /api/payments/tiers</t>
+          <t>POST /api/payments/recharge</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -2953,17 +2953,17 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>ROUTE-027</t>
+          <t>ROUTE-026</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>GET /api/payments/transactions</t>
+          <t>GET /api/payments/tiers</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
@@ -2990,30 +2990,67 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
+          <t>ROUTE-027</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>JWT</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>GET /api/payments/transactions</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Route is registered</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>internal/handler/payment_handler.go</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Route</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
           <t>ROUTE-028</t>
         </is>
       </c>
-      <c r="C73" t="inlineStr">
+      <c r="C74" t="inlineStr">
         <is>
           <t>Public</t>
         </is>
       </c>
-      <c r="D73" t="inlineStr">
+      <c r="D74" t="inlineStr">
         <is>
           <t>GET /api/tags</t>
         </is>
       </c>
-      <c r="E73" t="inlineStr">
+      <c r="E74" t="inlineStr">
         <is>
           <t>Route is registered</t>
         </is>
       </c>
-      <c r="F73" t="inlineStr">
+      <c r="F74" t="inlineStr">
         <is>
           <t>cmd/server/main.go</t>
         </is>
       </c>
-      <c r="G73" t="inlineStr">
+      <c r="G74" t="inlineStr">
         <is>
           <t>Implemented</t>
         </is>

</xml_diff>

<commit_message>
perf: two bundles, early data and image preloads, lighter openings
Measured on a mobile trace (Slow 4G, 4x CPU, DPR 2.6), detail LCP 7.5s → 2.96s,
home LCP 3.8s → 2.2s, CLS 0.15 → 0.
- The server serves CSS and JS as two gzipped bundles built from the files
  index.html lists (BUNDLE_ASSETS=0 serves them one by one); scripts are deferred.
- A journey deep link fetches its data from the page head and preloads its
  opening image (typed AVIF); share pages preload it server-side; the home
  opening preloads its AVIF only on the home route.
- Large derivatives use a lighter AVIF/WebP quality; later home scenes load
  shortly before they show.
- The main area keeps at least a screen of height so rendering never shifts the footer.
</commit_message>
<xml_diff>
--- a/app.xlsx
+++ b/app.xlsx
@@ -154,7 +154,7 @@
         </is>
       </c>
       <c r="B4">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -242,7 +242,7 @@
         </is>
       </c>
       <c r="E7">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="8">
@@ -1298,7 +1298,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>index_test</t>
+          <t>bundle_test</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>internal/webapp/index_test.go</t>
+          <t>internal/webapp/bundle_test.go</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1335,7 +1335,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>share_test</t>
+          <t>index_test</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -1345,7 +1345,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>internal/webapp/share_test.go</t>
+          <t>internal/webapp/index_test.go</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1367,12 +1367,12 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Playwright E2E</t>
+          <t>Go unit/integration / Go 单元集成</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>a11y.spec</t>
+          <t>share_test</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1382,7 +1382,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>e2e/tests/a11y.spec.js</t>
+          <t>internal/webapp/share_test.go</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1409,7 +1409,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>auth.spec</t>
+          <t>a11y.spec</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1419,7 +1419,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>e2e/tests/auth.spec.js</t>
+          <t>e2e/tests/a11y.spec.js</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -1446,7 +1446,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>detail.spec</t>
+          <t>auth.spec</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1456,7 +1456,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>e2e/tests/detail.spec.js</t>
+          <t>e2e/tests/auth.spec.js</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -1483,7 +1483,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>explore.spec</t>
+          <t>detail.spec</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -1493,7 +1493,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>e2e/tests/explore.spec.js</t>
+          <t>e2e/tests/detail.spec.js</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -1520,7 +1520,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>home.spec</t>
+          <t>explore.spec</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1530,7 +1530,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>e2e/tests/home.spec.js</t>
+          <t>e2e/tests/explore.spec.js</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -1557,7 +1557,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>i18n.spec</t>
+          <t>home.spec</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -1567,7 +1567,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>e2e/tests/i18n.spec.js</t>
+          <t>e2e/tests/home.spec.js</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -1594,7 +1594,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>mobile.spec</t>
+          <t>i18n.spec</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -1604,7 +1604,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>e2e/tests/mobile.spec.js</t>
+          <t>e2e/tests/i18n.spec.js</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -1631,7 +1631,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>orders.spec</t>
+          <t>mobile.spec</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -1641,7 +1641,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>e2e/tests/orders.spec.js</t>
+          <t>e2e/tests/mobile.spec.js</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -1668,7 +1668,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>persona.spec</t>
+          <t>orders.spec</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -1678,7 +1678,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>e2e/tests/persona.spec.js</t>
+          <t>e2e/tests/orders.spec.js</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -1705,7 +1705,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>space.spec</t>
+          <t>persona.spec</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -1715,7 +1715,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>e2e/tests/space.spec.js</t>
+          <t>e2e/tests/persona.spec.js</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -1737,12 +1737,12 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Playwright support / E2E 支撑文件</t>
+          <t>Playwright E2E</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>helpers</t>
+          <t>space.spec</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -1752,7 +1752,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>e2e/tests/helpers.js</t>
+          <t>e2e/tests/space.spec.js</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -1774,12 +1774,12 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Go stress</t>
+          <t>Playwright support / E2E 支撑文件</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>stress_test</t>
+          <t>helpers</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -1789,7 +1789,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>tests/stress/stress_test.go</t>
+          <t>e2e/tests/helpers.js</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -1811,12 +1811,12 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>k6 load / k6 负载</t>
+          <t>Go stress</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>admin-analytics-export.k6</t>
+          <t>stress_test</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -1826,7 +1826,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>tests/load/admin-analytics-export.k6.js</t>
+          <t>tests/stress/stress_test.go</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -1853,7 +1853,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>auth-register-login.k6</t>
+          <t>admin-analytics-export.k6</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -1863,7 +1863,7 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>tests/load/auth-register-login.k6.js</t>
+          <t>tests/load/admin-analytics-export.k6.js</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -1890,7 +1890,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>image-static-cache.k6</t>
+          <t>auth-register-login.k6</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -1900,7 +1900,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>tests/load/image-static-cache.k6.js</t>
+          <t>tests/load/auth-register-login.k6.js</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -1927,7 +1927,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>order-payment-audit.k6</t>
+          <t>image-static-cache.k6</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -1937,7 +1937,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>tests/load/order-payment-audit.k6.js</t>
+          <t>tests/load/image-static-cache.k6.js</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -1964,7 +1964,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>pet-chat-analytics.k6</t>
+          <t>order-payment-audit.k6</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -1974,7 +1974,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>tests/load/pet-chat-analytics.k6.js</t>
+          <t>tests/load/order-payment-audit.k6.js</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -2001,7 +2001,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>public-content-flow.k6</t>
+          <t>pet-chat-analytics.k6</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -2011,7 +2011,7 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>tests/load/public-content-flow.k6.js</t>
+          <t>tests/load/pet-chat-analytics.k6.js</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -2023,37 +2023,37 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Route</t>
+          <t>Test</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>ROUTE-001</t>
+          <t>TEST-041</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Admin</t>
+          <t>k6 load / k6 负载</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>GET /api/admin/export</t>
+          <t>public-content-flow.k6</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Route is registered</t>
+          <t>File exists and is part of repo</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>internal/handler/admin_handler.go</t>
+          <t>tests/load/public-content-flow.k6.js</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Specified</t>
         </is>
       </c>
     </row>
@@ -2065,7 +2065,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>ROUTE-002</t>
+          <t>ROUTE-001</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2075,7 +2075,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>GET /api/admin/stats</t>
+          <t>GET /api/admin/export</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -2102,7 +2102,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>ROUTE-003</t>
+          <t>ROUTE-002</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2112,7 +2112,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>GET /api/admin/users</t>
+          <t>GET /api/admin/stats</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -2139,17 +2139,17 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>ROUTE-004</t>
+          <t>ROUTE-003</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>Admin</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>POST /api/ai/chat</t>
+          <t>GET /api/admin/users</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -2159,7 +2159,7 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>internal/handler/admin_handler.go</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -2176,7 +2176,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>ROUTE-005</t>
+          <t>ROUTE-004</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2186,7 +2186,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>POST /api/analytics/events</t>
+          <t>POST /api/ai/chat</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -2213,7 +2213,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>ROUTE-006</t>
+          <t>ROUTE-005</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2223,7 +2223,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>POST /api/audit/client-error</t>
+          <t>POST /api/analytics/events</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -2250,17 +2250,17 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>ROUTE-007</t>
+          <t>ROUTE-006</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>POST /api/auth/avatar</t>
+          <t>POST /api/audit/client-error</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -2287,17 +2287,17 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>ROUTE-008</t>
+          <t>ROUTE-007</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>JWT</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>POST /api/auth/login</t>
+          <t>POST /api/auth/avatar</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -2324,17 +2324,17 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>ROUTE-009</t>
+          <t>ROUTE-008</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>PUT /api/auth/mbti</t>
+          <t>POST /api/auth/login</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -2344,7 +2344,7 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>internal/handler/me_handler.go</t>
+          <t>cmd/server/main.go</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -2361,7 +2361,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>ROUTE-010</t>
+          <t>ROUTE-009</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2371,7 +2371,7 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>GET /api/auth/me</t>
+          <t>PUT /api/auth/mbti</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -2381,7 +2381,7 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>internal/handler/me_handler.go</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -2398,17 +2398,17 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>ROUTE-011</t>
+          <t>ROUTE-010</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>JWT</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>POST /api/auth/register</t>
+          <t>GET /api/auth/me</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -2435,17 +2435,17 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>ROUTE-012</t>
+          <t>ROUTE-011</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>GET /api/auth/saved</t>
+          <t>POST /api/auth/register</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -2455,7 +2455,7 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>internal/handler/me_handler.go</t>
+          <t>cmd/server/main.go</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
@@ -2472,7 +2472,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>ROUTE-013</t>
+          <t>ROUTE-012</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -2482,7 +2482,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>DELETE /api/auth/saved/:slug</t>
+          <t>GET /api/auth/saved</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -2509,7 +2509,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>ROUTE-014</t>
+          <t>ROUTE-013</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -2519,7 +2519,7 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>PUT /api/auth/saved/:slug</t>
+          <t>DELETE /api/auth/saved/:slug</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -2546,17 +2546,17 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>ROUTE-015</t>
+          <t>ROUTE-014</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>JWT</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>GET /api/captcha</t>
+          <t>PUT /api/auth/saved/:slug</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -2566,7 +2566,7 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>internal/handler/me_handler.go</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -2583,7 +2583,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>ROUTE-016</t>
+          <t>ROUTE-015</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -2593,7 +2593,7 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>GET /api/health</t>
+          <t>GET /api/captcha</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -2620,7 +2620,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>ROUTE-017</t>
+          <t>ROUTE-016</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -2630,7 +2630,7 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>GET /api/journeys</t>
+          <t>GET /api/health</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -2657,7 +2657,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>ROUTE-018</t>
+          <t>ROUTE-017</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -2667,7 +2667,7 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>GET /api/journeys/:slug</t>
+          <t>GET /api/journeys</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -2694,7 +2694,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>ROUTE-019</t>
+          <t>ROUTE-018</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -2704,7 +2704,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>GET /api/journeys/:slug/book</t>
+          <t>GET /api/journeys/:slug</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -2731,7 +2731,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>ROUTE-020</t>
+          <t>ROUTE-019</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -2741,7 +2741,7 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>GET /api/mbti</t>
+          <t>GET /api/journeys/:slug/book</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -2768,17 +2768,17 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>ROUTE-021</t>
+          <t>ROUTE-020</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>GET /api/orders</t>
+          <t>GET /api/mbti</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -2788,7 +2788,7 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>internal/handler/order_handler.go</t>
+          <t>cmd/server/main.go</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -2805,7 +2805,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>ROUTE-022</t>
+          <t>ROUTE-021</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -2815,7 +2815,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>POST /api/orders</t>
+          <t>GET /api/orders</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -2842,7 +2842,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>ROUTE-023</t>
+          <t>ROUTE-022</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -2852,7 +2852,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>GET /api/orders/:id</t>
+          <t>POST /api/orders</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -2879,7 +2879,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>ROUTE-024</t>
+          <t>ROUTE-023</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -2889,7 +2889,7 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>POST /api/orders/:id/pay</t>
+          <t>GET /api/orders/:id</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -2916,7 +2916,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>ROUTE-025</t>
+          <t>ROUTE-024</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -2926,7 +2926,7 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>POST /api/payments/recharge</t>
+          <t>POST /api/orders/:id/pay</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -2936,7 +2936,7 @@
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>internal/handler/payment_handler.go</t>
+          <t>internal/handler/order_handler.go</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
@@ -2953,17 +2953,17 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>ROUTE-026</t>
+          <t>ROUTE-025</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>JWT</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>GET /api/payments/tiers</t>
+          <t>POST /api/payments/recharge</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
@@ -2990,17 +2990,17 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>ROUTE-027</t>
+          <t>ROUTE-026</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>GET /api/payments/transactions</t>
+          <t>GET /api/payments/tiers</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -3027,30 +3027,67 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
+          <t>ROUTE-027</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>JWT</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>GET /api/payments/transactions</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Route is registered</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>internal/handler/payment_handler.go</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Route</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
           <t>ROUTE-028</t>
         </is>
       </c>
-      <c r="C74" t="inlineStr">
+      <c r="C75" t="inlineStr">
         <is>
           <t>Public</t>
         </is>
       </c>
-      <c r="D74" t="inlineStr">
+      <c r="D75" t="inlineStr">
         <is>
           <t>GET /api/tags</t>
         </is>
       </c>
-      <c r="E74" t="inlineStr">
+      <c r="E75" t="inlineStr">
         <is>
           <t>Route is registered</t>
         </is>
       </c>
-      <c r="F74" t="inlineStr">
+      <c r="F75" t="inlineStr">
         <is>
           <t>cmd/server/main.go</t>
         </is>
       </c>
-      <c r="G74" t="inlineStr">
+      <c r="G75" t="inlineStr">
         <is>
           <t>Implemented</t>
         </is>

</xml_diff>

<commit_message>
Compose game: draw your own entrance (#4)
Piece a ticket together from paper slips (a place, an hour, a season, how long
you stay, a small ritual, what you take home) by tap, drag or keyboard; kept
tickets are stamped, merge into the account on sign-in and can be shared by a
read-only link. Fragments are validated like the entrances.
</commit_message>
<xml_diff>
--- a/app.xlsx
+++ b/app.xlsx
@@ -154,7 +154,7 @@
         </is>
       </c>
       <c r="B4">
-        <v>74</v>
+        <v>82</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -217,7 +217,7 @@
         </is>
       </c>
       <c r="E6">
-        <v>28</v>
+        <v>33</v>
       </c>
     </row>
     <row r="7">
@@ -242,7 +242,7 @@
         </is>
       </c>
       <c r="E7">
-        <v>41</v>
+        <v>44</v>
       </c>
     </row>
     <row r="8">
@@ -706,7 +706,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>content_test</t>
+          <t>compose_test</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -716,7 +716,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>internal/content/content_test.go</t>
+          <t>internal/compose/compose_test.go</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -743,7 +743,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>admin_handler_test</t>
+          <t>content_test</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -753,7 +753,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>internal/handler/admin_handler_test.go</t>
+          <t>internal/content/content_test.go</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -780,7 +780,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>auth_handler_test</t>
+          <t>admin_handler_test</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -790,7 +790,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>internal/handler/auth_handler_test.go</t>
+          <t>internal/handler/admin_handler_test.go</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -817,7 +817,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>journey_handler_test</t>
+          <t>auth_handler_test</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -827,7 +827,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>internal/handler/journey_handler_test.go</t>
+          <t>internal/handler/auth_handler_test.go</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -854,7 +854,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>me_handler_test</t>
+          <t>compose_handler_test</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -864,7 +864,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>internal/handler/me_handler_test.go</t>
+          <t>internal/handler/compose_handler_test.go</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -891,7 +891,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>order_handler_test</t>
+          <t>journey_handler_test</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -901,7 +901,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>internal/handler/order_handler_test.go</t>
+          <t>internal/handler/journey_handler_test.go</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -928,7 +928,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>payment_handler_test</t>
+          <t>me_handler_test</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -938,7 +938,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>internal/handler/payment_handler_test.go</t>
+          <t>internal/handler/me_handler_test.go</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -965,7 +965,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>cors_test</t>
+          <t>order_handler_test</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -975,7 +975,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>internal/middleware/cors_test.go</t>
+          <t>internal/handler/order_handler_test.go</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1002,7 +1002,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>jwt_test</t>
+          <t>payment_handler_test</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1012,7 +1012,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>internal/middleware/jwt_test.go</t>
+          <t>internal/handler/payment_handler_test.go</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1039,7 +1039,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>request_id_test</t>
+          <t>cors_test</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1049,7 +1049,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>internal/middleware/request_id_test.go</t>
+          <t>internal/middleware/cors_test.go</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1076,7 +1076,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>journey_repo_sqlite_test</t>
+          <t>jwt_test</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1086,7 +1086,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>internal/repository/journey_repo_sqlite_test.go</t>
+          <t>internal/middleware/jwt_test.go</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1113,7 +1113,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>migrate_test</t>
+          <t>request_id_test</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1123,7 +1123,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>internal/repository/migrate_test.go</t>
+          <t>internal/middleware/request_id_test.go</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1150,7 +1150,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>order_repo_test</t>
+          <t>journey_repo_sqlite_test</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1160,7 +1160,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>internal/repository/order_repo_test.go</t>
+          <t>internal/repository/journey_repo_sqlite_test.go</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1187,7 +1187,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>user_repo_test</t>
+          <t>migrate_test</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1197,7 +1197,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>internal/repository/user_repo_test.go</t>
+          <t>internal/repository/migrate_test.go</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1224,7 +1224,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>journey_service_test</t>
+          <t>order_repo_test</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1234,7 +1234,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>internal/service/journey_service_test.go</t>
+          <t>internal/repository/order_repo_test.go</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1261,7 +1261,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>locale_test</t>
+          <t>user_repo_test</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1271,7 +1271,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>internal/service/locale_test.go</t>
+          <t>internal/repository/user_repo_test.go</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1298,7 +1298,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>bundle_test</t>
+          <t>journey_service_test</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>internal/webapp/bundle_test.go</t>
+          <t>internal/service/journey_service_test.go</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1335,7 +1335,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>index_test</t>
+          <t>locale_test</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -1345,7 +1345,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>internal/webapp/index_test.go</t>
+          <t>internal/service/locale_test.go</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1372,7 +1372,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>share_test</t>
+          <t>bundle_test</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1382,7 +1382,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>internal/webapp/share_test.go</t>
+          <t>internal/webapp/bundle_test.go</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1404,12 +1404,12 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Playwright E2E</t>
+          <t>Go unit/integration / Go 单元集成</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>a11y.spec</t>
+          <t>index_test</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1419,7 +1419,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>e2e/tests/a11y.spec.js</t>
+          <t>internal/webapp/index_test.go</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -1441,12 +1441,12 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Playwright E2E</t>
+          <t>Go unit/integration / Go 单元集成</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>auth.spec</t>
+          <t>share_test</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1456,7 +1456,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>e2e/tests/auth.spec.js</t>
+          <t>internal/webapp/share_test.go</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -1483,7 +1483,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>detail.spec</t>
+          <t>a11y.spec</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -1493,7 +1493,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>e2e/tests/detail.spec.js</t>
+          <t>e2e/tests/a11y.spec.js</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -1520,7 +1520,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>explore.spec</t>
+          <t>auth.spec</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1530,7 +1530,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>e2e/tests/explore.spec.js</t>
+          <t>e2e/tests/auth.spec.js</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -1557,7 +1557,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>home.spec</t>
+          <t>compose.spec</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -1567,7 +1567,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>e2e/tests/home.spec.js</t>
+          <t>e2e/tests/compose.spec.js</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -1594,7 +1594,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>i18n.spec</t>
+          <t>detail.spec</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -1604,7 +1604,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>e2e/tests/i18n.spec.js</t>
+          <t>e2e/tests/detail.spec.js</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -1631,7 +1631,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>mobile.spec</t>
+          <t>explore.spec</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -1641,7 +1641,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>e2e/tests/mobile.spec.js</t>
+          <t>e2e/tests/explore.spec.js</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -1668,7 +1668,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>orders.spec</t>
+          <t>home.spec</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -1678,7 +1678,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>e2e/tests/orders.spec.js</t>
+          <t>e2e/tests/home.spec.js</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -1705,7 +1705,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>persona.spec</t>
+          <t>i18n.spec</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -1715,7 +1715,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>e2e/tests/persona.spec.js</t>
+          <t>e2e/tests/i18n.spec.js</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -1742,7 +1742,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>space.spec</t>
+          <t>mobile.spec</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -1752,7 +1752,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>e2e/tests/space.spec.js</t>
+          <t>e2e/tests/mobile.spec.js</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -1774,12 +1774,12 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Playwright support / E2E 支撑文件</t>
+          <t>Playwright E2E</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>helpers</t>
+          <t>orders.spec</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -1789,7 +1789,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>e2e/tests/helpers.js</t>
+          <t>e2e/tests/orders.spec.js</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -1811,12 +1811,12 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Go stress</t>
+          <t>Playwright E2E</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>stress_test</t>
+          <t>persona.spec</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -1826,7 +1826,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>tests/stress/stress_test.go</t>
+          <t>e2e/tests/persona.spec.js</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -1848,12 +1848,12 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>k6 load / k6 负载</t>
+          <t>Playwright E2E</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>admin-analytics-export.k6</t>
+          <t>space.spec</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -1863,7 +1863,7 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>tests/load/admin-analytics-export.k6.js</t>
+          <t>e2e/tests/space.spec.js</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -1885,12 +1885,12 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>k6 load / k6 负载</t>
+          <t>Playwright support / E2E 支撑文件</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>auth-register-login.k6</t>
+          <t>helpers</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -1900,7 +1900,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>tests/load/auth-register-login.k6.js</t>
+          <t>e2e/tests/helpers.js</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -1922,12 +1922,12 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>k6 load / k6 负载</t>
+          <t>Go stress</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>image-static-cache.k6</t>
+          <t>stress_test</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -1937,7 +1937,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>tests/load/image-static-cache.k6.js</t>
+          <t>tests/stress/stress_test.go</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -1964,7 +1964,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>order-payment-audit.k6</t>
+          <t>admin-analytics-export.k6</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -1974,7 +1974,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>tests/load/order-payment-audit.k6.js</t>
+          <t>tests/load/admin-analytics-export.k6.js</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -2001,7 +2001,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>pet-chat-analytics.k6</t>
+          <t>auth-register-login.k6</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -2011,7 +2011,7 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>tests/load/pet-chat-analytics.k6.js</t>
+          <t>tests/load/auth-register-login.k6.js</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -2038,7 +2038,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>public-content-flow.k6</t>
+          <t>image-static-cache.k6</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -2048,7 +2048,7 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>tests/load/public-content-flow.k6.js</t>
+          <t>tests/load/image-static-cache.k6.js</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -2060,111 +2060,111 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Route</t>
+          <t>Test</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>ROUTE-001</t>
+          <t>TEST-042</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Admin</t>
+          <t>k6 load / k6 负载</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>GET /api/admin/export</t>
+          <t>order-payment-audit.k6</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Route is registered</t>
+          <t>File exists and is part of repo</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>internal/handler/admin_handler.go</t>
+          <t>tests/load/order-payment-audit.k6.js</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Specified</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Route</t>
+          <t>Test</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>ROUTE-002</t>
+          <t>TEST-043</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Admin</t>
+          <t>k6 load / k6 负载</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>GET /api/admin/stats</t>
+          <t>pet-chat-analytics.k6</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Route is registered</t>
+          <t>File exists and is part of repo</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>internal/handler/admin_handler.go</t>
+          <t>tests/load/pet-chat-analytics.k6.js</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Specified</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Route</t>
+          <t>Test</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>ROUTE-003</t>
+          <t>TEST-044</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Admin</t>
+          <t>k6 load / k6 负载</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>GET /api/admin/users</t>
+          <t>public-content-flow.k6</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Route is registered</t>
+          <t>File exists and is part of repo</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>internal/handler/admin_handler.go</t>
+          <t>tests/load/public-content-flow.k6.js</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Specified</t>
         </is>
       </c>
     </row>
@@ -2176,17 +2176,17 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>ROUTE-004</t>
+          <t>ROUTE-001</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>Admin</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>POST /api/ai/chat</t>
+          <t>GET /api/admin/export</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -2196,7 +2196,7 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>internal/handler/admin_handler.go</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -2213,17 +2213,17 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>ROUTE-005</t>
+          <t>ROUTE-002</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>Admin</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>POST /api/analytics/events</t>
+          <t>GET /api/admin/stats</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -2233,7 +2233,7 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>internal/handler/admin_handler.go</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -2250,17 +2250,17 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>ROUTE-006</t>
+          <t>ROUTE-003</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>Admin</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>POST /api/audit/client-error</t>
+          <t>GET /api/admin/users</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -2270,7 +2270,7 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>internal/handler/admin_handler.go</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -2287,17 +2287,17 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>ROUTE-007</t>
+          <t>ROUTE-004</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>POST /api/auth/avatar</t>
+          <t>POST /api/ai/chat</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -2324,7 +2324,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>ROUTE-008</t>
+          <t>ROUTE-005</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2334,7 +2334,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>POST /api/auth/login</t>
+          <t>POST /api/analytics/events</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -2361,17 +2361,17 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>ROUTE-009</t>
+          <t>ROUTE-006</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>PUT /api/auth/mbti</t>
+          <t>POST /api/audit/client-error</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -2381,7 +2381,7 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>internal/handler/me_handler.go</t>
+          <t>cmd/server/main.go</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -2398,7 +2398,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>ROUTE-010</t>
+          <t>ROUTE-007</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -2408,7 +2408,7 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>GET /api/auth/me</t>
+          <t>POST /api/auth/avatar</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -2435,17 +2435,17 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>ROUTE-011</t>
+          <t>ROUTE-008</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>JWT</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>POST /api/auth/register</t>
+          <t>GET /api/auth/compositions</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -2455,7 +2455,7 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>internal/handler/compose_handler.go</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
@@ -2472,7 +2472,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>ROUTE-012</t>
+          <t>ROUTE-009</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -2482,7 +2482,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>GET /api/auth/saved</t>
+          <t>POST /api/auth/compositions</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -2492,7 +2492,7 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>internal/handler/me_handler.go</t>
+          <t>internal/handler/compose_handler.go</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
@@ -2509,7 +2509,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>ROUTE-013</t>
+          <t>ROUTE-010</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -2519,7 +2519,7 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>DELETE /api/auth/saved/:slug</t>
+          <t>DELETE /api/auth/compositions/:id</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -2529,7 +2529,7 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>internal/handler/me_handler.go</t>
+          <t>internal/handler/compose_handler.go</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -2546,17 +2546,17 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>ROUTE-014</t>
+          <t>ROUTE-011</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>PUT /api/auth/saved/:slug</t>
+          <t>POST /api/auth/login</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -2566,7 +2566,7 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>internal/handler/me_handler.go</t>
+          <t>cmd/server/main.go</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -2583,17 +2583,17 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>ROUTE-015</t>
+          <t>ROUTE-012</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>JWT</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>GET /api/captcha</t>
+          <t>PUT /api/auth/mbti</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -2603,7 +2603,7 @@
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>internal/handler/me_handler.go</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
@@ -2620,17 +2620,17 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>ROUTE-016</t>
+          <t>ROUTE-013</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>JWT</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>GET /api/health</t>
+          <t>GET /api/auth/me</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -2657,7 +2657,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>ROUTE-017</t>
+          <t>ROUTE-014</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -2667,7 +2667,7 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>GET /api/journeys</t>
+          <t>POST /api/auth/register</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -2694,17 +2694,17 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>ROUTE-018</t>
+          <t>ROUTE-015</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>JWT</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>GET /api/journeys/:slug</t>
+          <t>GET /api/auth/saved</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -2714,7 +2714,7 @@
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>internal/handler/me_handler.go</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
@@ -2731,17 +2731,17 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>ROUTE-019</t>
+          <t>ROUTE-016</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>JWT</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>GET /api/journeys/:slug/book</t>
+          <t>DELETE /api/auth/saved/:slug</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -2751,7 +2751,7 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>internal/handler/me_handler.go</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
@@ -2768,17 +2768,17 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>ROUTE-020</t>
+          <t>ROUTE-017</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>JWT</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>GET /api/mbti</t>
+          <t>PUT /api/auth/saved/:slug</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -2788,7 +2788,7 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>internal/handler/me_handler.go</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -2805,17 +2805,17 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>ROUTE-021</t>
+          <t>ROUTE-018</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>GET /api/orders</t>
+          <t>GET /api/captcha</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -2825,7 +2825,7 @@
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>internal/handler/order_handler.go</t>
+          <t>cmd/server/main.go</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
@@ -2842,17 +2842,17 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>ROUTE-022</t>
+          <t>ROUTE-019</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>POST /api/orders</t>
+          <t>GET /api/compose/fragments</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -2862,7 +2862,7 @@
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>internal/handler/order_handler.go</t>
+          <t>internal/handler/compose_handler.go</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
@@ -2879,17 +2879,17 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>ROUTE-023</t>
+          <t>ROUTE-020</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>GET /api/orders/:id</t>
+          <t>GET /api/compositions/:code</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -2899,7 +2899,7 @@
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>internal/handler/order_handler.go</t>
+          <t>internal/handler/compose_handler.go</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
@@ -2916,17 +2916,17 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>ROUTE-024</t>
+          <t>ROUTE-021</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>POST /api/orders/:id/pay</t>
+          <t>GET /api/health</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -2936,7 +2936,7 @@
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>internal/handler/order_handler.go</t>
+          <t>cmd/server/main.go</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
@@ -2953,17 +2953,17 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>ROUTE-025</t>
+          <t>ROUTE-022</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>POST /api/payments/recharge</t>
+          <t>GET /api/journeys</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
@@ -2973,7 +2973,7 @@
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>internal/handler/payment_handler.go</t>
+          <t>cmd/server/main.go</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
@@ -2990,7 +2990,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>ROUTE-026</t>
+          <t>ROUTE-023</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -3000,7 +3000,7 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>GET /api/payments/tiers</t>
+          <t>GET /api/journeys/:slug</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -3010,7 +3010,7 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>internal/handler/payment_handler.go</t>
+          <t>cmd/server/main.go</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -3027,17 +3027,17 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>ROUTE-027</t>
+          <t>ROUTE-024</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>GET /api/payments/transactions</t>
+          <t>GET /api/journeys/:slug/book</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -3047,7 +3047,7 @@
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>internal/handler/payment_handler.go</t>
+          <t>cmd/server/main.go</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
@@ -3064,30 +3064,326 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
+          <t>ROUTE-025</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>GET /api/mbti</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>Route is registered</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>cmd/server/main.go</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Route</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>ROUTE-026</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>JWT</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>GET /api/orders</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>Route is registered</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>internal/handler/order_handler.go</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Route</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>ROUTE-027</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>JWT</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>POST /api/orders</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>Route is registered</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>internal/handler/order_handler.go</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Route</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
           <t>ROUTE-028</t>
         </is>
       </c>
-      <c r="C75" t="inlineStr">
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>JWT</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>GET /api/orders/:id</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>Route is registered</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>internal/handler/order_handler.go</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Route</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>ROUTE-029</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>JWT</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>POST /api/orders/:id/pay</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>Route is registered</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>internal/handler/order_handler.go</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Route</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>ROUTE-030</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>JWT</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>POST /api/payments/recharge</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Route is registered</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>internal/handler/payment_handler.go</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Route</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>ROUTE-031</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
         <is>
           <t>Public</t>
         </is>
       </c>
-      <c r="D75" t="inlineStr">
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>GET /api/payments/tiers</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Route is registered</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>internal/handler/payment_handler.go</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Route</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>ROUTE-032</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>JWT</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>GET /api/payments/transactions</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>Route is registered</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>internal/handler/payment_handler.go</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Route</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>ROUTE-033</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
         <is>
           <t>GET /api/tags</t>
         </is>
       </c>
-      <c r="E75" t="inlineStr">
+      <c r="E83" t="inlineStr">
         <is>
           <t>Route is registered</t>
         </is>
       </c>
-      <c r="F75" t="inlineStr">
+      <c r="F83" t="inlineStr">
         <is>
           <t>cmd/server/main.go</t>
         </is>
       </c>
-      <c r="G75" t="inlineStr">
+      <c r="G83" t="inlineStr">
         <is>
           <t>Implemented</t>
         </is>

</xml_diff>

<commit_message>
road: mount between the practical notes and the small print; quieter copy
The entrance page no longer has a facts panel; the rubbing, the lantern and
the line of tickets now hang between the practical notes and the one line
of small print. Moments carry themselves: the headings over the rubbing,
the lantern, the line and the drifted tickets are for screen readers only,
the paper shows a worn corner instead of an instruction, and the lamp's
"it's up" is heard, not shown. The line scrolls sideways in a narrow column.
</commit_message>
<xml_diff>
--- a/app.xlsx
+++ b/app.xlsx
@@ -154,7 +154,7 @@
         </is>
       </c>
       <c r="B4">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -242,7 +242,7 @@
         </is>
       </c>
       <c r="E7">
-        <v>44</v>
+        <v>50</v>
       </c>
     </row>
     <row r="8">
@@ -743,7 +743,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>content_test</t>
+          <t>derive_test</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -753,7 +753,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>internal/content/content_test.go</t>
+          <t>internal/compose/derive_test.go</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -780,7 +780,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>admin_handler_test</t>
+          <t>content_test</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -790,7 +790,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>internal/handler/admin_handler_test.go</t>
+          <t>internal/content/content_test.go</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -817,7 +817,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>auth_handler_test</t>
+          <t>admin_handler_test</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -827,7 +827,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>internal/handler/auth_handler_test.go</t>
+          <t>internal/handler/admin_handler_test.go</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -854,7 +854,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>compose_handler_test</t>
+          <t>auth_handler_test</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -864,7 +864,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>internal/handler/compose_handler_test.go</t>
+          <t>internal/handler/auth_handler_test.go</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -891,7 +891,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>journey_handler_test</t>
+          <t>compose_handler_test</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -901,7 +901,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>internal/handler/journey_handler_test.go</t>
+          <t>internal/handler/compose_handler_test.go</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -928,7 +928,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>me_handler_test</t>
+          <t>journey_handler_test</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -938,7 +938,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>internal/handler/me_handler_test.go</t>
+          <t>internal/handler/journey_handler_test.go</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -965,7 +965,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>order_handler_test</t>
+          <t>me_handler_test</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -975,7 +975,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>internal/handler/order_handler_test.go</t>
+          <t>internal/handler/me_handler_test.go</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1002,7 +1002,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>payment_handler_test</t>
+          <t>order_handler_test</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1012,7 +1012,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>internal/handler/payment_handler_test.go</t>
+          <t>internal/handler/order_handler_test.go</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1039,7 +1039,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>cors_test</t>
+          <t>payment_handler_test</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1049,7 +1049,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>internal/middleware/cors_test.go</t>
+          <t>internal/handler/payment_handler_test.go</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1076,7 +1076,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>jwt_test</t>
+          <t>road_handler_test</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1086,7 +1086,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>internal/middleware/jwt_test.go</t>
+          <t>internal/handler/road_handler_test.go</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1113,7 +1113,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>request_id_test</t>
+          <t>cors_test</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1123,7 +1123,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>internal/middleware/request_id_test.go</t>
+          <t>internal/middleware/cors_test.go</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1150,7 +1150,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>journey_repo_sqlite_test</t>
+          <t>jwt_test</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1160,7 +1160,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>internal/repository/journey_repo_sqlite_test.go</t>
+          <t>internal/middleware/jwt_test.go</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1187,7 +1187,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>migrate_test</t>
+          <t>ratelimit_test</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1197,7 +1197,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>internal/repository/migrate_test.go</t>
+          <t>internal/middleware/ratelimit_test.go</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1224,7 +1224,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>order_repo_test</t>
+          <t>request_id_test</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1234,7 +1234,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>internal/repository/order_repo_test.go</t>
+          <t>internal/middleware/request_id_test.go</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1261,7 +1261,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>user_repo_test</t>
+          <t>journey_repo_sqlite_test</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1271,7 +1271,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>internal/repository/user_repo_test.go</t>
+          <t>internal/repository/journey_repo_sqlite_test.go</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1298,7 +1298,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>journey_service_test</t>
+          <t>migrate_test</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>internal/service/journey_service_test.go</t>
+          <t>internal/repository/migrate_test.go</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1335,7 +1335,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>locale_test</t>
+          <t>order_repo_test</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -1345,7 +1345,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>internal/service/locale_test.go</t>
+          <t>internal/repository/order_repo_test.go</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1372,7 +1372,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>bundle_test</t>
+          <t>user_repo_test</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1382,7 +1382,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>internal/webapp/bundle_test.go</t>
+          <t>internal/repository/user_repo_test.go</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1409,7 +1409,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>index_test</t>
+          <t>light_test</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1419,7 +1419,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>internal/webapp/index_test.go</t>
+          <t>internal/road/light/light_test.go</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -1446,7 +1446,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>share_test</t>
+          <t>road_test</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1456,7 +1456,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>internal/webapp/share_test.go</t>
+          <t>internal/road/road_test.go</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -1478,12 +1478,12 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Playwright E2E</t>
+          <t>Go unit/integration / Go 单元集成</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>a11y.spec</t>
+          <t>journey_service_test</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -1493,7 +1493,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>e2e/tests/a11y.spec.js</t>
+          <t>internal/service/journey_service_test.go</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -1515,12 +1515,12 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Playwright E2E</t>
+          <t>Go unit/integration / Go 单元集成</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>auth.spec</t>
+          <t>locale_test</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1530,7 +1530,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>e2e/tests/auth.spec.js</t>
+          <t>internal/service/locale_test.go</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -1552,12 +1552,12 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Playwright E2E</t>
+          <t>Go unit/integration / Go 单元集成</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>compose.spec</t>
+          <t>bundle_test</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -1567,7 +1567,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>e2e/tests/compose.spec.js</t>
+          <t>internal/webapp/bundle_test.go</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -1589,12 +1589,12 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Playwright E2E</t>
+          <t>Go unit/integration / Go 单元集成</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>detail.spec</t>
+          <t>index_test</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -1604,7 +1604,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>e2e/tests/detail.spec.js</t>
+          <t>internal/webapp/index_test.go</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -1626,12 +1626,12 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Playwright E2E</t>
+          <t>Go unit/integration / Go 单元集成</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>explore.spec</t>
+          <t>share_test</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -1641,7 +1641,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>e2e/tests/explore.spec.js</t>
+          <t>internal/webapp/share_test.go</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -1668,7 +1668,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>home.spec</t>
+          <t>a11y.spec</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -1678,7 +1678,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>e2e/tests/home.spec.js</t>
+          <t>e2e/tests/a11y.spec.js</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -1705,7 +1705,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>i18n.spec</t>
+          <t>auth.spec</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -1715,7 +1715,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>e2e/tests/i18n.spec.js</t>
+          <t>e2e/tests/auth.spec.js</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -1742,7 +1742,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>mobile.spec</t>
+          <t>compose.spec</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -1752,7 +1752,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>e2e/tests/mobile.spec.js</t>
+          <t>e2e/tests/compose.spec.js</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -1779,7 +1779,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>orders.spec</t>
+          <t>detail.spec</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -1789,7 +1789,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>e2e/tests/orders.spec.js</t>
+          <t>e2e/tests/detail.spec.js</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -1816,7 +1816,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>persona.spec</t>
+          <t>explore.spec</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -1826,7 +1826,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>e2e/tests/persona.spec.js</t>
+          <t>e2e/tests/explore.spec.js</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -1853,7 +1853,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>space.spec</t>
+          <t>home.spec</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -1863,7 +1863,7 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>e2e/tests/space.spec.js</t>
+          <t>e2e/tests/home.spec.js</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -1885,12 +1885,12 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Playwright support / E2E 支撑文件</t>
+          <t>Playwright E2E</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>helpers</t>
+          <t>i18n.spec</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -1900,7 +1900,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>e2e/tests/helpers.js</t>
+          <t>e2e/tests/i18n.spec.js</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -1922,12 +1922,12 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Go stress</t>
+          <t>Playwright E2E</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>stress_test</t>
+          <t>mobile.spec</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -1937,7 +1937,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>tests/stress/stress_test.go</t>
+          <t>e2e/tests/mobile.spec.js</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -1959,12 +1959,12 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>k6 load / k6 负载</t>
+          <t>Playwright E2E</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>admin-analytics-export.k6</t>
+          <t>orders.spec</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -1974,7 +1974,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>tests/load/admin-analytics-export.k6.js</t>
+          <t>e2e/tests/orders.spec.js</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -1996,12 +1996,12 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>k6 load / k6 负载</t>
+          <t>Playwright E2E</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>auth-register-login.k6</t>
+          <t>persona.spec</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -2011,7 +2011,7 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>tests/load/auth-register-login.k6.js</t>
+          <t>e2e/tests/persona.spec.js</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -2033,12 +2033,12 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>k6 load / k6 负载</t>
+          <t>Playwright E2E</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>image-static-cache.k6</t>
+          <t>road.spec</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -2048,7 +2048,7 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>tests/load/image-static-cache.k6.js</t>
+          <t>e2e/tests/road.spec.js</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -2070,12 +2070,12 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>k6 load / k6 负载</t>
+          <t>Playwright E2E</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>order-payment-audit.k6</t>
+          <t>space.spec</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -2085,7 +2085,7 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>tests/load/order-payment-audit.k6.js</t>
+          <t>e2e/tests/space.spec.js</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -2107,12 +2107,12 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>k6 load / k6 负载</t>
+          <t>Playwright support / E2E 支撑文件</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>pet-chat-analytics.k6</t>
+          <t>helpers</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -2122,7 +2122,7 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>tests/load/pet-chat-analytics.k6.js</t>
+          <t>e2e/tests/helpers.js</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -2144,12 +2144,12 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>k6 load / k6 负载</t>
+          <t>Go stress</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>public-content-flow.k6</t>
+          <t>stress_test</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -2159,7 +2159,7 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>tests/load/public-content-flow.k6.js</t>
+          <t>tests/stress/stress_test.go</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -2171,222 +2171,222 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Route</t>
+          <t>Test</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>ROUTE-001</t>
+          <t>TEST-045</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Admin</t>
+          <t>k6 load / k6 负载</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>GET /api/admin/export</t>
+          <t>admin-analytics-export.k6</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Route is registered</t>
+          <t>File exists and is part of repo</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>internal/handler/admin_handler.go</t>
+          <t>tests/load/admin-analytics-export.k6.js</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Specified</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Route</t>
+          <t>Test</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>ROUTE-002</t>
+          <t>TEST-046</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Admin</t>
+          <t>k6 load / k6 负载</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>GET /api/admin/stats</t>
+          <t>auth-register-login.k6</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Route is registered</t>
+          <t>File exists and is part of repo</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>internal/handler/admin_handler.go</t>
+          <t>tests/load/auth-register-login.k6.js</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Specified</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Route</t>
+          <t>Test</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>ROUTE-003</t>
+          <t>TEST-047</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Admin</t>
+          <t>k6 load / k6 负载</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>GET /api/admin/users</t>
+          <t>image-static-cache.k6</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Route is registered</t>
+          <t>File exists and is part of repo</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>internal/handler/admin_handler.go</t>
+          <t>tests/load/image-static-cache.k6.js</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Specified</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Route</t>
+          <t>Test</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>ROUTE-004</t>
+          <t>TEST-048</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>k6 load / k6 负载</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>POST /api/ai/chat</t>
+          <t>order-payment-audit.k6</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Route is registered</t>
+          <t>File exists and is part of repo</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>tests/load/order-payment-audit.k6.js</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Specified</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Route</t>
+          <t>Test</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>ROUTE-005</t>
+          <t>TEST-049</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>k6 load / k6 负载</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>POST /api/analytics/events</t>
+          <t>pet-chat-analytics.k6</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Route is registered</t>
+          <t>File exists and is part of repo</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>tests/load/pet-chat-analytics.k6.js</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Specified</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Route</t>
+          <t>Test</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>ROUTE-006</t>
+          <t>TEST-050</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>k6 load / k6 负载</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>POST /api/audit/client-error</t>
+          <t>public-content-flow.k6</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Route is registered</t>
+          <t>File exists and is part of repo</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>tests/load/public-content-flow.k6.js</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Specified</t>
         </is>
       </c>
     </row>
@@ -2398,17 +2398,17 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>ROUTE-007</t>
+          <t>ROUTE-001</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Admin</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>POST /api/auth/avatar</t>
+          <t>GET /api/admin/export</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -2418,7 +2418,7 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>internal/handler/admin_handler.go</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -2435,17 +2435,17 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>ROUTE-008</t>
+          <t>ROUTE-002</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Admin</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>GET /api/auth/compositions</t>
+          <t>GET /api/admin/stats</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -2455,7 +2455,7 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>internal/handler/compose_handler.go</t>
+          <t>internal/handler/admin_handler.go</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
@@ -2472,17 +2472,17 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>ROUTE-009</t>
+          <t>ROUTE-003</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Admin</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>POST /api/auth/compositions</t>
+          <t>GET /api/admin/users</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -2492,7 +2492,7 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>internal/handler/compose_handler.go</t>
+          <t>internal/handler/admin_handler.go</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
@@ -2509,17 +2509,17 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>ROUTE-010</t>
+          <t>ROUTE-004</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>DELETE /api/auth/compositions/:id</t>
+          <t>POST /api/ai/chat</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -2529,7 +2529,7 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>internal/handler/compose_handler.go</t>
+          <t>cmd/server/main.go</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -2546,7 +2546,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>ROUTE-011</t>
+          <t>ROUTE-005</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -2556,7 +2556,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>POST /api/auth/login</t>
+          <t>POST /api/analytics/events</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -2583,17 +2583,17 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>ROUTE-012</t>
+          <t>ROUTE-006</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>PUT /api/auth/mbti</t>
+          <t>POST /api/audit/client-error</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -2603,7 +2603,7 @@
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>internal/handler/me_handler.go</t>
+          <t>cmd/server/main.go</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
@@ -2620,7 +2620,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>ROUTE-013</t>
+          <t>ROUTE-007</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -2630,7 +2630,7 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>GET /api/auth/me</t>
+          <t>POST /api/auth/avatar</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -2657,17 +2657,17 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>ROUTE-014</t>
+          <t>ROUTE-008</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>JWT</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>POST /api/auth/register</t>
+          <t>GET /api/auth/compositions</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -2677,7 +2677,7 @@
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>internal/handler/compose_handler.go</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -2694,7 +2694,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>ROUTE-015</t>
+          <t>ROUTE-009</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -2704,7 +2704,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>GET /api/auth/saved</t>
+          <t>POST /api/auth/compositions</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -2714,7 +2714,7 @@
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>internal/handler/me_handler.go</t>
+          <t>internal/handler/compose_handler.go</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
@@ -2731,7 +2731,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>ROUTE-016</t>
+          <t>ROUTE-010</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -2741,7 +2741,7 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>DELETE /api/auth/saved/:slug</t>
+          <t>DELETE /api/auth/compositions/:id</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -2751,7 +2751,7 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>internal/handler/me_handler.go</t>
+          <t>internal/handler/compose_handler.go</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
@@ -2768,17 +2768,17 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>ROUTE-017</t>
+          <t>ROUTE-011</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>PUT /api/auth/saved/:slug</t>
+          <t>POST /api/auth/login</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -2788,7 +2788,7 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>internal/handler/me_handler.go</t>
+          <t>cmd/server/main.go</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -2805,17 +2805,17 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>ROUTE-018</t>
+          <t>ROUTE-012</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>JWT</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>GET /api/captcha</t>
+          <t>PUT /api/auth/mbti</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -2825,7 +2825,7 @@
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>internal/handler/me_handler.go</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
@@ -2842,17 +2842,17 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>ROUTE-019</t>
+          <t>ROUTE-013</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>JWT</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>GET /api/compose/fragments</t>
+          <t>GET /api/auth/me</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -2862,7 +2862,7 @@
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>internal/handler/compose_handler.go</t>
+          <t>cmd/server/main.go</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
@@ -2879,7 +2879,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>ROUTE-020</t>
+          <t>ROUTE-014</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -2889,7 +2889,7 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>GET /api/compositions/:code</t>
+          <t>POST /api/auth/register</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -2899,7 +2899,7 @@
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>internal/handler/compose_handler.go</t>
+          <t>cmd/server/main.go</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
@@ -2916,17 +2916,17 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>ROUTE-021</t>
+          <t>ROUTE-015</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>JWT</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>GET /api/health</t>
+          <t>GET /api/auth/saved</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -2936,7 +2936,7 @@
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>internal/handler/me_handler.go</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
@@ -2953,17 +2953,17 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>ROUTE-022</t>
+          <t>ROUTE-016</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>JWT</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>GET /api/journeys</t>
+          <t>DELETE /api/auth/saved/:slug</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
@@ -2973,7 +2973,7 @@
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>internal/handler/me_handler.go</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
@@ -2990,17 +2990,17 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>ROUTE-023</t>
+          <t>ROUTE-017</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>JWT</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>GET /api/journeys/:slug</t>
+          <t>PUT /api/auth/saved/:slug</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -3010,7 +3010,7 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>internal/handler/me_handler.go</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>ROUTE-024</t>
+          <t>ROUTE-018</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -3037,7 +3037,7 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>GET /api/journeys/:slug/book</t>
+          <t>GET /api/captcha</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -3064,7 +3064,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>ROUTE-025</t>
+          <t>ROUTE-019</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -3074,7 +3074,7 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>GET /api/mbti</t>
+          <t>GET /api/compose/fragments</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -3084,7 +3084,7 @@
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>internal/handler/compose_handler.go</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
@@ -3101,17 +3101,17 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>ROUTE-026</t>
+          <t>ROUTE-020</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>GET /api/orders</t>
+          <t>GET /api/compositions/:code</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -3121,7 +3121,7 @@
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>internal/handler/order_handler.go</t>
+          <t>internal/handler/compose_handler.go</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
@@ -3138,17 +3138,17 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>ROUTE-027</t>
+          <t>ROUTE-021</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>POST /api/orders</t>
+          <t>GET /api/health</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -3158,7 +3158,7 @@
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>internal/handler/order_handler.go</t>
+          <t>cmd/server/main.go</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
@@ -3175,17 +3175,17 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>ROUTE-028</t>
+          <t>ROUTE-022</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>GET /api/orders/:id</t>
+          <t>GET /api/journeys</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -3195,7 +3195,7 @@
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>internal/handler/order_handler.go</t>
+          <t>cmd/server/main.go</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
@@ -3212,17 +3212,17 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>ROUTE-029</t>
+          <t>ROUTE-023</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>POST /api/orders/:id/pay</t>
+          <t>GET /api/journeys/:slug</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
@@ -3232,7 +3232,7 @@
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>internal/handler/order_handler.go</t>
+          <t>cmd/server/main.go</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
@@ -3249,17 +3249,17 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>ROUTE-030</t>
+          <t>ROUTE-024</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>POST /api/payments/recharge</t>
+          <t>GET /api/journeys/:slug/book</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
@@ -3269,7 +3269,7 @@
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>internal/handler/payment_handler.go</t>
+          <t>cmd/server/main.go</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
@@ -3286,7 +3286,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>ROUTE-031</t>
+          <t>ROUTE-025</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -3296,7 +3296,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>GET /api/payments/tiers</t>
+          <t>GET /api/mbti</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -3306,7 +3306,7 @@
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>internal/handler/payment_handler.go</t>
+          <t>cmd/server/main.go</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
@@ -3323,7 +3323,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>ROUTE-032</t>
+          <t>ROUTE-026</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -3333,7 +3333,7 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>GET /api/payments/transactions</t>
+          <t>GET /api/orders</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
@@ -3343,7 +3343,7 @@
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>internal/handler/payment_handler.go</t>
+          <t>internal/handler/order_handler.go</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
@@ -3360,30 +3360,252 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
+          <t>ROUTE-027</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>JWT</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>POST /api/orders</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>Route is registered</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>internal/handler/order_handler.go</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Route</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>ROUTE-028</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>JWT</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>GET /api/orders/:id</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>Route is registered</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>internal/handler/order_handler.go</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Route</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>ROUTE-029</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>JWT</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>POST /api/orders/:id/pay</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Route is registered</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>internal/handler/order_handler.go</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Route</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>ROUTE-030</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>JWT</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>POST /api/payments/recharge</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>Route is registered</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>internal/handler/payment_handler.go</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Route</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>ROUTE-031</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>GET /api/payments/tiers</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>Route is registered</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>internal/handler/payment_handler.go</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Route</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>ROUTE-032</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>JWT</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>GET /api/payments/transactions</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>Route is registered</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>internal/handler/payment_handler.go</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Route</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
           <t>ROUTE-033</t>
         </is>
       </c>
-      <c r="C83" t="inlineStr">
+      <c r="C89" t="inlineStr">
         <is>
           <t>Public</t>
         </is>
       </c>
-      <c r="D83" t="inlineStr">
+      <c r="D89" t="inlineStr">
         <is>
           <t>GET /api/tags</t>
         </is>
       </c>
-      <c r="E83" t="inlineStr">
+      <c r="E89" t="inlineStr">
         <is>
           <t>Route is registered</t>
         </is>
       </c>
-      <c r="F83" t="inlineStr">
+      <c r="F89" t="inlineStr">
         <is>
           <t>cmd/server/main.go</t>
         </is>
       </c>
-      <c r="G83" t="inlineStr">
+      <c r="G89" t="inlineStr">
         <is>
           <t>Implemented</t>
         </is>

</xml_diff>

<commit_message>
The Ticket Road (v1.6.0): rubbings, the Night Station, lanterns, the line by the door (#8)
Rubbings from every entrance, the Night Station (#/station), lanterns on tickets and journeys, the line of tickets by each door, and the safety base (reports, blocks, review queue, age bands, caps). New tables are created if missing; three columns are added; analytics_events is rebuilt once.
</commit_message>
<xml_diff>
--- a/app.xlsx
+++ b/app.xlsx
@@ -154,7 +154,7 @@
         </is>
       </c>
       <c r="B4">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -242,7 +242,7 @@
         </is>
       </c>
       <c r="E7">
-        <v>44</v>
+        <v>50</v>
       </c>
     </row>
     <row r="8">
@@ -743,7 +743,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>content_test</t>
+          <t>derive_test</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -753,7 +753,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>internal/content/content_test.go</t>
+          <t>internal/compose/derive_test.go</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -780,7 +780,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>admin_handler_test</t>
+          <t>content_test</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -790,7 +790,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>internal/handler/admin_handler_test.go</t>
+          <t>internal/content/content_test.go</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -817,7 +817,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>auth_handler_test</t>
+          <t>admin_handler_test</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -827,7 +827,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>internal/handler/auth_handler_test.go</t>
+          <t>internal/handler/admin_handler_test.go</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -854,7 +854,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>compose_handler_test</t>
+          <t>auth_handler_test</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -864,7 +864,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>internal/handler/compose_handler_test.go</t>
+          <t>internal/handler/auth_handler_test.go</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -891,7 +891,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>journey_handler_test</t>
+          <t>compose_handler_test</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -901,7 +901,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>internal/handler/journey_handler_test.go</t>
+          <t>internal/handler/compose_handler_test.go</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -928,7 +928,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>me_handler_test</t>
+          <t>journey_handler_test</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -938,7 +938,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>internal/handler/me_handler_test.go</t>
+          <t>internal/handler/journey_handler_test.go</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -965,7 +965,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>order_handler_test</t>
+          <t>me_handler_test</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -975,7 +975,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>internal/handler/order_handler_test.go</t>
+          <t>internal/handler/me_handler_test.go</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1002,7 +1002,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>payment_handler_test</t>
+          <t>order_handler_test</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1012,7 +1012,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>internal/handler/payment_handler_test.go</t>
+          <t>internal/handler/order_handler_test.go</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1039,7 +1039,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>cors_test</t>
+          <t>payment_handler_test</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1049,7 +1049,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>internal/middleware/cors_test.go</t>
+          <t>internal/handler/payment_handler_test.go</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1076,7 +1076,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>jwt_test</t>
+          <t>road_handler_test</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1086,7 +1086,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>internal/middleware/jwt_test.go</t>
+          <t>internal/handler/road_handler_test.go</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1113,7 +1113,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>request_id_test</t>
+          <t>cors_test</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1123,7 +1123,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>internal/middleware/request_id_test.go</t>
+          <t>internal/middleware/cors_test.go</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1150,7 +1150,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>journey_repo_sqlite_test</t>
+          <t>jwt_test</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1160,7 +1160,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>internal/repository/journey_repo_sqlite_test.go</t>
+          <t>internal/middleware/jwt_test.go</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1187,7 +1187,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>migrate_test</t>
+          <t>ratelimit_test</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1197,7 +1197,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>internal/repository/migrate_test.go</t>
+          <t>internal/middleware/ratelimit_test.go</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1224,7 +1224,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>order_repo_test</t>
+          <t>request_id_test</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1234,7 +1234,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>internal/repository/order_repo_test.go</t>
+          <t>internal/middleware/request_id_test.go</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1261,7 +1261,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>user_repo_test</t>
+          <t>journey_repo_sqlite_test</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1271,7 +1271,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>internal/repository/user_repo_test.go</t>
+          <t>internal/repository/journey_repo_sqlite_test.go</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1298,7 +1298,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>journey_service_test</t>
+          <t>migrate_test</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>internal/service/journey_service_test.go</t>
+          <t>internal/repository/migrate_test.go</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1335,7 +1335,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>locale_test</t>
+          <t>order_repo_test</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -1345,7 +1345,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>internal/service/locale_test.go</t>
+          <t>internal/repository/order_repo_test.go</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1372,7 +1372,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>bundle_test</t>
+          <t>user_repo_test</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1382,7 +1382,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>internal/webapp/bundle_test.go</t>
+          <t>internal/repository/user_repo_test.go</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1409,7 +1409,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>index_test</t>
+          <t>light_test</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1419,7 +1419,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>internal/webapp/index_test.go</t>
+          <t>internal/road/light/light_test.go</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -1446,7 +1446,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>share_test</t>
+          <t>road_test</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1456,7 +1456,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>internal/webapp/share_test.go</t>
+          <t>internal/road/road_test.go</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -1478,12 +1478,12 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Playwright E2E</t>
+          <t>Go unit/integration / Go 单元集成</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>a11y.spec</t>
+          <t>journey_service_test</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -1493,7 +1493,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>e2e/tests/a11y.spec.js</t>
+          <t>internal/service/journey_service_test.go</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -1515,12 +1515,12 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Playwright E2E</t>
+          <t>Go unit/integration / Go 单元集成</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>auth.spec</t>
+          <t>locale_test</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1530,7 +1530,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>e2e/tests/auth.spec.js</t>
+          <t>internal/service/locale_test.go</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -1552,12 +1552,12 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Playwright E2E</t>
+          <t>Go unit/integration / Go 单元集成</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>compose.spec</t>
+          <t>bundle_test</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -1567,7 +1567,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>e2e/tests/compose.spec.js</t>
+          <t>internal/webapp/bundle_test.go</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -1589,12 +1589,12 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Playwright E2E</t>
+          <t>Go unit/integration / Go 单元集成</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>detail.spec</t>
+          <t>index_test</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -1604,7 +1604,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>e2e/tests/detail.spec.js</t>
+          <t>internal/webapp/index_test.go</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -1626,12 +1626,12 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Playwright E2E</t>
+          <t>Go unit/integration / Go 单元集成</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>explore.spec</t>
+          <t>share_test</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -1641,7 +1641,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>e2e/tests/explore.spec.js</t>
+          <t>internal/webapp/share_test.go</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -1668,7 +1668,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>home.spec</t>
+          <t>a11y.spec</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -1678,7 +1678,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>e2e/tests/home.spec.js</t>
+          <t>e2e/tests/a11y.spec.js</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -1705,7 +1705,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>i18n.spec</t>
+          <t>auth.spec</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -1715,7 +1715,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>e2e/tests/i18n.spec.js</t>
+          <t>e2e/tests/auth.spec.js</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -1742,7 +1742,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>mobile.spec</t>
+          <t>compose.spec</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -1752,7 +1752,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>e2e/tests/mobile.spec.js</t>
+          <t>e2e/tests/compose.spec.js</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -1779,7 +1779,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>orders.spec</t>
+          <t>detail.spec</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -1789,7 +1789,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>e2e/tests/orders.spec.js</t>
+          <t>e2e/tests/detail.spec.js</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -1816,7 +1816,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>persona.spec</t>
+          <t>explore.spec</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -1826,7 +1826,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>e2e/tests/persona.spec.js</t>
+          <t>e2e/tests/explore.spec.js</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -1853,7 +1853,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>space.spec</t>
+          <t>home.spec</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -1863,7 +1863,7 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>e2e/tests/space.spec.js</t>
+          <t>e2e/tests/home.spec.js</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -1885,12 +1885,12 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Playwright support / E2E 支撑文件</t>
+          <t>Playwright E2E</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>helpers</t>
+          <t>i18n.spec</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -1900,7 +1900,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>e2e/tests/helpers.js</t>
+          <t>e2e/tests/i18n.spec.js</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -1922,12 +1922,12 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Go stress</t>
+          <t>Playwright E2E</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>stress_test</t>
+          <t>mobile.spec</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -1937,7 +1937,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>tests/stress/stress_test.go</t>
+          <t>e2e/tests/mobile.spec.js</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -1959,12 +1959,12 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>k6 load / k6 负载</t>
+          <t>Playwright E2E</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>admin-analytics-export.k6</t>
+          <t>orders.spec</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -1974,7 +1974,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>tests/load/admin-analytics-export.k6.js</t>
+          <t>e2e/tests/orders.spec.js</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -1996,12 +1996,12 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>k6 load / k6 负载</t>
+          <t>Playwright E2E</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>auth-register-login.k6</t>
+          <t>persona.spec</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -2011,7 +2011,7 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>tests/load/auth-register-login.k6.js</t>
+          <t>e2e/tests/persona.spec.js</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -2033,12 +2033,12 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>k6 load / k6 负载</t>
+          <t>Playwright E2E</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>image-static-cache.k6</t>
+          <t>road.spec</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -2048,7 +2048,7 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>tests/load/image-static-cache.k6.js</t>
+          <t>e2e/tests/road.spec.js</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -2070,12 +2070,12 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>k6 load / k6 负载</t>
+          <t>Playwright E2E</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>order-payment-audit.k6</t>
+          <t>space.spec</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -2085,7 +2085,7 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>tests/load/order-payment-audit.k6.js</t>
+          <t>e2e/tests/space.spec.js</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -2107,12 +2107,12 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>k6 load / k6 负载</t>
+          <t>Playwright support / E2E 支撑文件</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>pet-chat-analytics.k6</t>
+          <t>helpers</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -2122,7 +2122,7 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>tests/load/pet-chat-analytics.k6.js</t>
+          <t>e2e/tests/helpers.js</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -2144,12 +2144,12 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>k6 load / k6 负载</t>
+          <t>Go stress</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>public-content-flow.k6</t>
+          <t>stress_test</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -2159,7 +2159,7 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>tests/load/public-content-flow.k6.js</t>
+          <t>tests/stress/stress_test.go</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -2171,222 +2171,222 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Route</t>
+          <t>Test</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>ROUTE-001</t>
+          <t>TEST-045</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Admin</t>
+          <t>k6 load / k6 负载</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>GET /api/admin/export</t>
+          <t>admin-analytics-export.k6</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Route is registered</t>
+          <t>File exists and is part of repo</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>internal/handler/admin_handler.go</t>
+          <t>tests/load/admin-analytics-export.k6.js</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Specified</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Route</t>
+          <t>Test</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>ROUTE-002</t>
+          <t>TEST-046</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Admin</t>
+          <t>k6 load / k6 负载</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>GET /api/admin/stats</t>
+          <t>auth-register-login.k6</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Route is registered</t>
+          <t>File exists and is part of repo</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>internal/handler/admin_handler.go</t>
+          <t>tests/load/auth-register-login.k6.js</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Specified</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Route</t>
+          <t>Test</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>ROUTE-003</t>
+          <t>TEST-047</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Admin</t>
+          <t>k6 load / k6 负载</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>GET /api/admin/users</t>
+          <t>image-static-cache.k6</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Route is registered</t>
+          <t>File exists and is part of repo</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>internal/handler/admin_handler.go</t>
+          <t>tests/load/image-static-cache.k6.js</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Specified</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Route</t>
+          <t>Test</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>ROUTE-004</t>
+          <t>TEST-048</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>k6 load / k6 负载</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>POST /api/ai/chat</t>
+          <t>order-payment-audit.k6</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Route is registered</t>
+          <t>File exists and is part of repo</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>tests/load/order-payment-audit.k6.js</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Specified</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Route</t>
+          <t>Test</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>ROUTE-005</t>
+          <t>TEST-049</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>k6 load / k6 负载</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>POST /api/analytics/events</t>
+          <t>pet-chat-analytics.k6</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Route is registered</t>
+          <t>File exists and is part of repo</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>tests/load/pet-chat-analytics.k6.js</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Specified</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Route</t>
+          <t>Test</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>ROUTE-006</t>
+          <t>TEST-050</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>k6 load / k6 负载</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>POST /api/audit/client-error</t>
+          <t>public-content-flow.k6</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Route is registered</t>
+          <t>File exists and is part of repo</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>tests/load/public-content-flow.k6.js</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Specified</t>
         </is>
       </c>
     </row>
@@ -2398,17 +2398,17 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>ROUTE-007</t>
+          <t>ROUTE-001</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Admin</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>POST /api/auth/avatar</t>
+          <t>GET /api/admin/export</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -2418,7 +2418,7 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>internal/handler/admin_handler.go</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -2435,17 +2435,17 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>ROUTE-008</t>
+          <t>ROUTE-002</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Admin</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>GET /api/auth/compositions</t>
+          <t>GET /api/admin/stats</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -2455,7 +2455,7 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>internal/handler/compose_handler.go</t>
+          <t>internal/handler/admin_handler.go</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
@@ -2472,17 +2472,17 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>ROUTE-009</t>
+          <t>ROUTE-003</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Admin</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>POST /api/auth/compositions</t>
+          <t>GET /api/admin/users</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -2492,7 +2492,7 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>internal/handler/compose_handler.go</t>
+          <t>internal/handler/admin_handler.go</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
@@ -2509,17 +2509,17 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>ROUTE-010</t>
+          <t>ROUTE-004</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>DELETE /api/auth/compositions/:id</t>
+          <t>POST /api/ai/chat</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -2529,7 +2529,7 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>internal/handler/compose_handler.go</t>
+          <t>cmd/server/main.go</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -2546,7 +2546,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>ROUTE-011</t>
+          <t>ROUTE-005</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -2556,7 +2556,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>POST /api/auth/login</t>
+          <t>POST /api/analytics/events</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -2583,17 +2583,17 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>ROUTE-012</t>
+          <t>ROUTE-006</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>PUT /api/auth/mbti</t>
+          <t>POST /api/audit/client-error</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -2603,7 +2603,7 @@
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>internal/handler/me_handler.go</t>
+          <t>cmd/server/main.go</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
@@ -2620,7 +2620,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>ROUTE-013</t>
+          <t>ROUTE-007</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -2630,7 +2630,7 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>GET /api/auth/me</t>
+          <t>POST /api/auth/avatar</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -2657,17 +2657,17 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>ROUTE-014</t>
+          <t>ROUTE-008</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>JWT</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>POST /api/auth/register</t>
+          <t>GET /api/auth/compositions</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -2677,7 +2677,7 @@
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>internal/handler/compose_handler.go</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -2694,7 +2694,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>ROUTE-015</t>
+          <t>ROUTE-009</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -2704,7 +2704,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>GET /api/auth/saved</t>
+          <t>POST /api/auth/compositions</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -2714,7 +2714,7 @@
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>internal/handler/me_handler.go</t>
+          <t>internal/handler/compose_handler.go</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
@@ -2731,7 +2731,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>ROUTE-016</t>
+          <t>ROUTE-010</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -2741,7 +2741,7 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>DELETE /api/auth/saved/:slug</t>
+          <t>DELETE /api/auth/compositions/:id</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -2751,7 +2751,7 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>internal/handler/me_handler.go</t>
+          <t>internal/handler/compose_handler.go</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
@@ -2768,17 +2768,17 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>ROUTE-017</t>
+          <t>ROUTE-011</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>PUT /api/auth/saved/:slug</t>
+          <t>POST /api/auth/login</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -2788,7 +2788,7 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>internal/handler/me_handler.go</t>
+          <t>cmd/server/main.go</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -2805,17 +2805,17 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>ROUTE-018</t>
+          <t>ROUTE-012</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>JWT</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>GET /api/captcha</t>
+          <t>PUT /api/auth/mbti</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -2825,7 +2825,7 @@
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>internal/handler/me_handler.go</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
@@ -2842,17 +2842,17 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>ROUTE-019</t>
+          <t>ROUTE-013</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>JWT</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>GET /api/compose/fragments</t>
+          <t>GET /api/auth/me</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -2862,7 +2862,7 @@
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>internal/handler/compose_handler.go</t>
+          <t>cmd/server/main.go</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
@@ -2879,7 +2879,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>ROUTE-020</t>
+          <t>ROUTE-014</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -2889,7 +2889,7 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>GET /api/compositions/:code</t>
+          <t>POST /api/auth/register</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -2899,7 +2899,7 @@
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>internal/handler/compose_handler.go</t>
+          <t>cmd/server/main.go</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
@@ -2916,17 +2916,17 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>ROUTE-021</t>
+          <t>ROUTE-015</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>JWT</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>GET /api/health</t>
+          <t>GET /api/auth/saved</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -2936,7 +2936,7 @@
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>internal/handler/me_handler.go</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
@@ -2953,17 +2953,17 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>ROUTE-022</t>
+          <t>ROUTE-016</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>JWT</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>GET /api/journeys</t>
+          <t>DELETE /api/auth/saved/:slug</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
@@ -2973,7 +2973,7 @@
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>internal/handler/me_handler.go</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
@@ -2990,17 +2990,17 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>ROUTE-023</t>
+          <t>ROUTE-017</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>JWT</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>GET /api/journeys/:slug</t>
+          <t>PUT /api/auth/saved/:slug</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -3010,7 +3010,7 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>internal/handler/me_handler.go</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>ROUTE-024</t>
+          <t>ROUTE-018</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -3037,7 +3037,7 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>GET /api/journeys/:slug/book</t>
+          <t>GET /api/captcha</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -3064,7 +3064,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>ROUTE-025</t>
+          <t>ROUTE-019</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -3074,7 +3074,7 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>GET /api/mbti</t>
+          <t>GET /api/compose/fragments</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -3084,7 +3084,7 @@
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>internal/handler/compose_handler.go</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
@@ -3101,17 +3101,17 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>ROUTE-026</t>
+          <t>ROUTE-020</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>GET /api/orders</t>
+          <t>GET /api/compositions/:code</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -3121,7 +3121,7 @@
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>internal/handler/order_handler.go</t>
+          <t>internal/handler/compose_handler.go</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
@@ -3138,17 +3138,17 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>ROUTE-027</t>
+          <t>ROUTE-021</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>POST /api/orders</t>
+          <t>GET /api/health</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -3158,7 +3158,7 @@
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>internal/handler/order_handler.go</t>
+          <t>cmd/server/main.go</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
@@ -3175,17 +3175,17 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>ROUTE-028</t>
+          <t>ROUTE-022</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>GET /api/orders/:id</t>
+          <t>GET /api/journeys</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -3195,7 +3195,7 @@
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>internal/handler/order_handler.go</t>
+          <t>cmd/server/main.go</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
@@ -3212,17 +3212,17 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>ROUTE-029</t>
+          <t>ROUTE-023</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>POST /api/orders/:id/pay</t>
+          <t>GET /api/journeys/:slug</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
@@ -3232,7 +3232,7 @@
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>internal/handler/order_handler.go</t>
+          <t>cmd/server/main.go</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
@@ -3249,17 +3249,17 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>ROUTE-030</t>
+          <t>ROUTE-024</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>POST /api/payments/recharge</t>
+          <t>GET /api/journeys/:slug/book</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
@@ -3269,7 +3269,7 @@
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>internal/handler/payment_handler.go</t>
+          <t>cmd/server/main.go</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
@@ -3286,7 +3286,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>ROUTE-031</t>
+          <t>ROUTE-025</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -3296,7 +3296,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>GET /api/payments/tiers</t>
+          <t>GET /api/mbti</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -3306,7 +3306,7 @@
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>internal/handler/payment_handler.go</t>
+          <t>cmd/server/main.go</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
@@ -3323,7 +3323,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>ROUTE-032</t>
+          <t>ROUTE-026</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -3333,7 +3333,7 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>GET /api/payments/transactions</t>
+          <t>GET /api/orders</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
@@ -3343,7 +3343,7 @@
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>internal/handler/payment_handler.go</t>
+          <t>internal/handler/order_handler.go</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
@@ -3360,30 +3360,252 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
+          <t>ROUTE-027</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>JWT</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>POST /api/orders</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>Route is registered</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>internal/handler/order_handler.go</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Route</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>ROUTE-028</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>JWT</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>GET /api/orders/:id</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>Route is registered</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>internal/handler/order_handler.go</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Route</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>ROUTE-029</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>JWT</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>POST /api/orders/:id/pay</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Route is registered</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>internal/handler/order_handler.go</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Route</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>ROUTE-030</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>JWT</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>POST /api/payments/recharge</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>Route is registered</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>internal/handler/payment_handler.go</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Route</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>ROUTE-031</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>GET /api/payments/tiers</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>Route is registered</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>internal/handler/payment_handler.go</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Route</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>ROUTE-032</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>JWT</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>GET /api/payments/transactions</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>Route is registered</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>internal/handler/payment_handler.go</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Route</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
           <t>ROUTE-033</t>
         </is>
       </c>
-      <c r="C83" t="inlineStr">
+      <c r="C89" t="inlineStr">
         <is>
           <t>Public</t>
         </is>
       </c>
-      <c r="D83" t="inlineStr">
+      <c r="D89" t="inlineStr">
         <is>
           <t>GET /api/tags</t>
         </is>
       </c>
-      <c r="E83" t="inlineStr">
+      <c r="E89" t="inlineStr">
         <is>
           <t>Route is registered</t>
         </is>
       </c>
-      <c r="F83" t="inlineStr">
+      <c r="F89" t="inlineStr">
         <is>
           <t>cmd/server/main.go</t>
         </is>
       </c>
-      <c r="G83" t="inlineStr">
+      <c r="G89" t="inlineStr">
         <is>
           <t>Implemented</t>
         </is>

</xml_diff>

<commit_message>
fonts: self-hosted story serif, sliced by page
- Noto Serif SC (Chinese, 400/700) and Newsreader (English, 400/700), both SIL OFL 1.1, subset to
  the characters the site's own text uses and served as WOFF2 from /static/assets/fonts.
- Chinese is cut into unicode-range slices by the pages that use each character, so the home
  page loads about 56 KB and a journey 110-140 KB; English loads 28 KB.
- font-display: swap with fixed vertical metrics and a size-adjusted Georgia stand-in, so a swap
  does not move lines; the home page preloads its title's slices.
- Characters outside the subset fall to a local Song face, then the UI sans.
- The 11px door labels on the home page use the UI sans, which reads better at that size.
- scripts/fonts (measure + build), docs/content/FONTS.md with sources and licences, UT-WEB-007,
  E2E-FONT-001/002.
</commit_message>
<xml_diff>
--- a/app.xlsx
+++ b/app.xlsx
@@ -154,7 +154,7 @@
         </is>
       </c>
       <c r="B4">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -242,7 +242,7 @@
         </is>
       </c>
       <c r="E7">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="8">
@@ -1594,7 +1594,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>index_test</t>
+          <t>fonts_test</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -1604,7 +1604,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>internal/webapp/index_test.go</t>
+          <t>internal/webapp/fonts_test.go</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -1631,7 +1631,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>share_test</t>
+          <t>index_test</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -1641,7 +1641,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>internal/webapp/share_test.go</t>
+          <t>internal/webapp/index_test.go</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -1663,12 +1663,12 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Playwright E2E</t>
+          <t>Go unit/integration / Go 单元集成</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>a11y.spec</t>
+          <t>share_test</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -1678,7 +1678,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>e2e/tests/a11y.spec.js</t>
+          <t>internal/webapp/share_test.go</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -1705,7 +1705,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>auth.spec</t>
+          <t>a11y.spec</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -1715,7 +1715,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>e2e/tests/auth.spec.js</t>
+          <t>e2e/tests/a11y.spec.js</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -1742,7 +1742,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>compose.spec</t>
+          <t>auth.spec</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -1752,7 +1752,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>e2e/tests/compose.spec.js</t>
+          <t>e2e/tests/auth.spec.js</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -1779,7 +1779,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>detail.spec</t>
+          <t>compose.spec</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -1789,7 +1789,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>e2e/tests/detail.spec.js</t>
+          <t>e2e/tests/compose.spec.js</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -1816,7 +1816,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>explore.spec</t>
+          <t>detail.spec</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -1826,7 +1826,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>e2e/tests/explore.spec.js</t>
+          <t>e2e/tests/detail.spec.js</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -1853,7 +1853,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>home.spec</t>
+          <t>explore.spec</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -1863,7 +1863,7 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>e2e/tests/home.spec.js</t>
+          <t>e2e/tests/explore.spec.js</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -1890,7 +1890,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>i18n.spec</t>
+          <t>fonts.spec</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -1900,7 +1900,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>e2e/tests/i18n.spec.js</t>
+          <t>e2e/tests/fonts.spec.js</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -1927,7 +1927,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>mobile.spec</t>
+          <t>home.spec</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -1937,7 +1937,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>e2e/tests/mobile.spec.js</t>
+          <t>e2e/tests/home.spec.js</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -1964,7 +1964,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>orders.spec</t>
+          <t>i18n.spec</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -1974,7 +1974,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>e2e/tests/orders.spec.js</t>
+          <t>e2e/tests/i18n.spec.js</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -2001,7 +2001,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>persona.spec</t>
+          <t>mobile.spec</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -2011,7 +2011,7 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>e2e/tests/persona.spec.js</t>
+          <t>e2e/tests/mobile.spec.js</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -2038,7 +2038,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>road.spec</t>
+          <t>orders.spec</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -2048,7 +2048,7 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>e2e/tests/road.spec.js</t>
+          <t>e2e/tests/orders.spec.js</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -2075,7 +2075,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>space.spec</t>
+          <t>persona.spec</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -2085,7 +2085,7 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>e2e/tests/space.spec.js</t>
+          <t>e2e/tests/persona.spec.js</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -2107,12 +2107,12 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Playwright support / E2E 支撑文件</t>
+          <t>Playwright E2E</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>helpers</t>
+          <t>road.spec</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -2122,7 +2122,7 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>e2e/tests/helpers.js</t>
+          <t>e2e/tests/road.spec.js</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -2144,12 +2144,12 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Go stress</t>
+          <t>Playwright E2E</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>stress_test</t>
+          <t>space.spec</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -2159,7 +2159,7 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>tests/stress/stress_test.go</t>
+          <t>e2e/tests/space.spec.js</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -2181,12 +2181,12 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>k6 load / k6 负载</t>
+          <t>Playwright support / E2E 支撑文件</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>admin-analytics-export.k6</t>
+          <t>helpers</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -2196,7 +2196,7 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>tests/load/admin-analytics-export.k6.js</t>
+          <t>e2e/tests/helpers.js</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -2218,12 +2218,12 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>k6 load / k6 负载</t>
+          <t>Go stress</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>auth-register-login.k6</t>
+          <t>stress_test</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -2233,7 +2233,7 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>tests/load/auth-register-login.k6.js</t>
+          <t>tests/stress/stress_test.go</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -2260,7 +2260,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>image-static-cache.k6</t>
+          <t>admin-analytics-export.k6</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -2270,7 +2270,7 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>tests/load/image-static-cache.k6.js</t>
+          <t>tests/load/admin-analytics-export.k6.js</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -2297,7 +2297,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>order-payment-audit.k6</t>
+          <t>auth-register-login.k6</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -2307,7 +2307,7 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>tests/load/order-payment-audit.k6.js</t>
+          <t>tests/load/auth-register-login.k6.js</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -2334,7 +2334,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>pet-chat-analytics.k6</t>
+          <t>image-static-cache.k6</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -2344,7 +2344,7 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>tests/load/pet-chat-analytics.k6.js</t>
+          <t>tests/load/image-static-cache.k6.js</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -2371,7 +2371,7 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>public-content-flow.k6</t>
+          <t>order-payment-audit.k6</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -2381,7 +2381,7 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>tests/load/public-content-flow.k6.js</t>
+          <t>tests/load/order-payment-audit.k6.js</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -2393,74 +2393,74 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Route</t>
+          <t>Test</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>ROUTE-001</t>
+          <t>TEST-051</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Admin</t>
+          <t>k6 load / k6 负载</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>GET /api/admin/export</t>
+          <t>pet-chat-analytics.k6</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Route is registered</t>
+          <t>File exists and is part of repo</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>internal/handler/admin_handler.go</t>
+          <t>tests/load/pet-chat-analytics.k6.js</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Specified</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Route</t>
+          <t>Test</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>ROUTE-002</t>
+          <t>TEST-052</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Admin</t>
+          <t>k6 load / k6 负载</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>GET /api/admin/stats</t>
+          <t>public-content-flow.k6</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Route is registered</t>
+          <t>File exists and is part of repo</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>internal/handler/admin_handler.go</t>
+          <t>tests/load/public-content-flow.k6.js</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Specified</t>
         </is>
       </c>
     </row>
@@ -2472,7 +2472,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>ROUTE-003</t>
+          <t>ROUTE-001</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -2482,7 +2482,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>GET /api/admin/users</t>
+          <t>GET /api/admin/export</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -2509,17 +2509,17 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>ROUTE-004</t>
+          <t>ROUTE-002</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>Admin</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>POST /api/ai/chat</t>
+          <t>GET /api/admin/stats</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -2529,7 +2529,7 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>internal/handler/admin_handler.go</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -2546,17 +2546,17 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>ROUTE-005</t>
+          <t>ROUTE-003</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>Admin</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>POST /api/analytics/events</t>
+          <t>GET /api/admin/users</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -2566,7 +2566,7 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>internal/handler/admin_handler.go</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -2583,7 +2583,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>ROUTE-006</t>
+          <t>ROUTE-004</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -2593,7 +2593,7 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>POST /api/audit/client-error</t>
+          <t>POST /api/ai/chat</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -2620,17 +2620,17 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>ROUTE-007</t>
+          <t>ROUTE-005</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>POST /api/auth/avatar</t>
+          <t>POST /api/analytics/events</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -2657,17 +2657,17 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>ROUTE-008</t>
+          <t>ROUTE-006</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>GET /api/auth/compositions</t>
+          <t>POST /api/audit/client-error</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -2677,7 +2677,7 @@
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>internal/handler/compose_handler.go</t>
+          <t>cmd/server/main.go</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -2694,7 +2694,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>ROUTE-009</t>
+          <t>ROUTE-007</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -2704,7 +2704,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>POST /api/auth/compositions</t>
+          <t>POST /api/auth/avatar</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -2714,7 +2714,7 @@
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>internal/handler/compose_handler.go</t>
+          <t>cmd/server/main.go</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
@@ -2731,7 +2731,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>ROUTE-010</t>
+          <t>ROUTE-008</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -2741,7 +2741,7 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>DELETE /api/auth/compositions/:id</t>
+          <t>GET /api/auth/compositions</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -2768,17 +2768,17 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>ROUTE-011</t>
+          <t>ROUTE-009</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>JWT</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>POST /api/auth/login</t>
+          <t>POST /api/auth/compositions</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -2788,7 +2788,7 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>internal/handler/compose_handler.go</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -2805,7 +2805,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>ROUTE-012</t>
+          <t>ROUTE-010</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -2815,7 +2815,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>PUT /api/auth/mbti</t>
+          <t>DELETE /api/auth/compositions/:id</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -2825,7 +2825,7 @@
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>internal/handler/me_handler.go</t>
+          <t>internal/handler/compose_handler.go</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
@@ -2842,17 +2842,17 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>ROUTE-013</t>
+          <t>ROUTE-011</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>GET /api/auth/me</t>
+          <t>POST /api/auth/login</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -2879,17 +2879,17 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>ROUTE-014</t>
+          <t>ROUTE-012</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>JWT</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>POST /api/auth/register</t>
+          <t>PUT /api/auth/mbti</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -2899,7 +2899,7 @@
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>internal/handler/me_handler.go</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
@@ -2916,7 +2916,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>ROUTE-015</t>
+          <t>ROUTE-013</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -2926,7 +2926,7 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>GET /api/auth/saved</t>
+          <t>GET /api/auth/me</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -2936,7 +2936,7 @@
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>internal/handler/me_handler.go</t>
+          <t>cmd/server/main.go</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
@@ -2953,17 +2953,17 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>ROUTE-016</t>
+          <t>ROUTE-014</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>DELETE /api/auth/saved/:slug</t>
+          <t>POST /api/auth/register</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
@@ -2973,7 +2973,7 @@
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>internal/handler/me_handler.go</t>
+          <t>cmd/server/main.go</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
@@ -2990,7 +2990,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>ROUTE-017</t>
+          <t>ROUTE-015</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -3000,7 +3000,7 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>PUT /api/auth/saved/:slug</t>
+          <t>GET /api/auth/saved</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -3027,17 +3027,17 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>ROUTE-018</t>
+          <t>ROUTE-016</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>JWT</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>GET /api/captcha</t>
+          <t>DELETE /api/auth/saved/:slug</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -3047,7 +3047,7 @@
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>internal/handler/me_handler.go</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
@@ -3064,17 +3064,17 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>ROUTE-019</t>
+          <t>ROUTE-017</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>JWT</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>GET /api/compose/fragments</t>
+          <t>PUT /api/auth/saved/:slug</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -3084,7 +3084,7 @@
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>internal/handler/compose_handler.go</t>
+          <t>internal/handler/me_handler.go</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
@@ -3101,7 +3101,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>ROUTE-020</t>
+          <t>ROUTE-018</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -3111,7 +3111,7 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>GET /api/compositions/:code</t>
+          <t>GET /api/captcha</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -3121,7 +3121,7 @@
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>internal/handler/compose_handler.go</t>
+          <t>cmd/server/main.go</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
@@ -3138,7 +3138,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>ROUTE-021</t>
+          <t>ROUTE-019</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -3148,7 +3148,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>GET /api/health</t>
+          <t>GET /api/compose/fragments</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -3158,7 +3158,7 @@
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>internal/handler/compose_handler.go</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
@@ -3175,7 +3175,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>ROUTE-022</t>
+          <t>ROUTE-020</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -3185,7 +3185,7 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>GET /api/journeys</t>
+          <t>GET /api/compositions/:code</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -3195,7 +3195,7 @@
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>internal/handler/compose_handler.go</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
@@ -3212,7 +3212,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>ROUTE-023</t>
+          <t>ROUTE-021</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -3222,7 +3222,7 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>GET /api/journeys/:slug</t>
+          <t>GET /api/health</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
@@ -3249,7 +3249,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>ROUTE-024</t>
+          <t>ROUTE-022</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -3259,7 +3259,7 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>GET /api/journeys/:slug/book</t>
+          <t>GET /api/journeys</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
@@ -3286,7 +3286,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>ROUTE-025</t>
+          <t>ROUTE-023</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -3296,7 +3296,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>GET /api/mbti</t>
+          <t>GET /api/journeys/:slug</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -3323,17 +3323,17 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>ROUTE-026</t>
+          <t>ROUTE-024</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>GET /api/orders</t>
+          <t>GET /api/journeys/:slug/book</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
@@ -3343,7 +3343,7 @@
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>internal/handler/order_handler.go</t>
+          <t>cmd/server/main.go</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
@@ -3360,17 +3360,17 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>ROUTE-027</t>
+          <t>ROUTE-025</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>POST /api/orders</t>
+          <t>GET /api/mbti</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -3380,7 +3380,7 @@
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>internal/handler/order_handler.go</t>
+          <t>cmd/server/main.go</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
@@ -3397,7 +3397,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>ROUTE-028</t>
+          <t>ROUTE-026</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -3407,7 +3407,7 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>GET /api/orders/:id</t>
+          <t>GET /api/orders</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
@@ -3434,7 +3434,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>ROUTE-029</t>
+          <t>ROUTE-027</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -3444,7 +3444,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>POST /api/orders/:id/pay</t>
+          <t>POST /api/orders</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -3471,7 +3471,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>ROUTE-030</t>
+          <t>ROUTE-028</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -3481,7 +3481,7 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>POST /api/payments/recharge</t>
+          <t>GET /api/orders/:id</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
@@ -3491,7 +3491,7 @@
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>internal/handler/payment_handler.go</t>
+          <t>internal/handler/order_handler.go</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
@@ -3508,17 +3508,17 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>ROUTE-031</t>
+          <t>ROUTE-029</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>JWT</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>GET /api/payments/tiers</t>
+          <t>POST /api/orders/:id/pay</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
@@ -3528,7 +3528,7 @@
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>internal/handler/payment_handler.go</t>
+          <t>internal/handler/order_handler.go</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
@@ -3545,7 +3545,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>ROUTE-032</t>
+          <t>ROUTE-030</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -3555,7 +3555,7 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>GET /api/payments/transactions</t>
+          <t>POST /api/payments/recharge</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
@@ -3582,30 +3582,104 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
+          <t>ROUTE-031</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>GET /api/payments/tiers</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Route is registered</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>internal/handler/payment_handler.go</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Route</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>ROUTE-032</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>JWT</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>GET /api/payments/transactions</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>Route is registered</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>internal/handler/payment_handler.go</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Route</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
           <t>ROUTE-033</t>
         </is>
       </c>
-      <c r="C89" t="inlineStr">
+      <c r="C91" t="inlineStr">
         <is>
           <t>Public</t>
         </is>
       </c>
-      <c r="D89" t="inlineStr">
+      <c r="D91" t="inlineStr">
         <is>
           <t>GET /api/tags</t>
         </is>
       </c>
-      <c r="E89" t="inlineStr">
+      <c r="E91" t="inlineStr">
         <is>
           <t>Route is registered</t>
         </is>
       </c>
-      <c r="F89" t="inlineStr">
+      <c r="F91" t="inlineStr">
         <is>
           <t>cmd/server/main.go</t>
         </is>
       </c>
-      <c r="G89" t="inlineStr">
+      <c r="G91" t="inlineStr">
         <is>
           <t>Implemented</t>
         </is>

</xml_diff>

<commit_message>
i18n: door plates in English, a readable closing column, a text layout check
- Door tiles: the number and the name are two rows in the flow, so a name never covers the number;
  no word is split, Chinese names wrap to two lines at most. English tiles carry the number as a
  plate; the name is in the card beside it (hover, focus, tap) and in the door's label.
- Closing section in English: the credit sits under the quote, the side column keeps a readable
  width, and the arrow follows the last word; it stacks below 960px.
- e2e/tests/text-layout.js finds split words, text drawn over text and columns squeezed to a word
  per line; E2E-LAYOUT-001/002 run it on home, explore, a journey and the station (en at 1440, 768
  and 375; zh at 1440 and 375). A sweep of 13 pages at four widths in both languages finds nothing.
</commit_message>
<xml_diff>
--- a/app.xlsx
+++ b/app.xlsx
@@ -154,7 +154,7 @@
         </is>
       </c>
       <c r="B4">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -242,7 +242,7 @@
         </is>
       </c>
       <c r="E7">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
     <row r="8">
@@ -2001,7 +2001,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>mobile.spec</t>
+          <t>layout.spec</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -2011,7 +2011,7 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>e2e/tests/mobile.spec.js</t>
+          <t>e2e/tests/layout.spec.js</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -2038,7 +2038,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>orders.spec</t>
+          <t>mobile.spec</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -2048,7 +2048,7 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>e2e/tests/orders.spec.js</t>
+          <t>e2e/tests/mobile.spec.js</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -2075,7 +2075,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>persona.spec</t>
+          <t>orders.spec</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -2085,7 +2085,7 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>e2e/tests/persona.spec.js</t>
+          <t>e2e/tests/orders.spec.js</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -2112,7 +2112,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>road.spec</t>
+          <t>persona.spec</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -2122,7 +2122,7 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>e2e/tests/road.spec.js</t>
+          <t>e2e/tests/persona.spec.js</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -2149,7 +2149,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>space.spec</t>
+          <t>road.spec</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -2159,7 +2159,7 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>e2e/tests/space.spec.js</t>
+          <t>e2e/tests/road.spec.js</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -2181,12 +2181,12 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Playwright support / E2E 支撑文件</t>
+          <t>Playwright E2E</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>helpers</t>
+          <t>space.spec</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -2196,7 +2196,7 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>e2e/tests/helpers.js</t>
+          <t>e2e/tests/space.spec.js</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -2218,12 +2218,12 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Go stress</t>
+          <t>Playwright support / E2E 支撑文件</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>stress_test</t>
+          <t>helpers</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -2233,7 +2233,7 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>tests/stress/stress_test.go</t>
+          <t>e2e/tests/helpers.js</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -2255,12 +2255,12 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>k6 load / k6 负载</t>
+          <t>Playwright support / E2E 支撑文件</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>admin-analytics-export.k6</t>
+          <t>text-layout</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -2270,7 +2270,7 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>tests/load/admin-analytics-export.k6.js</t>
+          <t>e2e/tests/text-layout.js</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -2292,12 +2292,12 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>k6 load / k6 负载</t>
+          <t>Go stress</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>auth-register-login.k6</t>
+          <t>stress_test</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -2307,7 +2307,7 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>tests/load/auth-register-login.k6.js</t>
+          <t>tests/stress/stress_test.go</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -2334,7 +2334,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>image-static-cache.k6</t>
+          <t>admin-analytics-export.k6</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -2344,7 +2344,7 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>tests/load/image-static-cache.k6.js</t>
+          <t>tests/load/admin-analytics-export.k6.js</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -2371,7 +2371,7 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>order-payment-audit.k6</t>
+          <t>auth-register-login.k6</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -2381,7 +2381,7 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>tests/load/order-payment-audit.k6.js</t>
+          <t>tests/load/auth-register-login.k6.js</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -2408,7 +2408,7 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>pet-chat-analytics.k6</t>
+          <t>image-static-cache.k6</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -2418,7 +2418,7 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>tests/load/pet-chat-analytics.k6.js</t>
+          <t>tests/load/image-static-cache.k6.js</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -2445,7 +2445,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>public-content-flow.k6</t>
+          <t>order-payment-audit.k6</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -2455,7 +2455,7 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>tests/load/public-content-flow.k6.js</t>
+          <t>tests/load/order-payment-audit.k6.js</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
@@ -2467,74 +2467,74 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Route</t>
+          <t>Test</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>ROUTE-001</t>
+          <t>TEST-053</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Admin</t>
+          <t>k6 load / k6 负载</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>GET /api/admin/export</t>
+          <t>pet-chat-analytics.k6</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Route is registered</t>
+          <t>File exists and is part of repo</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>internal/handler/admin_handler.go</t>
+          <t>tests/load/pet-chat-analytics.k6.js</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Specified</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Route</t>
+          <t>Test</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>ROUTE-002</t>
+          <t>TEST-054</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Admin</t>
+          <t>k6 load / k6 负载</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>GET /api/admin/stats</t>
+          <t>public-content-flow.k6</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Route is registered</t>
+          <t>File exists and is part of repo</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>internal/handler/admin_handler.go</t>
+          <t>tests/load/public-content-flow.k6.js</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Specified</t>
         </is>
       </c>
     </row>
@@ -2546,7 +2546,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>ROUTE-003</t>
+          <t>ROUTE-001</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -2556,7 +2556,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>GET /api/admin/users</t>
+          <t>GET /api/admin/export</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -2583,17 +2583,17 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>ROUTE-004</t>
+          <t>ROUTE-002</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>Admin</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>POST /api/ai/chat</t>
+          <t>GET /api/admin/stats</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -2603,7 +2603,7 @@
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>internal/handler/admin_handler.go</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
@@ -2620,17 +2620,17 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>ROUTE-005</t>
+          <t>ROUTE-003</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>Admin</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>POST /api/analytics/events</t>
+          <t>GET /api/admin/users</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -2640,7 +2640,7 @@
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>internal/handler/admin_handler.go</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
@@ -2657,7 +2657,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>ROUTE-006</t>
+          <t>ROUTE-004</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -2667,7 +2667,7 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>POST /api/audit/client-error</t>
+          <t>POST /api/ai/chat</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -2694,17 +2694,17 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>ROUTE-007</t>
+          <t>ROUTE-005</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>POST /api/auth/avatar</t>
+          <t>POST /api/analytics/events</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -2731,17 +2731,17 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>ROUTE-008</t>
+          <t>ROUTE-006</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>GET /api/auth/compositions</t>
+          <t>POST /api/audit/client-error</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -2751,7 +2751,7 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>internal/handler/compose_handler.go</t>
+          <t>cmd/server/main.go</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
@@ -2768,7 +2768,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>ROUTE-009</t>
+          <t>ROUTE-007</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -2778,7 +2778,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>POST /api/auth/compositions</t>
+          <t>POST /api/auth/avatar</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -2788,7 +2788,7 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>internal/handler/compose_handler.go</t>
+          <t>cmd/server/main.go</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -2805,7 +2805,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>ROUTE-010</t>
+          <t>ROUTE-008</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -2815,7 +2815,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>DELETE /api/auth/compositions/:id</t>
+          <t>GET /api/auth/compositions</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -2842,17 +2842,17 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>ROUTE-011</t>
+          <t>ROUTE-009</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>JWT</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>POST /api/auth/login</t>
+          <t>POST /api/auth/compositions</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -2862,7 +2862,7 @@
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>internal/handler/compose_handler.go</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
@@ -2879,7 +2879,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>ROUTE-012</t>
+          <t>ROUTE-010</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -2889,7 +2889,7 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>PUT /api/auth/mbti</t>
+          <t>DELETE /api/auth/compositions/:id</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -2899,7 +2899,7 @@
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>internal/handler/me_handler.go</t>
+          <t>internal/handler/compose_handler.go</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
@@ -2916,17 +2916,17 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>ROUTE-013</t>
+          <t>ROUTE-011</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>GET /api/auth/me</t>
+          <t>POST /api/auth/login</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -2953,17 +2953,17 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>ROUTE-014</t>
+          <t>ROUTE-012</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>JWT</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>POST /api/auth/register</t>
+          <t>PUT /api/auth/mbti</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
@@ -2973,7 +2973,7 @@
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>internal/handler/me_handler.go</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
@@ -2990,7 +2990,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>ROUTE-015</t>
+          <t>ROUTE-013</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -3000,7 +3000,7 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>GET /api/auth/saved</t>
+          <t>GET /api/auth/me</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -3010,7 +3010,7 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>internal/handler/me_handler.go</t>
+          <t>cmd/server/main.go</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -3027,17 +3027,17 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>ROUTE-016</t>
+          <t>ROUTE-014</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>DELETE /api/auth/saved/:slug</t>
+          <t>POST /api/auth/register</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -3047,7 +3047,7 @@
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>internal/handler/me_handler.go</t>
+          <t>cmd/server/main.go</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
@@ -3064,7 +3064,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>ROUTE-017</t>
+          <t>ROUTE-015</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -3074,7 +3074,7 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>PUT /api/auth/saved/:slug</t>
+          <t>GET /api/auth/saved</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -3101,17 +3101,17 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>ROUTE-018</t>
+          <t>ROUTE-016</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>JWT</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>GET /api/captcha</t>
+          <t>DELETE /api/auth/saved/:slug</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -3121,7 +3121,7 @@
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>internal/handler/me_handler.go</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
@@ -3138,17 +3138,17 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>ROUTE-019</t>
+          <t>ROUTE-017</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>JWT</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>GET /api/compose/fragments</t>
+          <t>PUT /api/auth/saved/:slug</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -3158,7 +3158,7 @@
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>internal/handler/compose_handler.go</t>
+          <t>internal/handler/me_handler.go</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
@@ -3175,7 +3175,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>ROUTE-020</t>
+          <t>ROUTE-018</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -3185,7 +3185,7 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>GET /api/compositions/:code</t>
+          <t>GET /api/captcha</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -3195,7 +3195,7 @@
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>internal/handler/compose_handler.go</t>
+          <t>cmd/server/main.go</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
@@ -3212,7 +3212,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>ROUTE-021</t>
+          <t>ROUTE-019</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -3222,7 +3222,7 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>GET /api/health</t>
+          <t>GET /api/compose/fragments</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
@@ -3232,7 +3232,7 @@
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>internal/handler/compose_handler.go</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
@@ -3249,7 +3249,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>ROUTE-022</t>
+          <t>ROUTE-020</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -3259,7 +3259,7 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>GET /api/journeys</t>
+          <t>GET /api/compositions/:code</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
@@ -3269,7 +3269,7 @@
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>cmd/server/main.go</t>
+          <t>internal/handler/compose_handler.go</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
@@ -3286,7 +3286,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>ROUTE-023</t>
+          <t>ROUTE-021</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -3296,7 +3296,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>GET /api/journeys/:slug</t>
+          <t>GET /api/health</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -3323,7 +3323,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>ROUTE-024</t>
+          <t>ROUTE-022</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -3333,7 +3333,7 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>GET /api/journeys/:slug/book</t>
+          <t>GET /api/journeys</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
@@ -3360,7 +3360,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>ROUTE-025</t>
+          <t>ROUTE-023</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -3370,7 +3370,7 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>GET /api/mbti</t>
+          <t>GET /api/journeys/:slug</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -3397,17 +3397,17 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>ROUTE-026</t>
+          <t>ROUTE-024</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>GET /api/orders</t>
+          <t>GET /api/journeys/:slug/book</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
@@ -3417,7 +3417,7 @@
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>internal/handler/order_handler.go</t>
+          <t>cmd/server/main.go</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
@@ -3434,17 +3434,17 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>ROUTE-027</t>
+          <t>ROUTE-025</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>JWT</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>POST /api/orders</t>
+          <t>GET /api/mbti</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -3454,7 +3454,7 @@
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>internal/handler/order_handler.go</t>
+          <t>cmd/server/main.go</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
@@ -3471,7 +3471,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>ROUTE-028</t>
+          <t>ROUTE-026</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -3481,7 +3481,7 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>GET /api/orders/:id</t>
+          <t>GET /api/orders</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
@@ -3508,7 +3508,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>ROUTE-029</t>
+          <t>ROUTE-027</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -3518,7 +3518,7 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>POST /api/orders/:id/pay</t>
+          <t>POST /api/orders</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
@@ -3545,7 +3545,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>ROUTE-030</t>
+          <t>ROUTE-028</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -3555,7 +3555,7 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>POST /api/payments/recharge</t>
+          <t>GET /api/orders/:id</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
@@ -3565,7 +3565,7 @@
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>internal/handler/payment_handler.go</t>
+          <t>internal/handler/order_handler.go</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
@@ -3582,17 +3582,17 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>ROUTE-031</t>
+          <t>ROUTE-029</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>JWT</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>GET /api/payments/tiers</t>
+          <t>POST /api/orders/:id/pay</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
@@ -3602,7 +3602,7 @@
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>internal/handler/payment_handler.go</t>
+          <t>internal/handler/order_handler.go</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
@@ -3619,7 +3619,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>ROUTE-032</t>
+          <t>ROUTE-030</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -3629,7 +3629,7 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>GET /api/payments/transactions</t>
+          <t>POST /api/payments/recharge</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
@@ -3656,30 +3656,104 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
+          <t>ROUTE-031</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>GET /api/payments/tiers</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>Route is registered</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>internal/handler/payment_handler.go</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Route</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>ROUTE-032</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>JWT</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>GET /api/payments/transactions</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>Route is registered</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>internal/handler/payment_handler.go</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Route</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
           <t>ROUTE-033</t>
         </is>
       </c>
-      <c r="C91" t="inlineStr">
+      <c r="C93" t="inlineStr">
         <is>
           <t>Public</t>
         </is>
       </c>
-      <c r="D91" t="inlineStr">
+      <c r="D93" t="inlineStr">
         <is>
           <t>GET /api/tags</t>
         </is>
       </c>
-      <c r="E91" t="inlineStr">
+      <c r="E93" t="inlineStr">
         <is>
           <t>Route is registered</t>
         </is>
       </c>
-      <c r="F91" t="inlineStr">
+      <c r="F93" t="inlineStr">
         <is>
           <t>cmd/server/main.go</t>
         </is>
       </c>
-      <c r="G91" t="inlineStr">
+      <c r="G93" t="inlineStr">
         <is>
           <t>Implemented</t>
         </is>

</xml_diff>